<commit_message>
Add marketing-backed operating case
</commit_message>
<xml_diff>
--- a/assets/MIMAR_Investor_Revenue_Model_2026-08-28.xlsx
+++ b/assets/MIMAR_Investor_Revenue_Model_2026-08-28.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rab2c2e59d8604407"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beta Plan" sheetId="2" r:id="Rb6e7650fea884b25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Rd41fa9ec09984b81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Bridge" sheetId="4" r:id="R14eedadd23364e8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Monthly" sheetId="5" r:id="R96dff2f2be114b36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engage Monthly" sheetId="6" r:id="Rf7a3a0c8b5174004"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="7" r:id="Raf81367c393f4ef0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R53f2336b505b4cd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R8745177812e245ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R9ea471d298f14e5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beta Plan" sheetId="2" r:id="Rc4c7509d92e84482"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R13f17d7acc5144b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Bridge" sheetId="4" r:id="R12aeec3605984f07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Monthly" sheetId="5" r:id="R20da8b315e56467e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engage Monthly" sheetId="6" r:id="R8e127d1bf9544444"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="7" r:id="R66de412e2ae94a99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="Rddc47d5a6d944ee7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R327c7abce2c54d99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GTM Plan" sheetId="10" r:id="Rf58b19ae75234487"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -96,7 +97,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="7">
+  <x:numFmts count="9">
     <x:numFmt numFmtId="200" formatCode="mmm yyyy"/>
     <x:numFmt numFmtId="201" formatCode="0.0%;[Red](0.0%);-"/>
     <x:numFmt numFmtId="202" formatCode="$#,##0;[Red]($#,##0);-"/>
@@ -104,8 +105,10 @@
     <x:numFmt numFmtId="204" formatCode="#,##0.0;[Red](#,##0.0);-"/>
     <x:numFmt numFmtId="205" formatCode="$#,##0.0;[Red]($#,##0.0);-"/>
     <x:numFmt numFmtId="206" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="207" formatCode="0"/>
+    <x:numFmt numFmtId="208" formatCode="#,##0;[Red](#,##0);-"/>
   </x:numFmts>
-  <x:fonts count="18">
+  <x:fonts count="23">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -206,8 +209,35 @@
       <x:color rgb="FFC2410C"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF166534"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF166534"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF166534"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -239,8 +269,33 @@
         <x:fgColor rgb="FFDFF7FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F2FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCFCE7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B1016"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF10232D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B1016"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="4">
     <x:border/>
     <x:border>
       <x:bottom style="medium">
@@ -252,11 +307,16 @@
         <x:color rgb="FF4CD6E5"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FF4CD6E5"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="82">
+  <x:cellXfs count="133">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -407,6 +467,91 @@
     <x:xf numFmtId="206" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="19" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="19" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="19" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="208" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="208" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -417,7 +562,7 @@
         <x:color rgb="FF067647"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF5E8"/>
         </x:patternFill>
       </x:fill>
@@ -427,7 +572,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE7E3"/>
         </x:patternFill>
       </x:fill>
@@ -574,6 +719,144 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/drawings/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:t>Acquisition plan lifts revenue without changing retention ($)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Underwritten Base</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'GTM Plan'!$I$5:$I$7</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'GTM Plan'!$J$5:$J$7</c:f>
+              <c:numCache>
+                <c:formatCode>$#,##0;[Red]($#,##0);-</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Marketing-backed</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'GTM Plan'!$I$5:$I$7</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'GTM Plan'!$K$5:$K$7</c:f>
+              <c:numCache>
+                <c:formatCode>$#,##0;[Red]($#,##0);-</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="$0.0,,&quot;M&quot;"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
@@ -600,7 +883,42 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb8a77a71d3954ec4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8f497707cb384624"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra793544cd1e24fbf"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1508,15 +1826,15 @@
         <x:v>Model status</x:v>
       </x:c>
       <x:c r="B29" s="29" t="str">
-        <x:f>"PASS"</x:f>
+        <x:f>IF(COUNTIF('Checks'!$E$5:$E$19,"FAIL")=0,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C29" s="29" t="str">
-        <x:f>"PASS"</x:f>
+        <x:f>IF(COUNTIF('Checks'!$E$5:$E$19,"FAIL")=0,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="D29" s="29" t="str">
-        <x:f>"PASS"</x:f>
+        <x:f>IF(COUNTIF('Checks'!$E$5:$E$19,"FAIL")=0,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="E29" s="29"/>
@@ -1591,27 +1909,45 @@
       <x:c r="I32" s="29"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="29" t="str">
+      <x:c r="A33" s="86" t="str">
         <x:f>'Scenarios'!A7</x:f>
-        <x:v>Upside</x:v>
-      </x:c>
-      <x:c r="B33" s="62" t="n">
+        <x:v>Marketing-backed</x:v>
+      </x:c>
+      <x:c r="B33" s="97" t="n">
         <x:f>'Scenarios'!B7</x:f>
-        <x:v>158029.61000000002</x:v>
-      </x:c>
-      <x:c r="C33" s="62" t="n">
+        <x:v>145134</x:v>
+      </x:c>
+      <x:c r="C33" s="97" t="n">
         <x:f>'Scenarios'!C7</x:f>
-        <x:v>497099.47079999995</x:v>
-      </x:c>
-      <x:c r="D33" s="62" t="n">
+        <x:v>450255.11666666664</x:v>
+      </x:c>
+      <x:c r="D33" s="97" t="n">
         <x:f>'Scenarios'!D7</x:f>
-        <x:v>1335461.514858</x:v>
+        <x:v>1199682.4014</x:v>
       </x:c>
       <x:c r="E33" s="29"/>
       <x:c r="F33" s="29"/>
       <x:c r="G33" s="29"/>
       <x:c r="H33" s="29"/>
       <x:c r="I33" s="29"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="98" t="str">
+        <x:f>'Scenarios'!A8</x:f>
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="B34" s="99" t="n">
+        <x:f>'Scenarios'!B8</x:f>
+        <x:v>158029.61000000002</x:v>
+      </x:c>
+      <x:c r="C34" s="99" t="n">
+        <x:f>'Scenarios'!C8</x:f>
+        <x:v>497099.47079999995</x:v>
+      </x:c>
+      <x:c r="D34" s="99" t="n">
+        <x:f>'Scenarios'!D8</x:f>
+        <x:v>1335461.514858</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1620,7 +1956,665 @@
     <x:mergeCell ref="F26:I28"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03b475a400374666"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd583ce6db775400b"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="21" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="126" t="str">
+        <x:v>Marketing-Backed Operating Plan</x:v>
+      </x:c>
+      <x:c r="B1" s="126"/>
+      <x:c r="C1" s="126"/>
+      <x:c r="D1" s="126"/>
+      <x:c r="E1" s="126"/>
+      <x:c r="F1" s="126"/>
+      <x:c r="G1" s="126"/>
+      <x:c r="H1" s="126"/>
+      <x:c r="I1" s="126"/>
+      <x:c r="J1" s="126"/>
+      <x:c r="K1" s="126"/>
+      <x:c r="L1" s="126"/>
+    </x:row>
+    <x:row r="2" ht="26" customHeight="1">
+      <x:c r="A2" s="127" t="str">
+        <x:v>The Underwritten Base remains the investor commitment. This case keeps price and retention unchanged and increases gross-new acquisition only.</x:v>
+      </x:c>
+      <x:c r="B2" s="127"/>
+      <x:c r="C2" s="127"/>
+      <x:c r="D2" s="127"/>
+      <x:c r="E2" s="127"/>
+      <x:c r="F2" s="127"/>
+      <x:c r="G2" s="127"/>
+      <x:c r="H2" s="127"/>
+      <x:c r="I2" s="127"/>
+      <x:c r="J2" s="127"/>
+      <x:c r="K2" s="127"/>
+      <x:c r="L2" s="127"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="107" t="str">
+        <x:v>Revenue case</x:v>
+      </x:c>
+      <x:c r="B4" s="107" t="str">
+        <x:v>Y1</x:v>
+      </x:c>
+      <x:c r="C4" s="107" t="str">
+        <x:v>Y2</x:v>
+      </x:c>
+      <x:c r="D4" s="107" t="str">
+        <x:v>Y3</x:v>
+      </x:c>
+      <x:c r="I4" s="107" t="str">
+        <x:v>Year</x:v>
+      </x:c>
+      <x:c r="J4" s="107" t="str">
+        <x:v>Underwritten Base</x:v>
+      </x:c>
+      <x:c r="K4" s="107" t="str">
+        <x:v>Marketing-backed</x:v>
+      </x:c>
+      <x:c r="L4" s="107" t="str">
+        <x:v>Increment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Underwritten Base</x:v>
+      </x:c>
+      <x:c r="B5" s="49" t="n">
+        <x:f>'Scenarios'!B6</x:f>
+        <x:v>122363</x:v>
+      </x:c>
+      <x:c r="C5" s="49" t="n">
+        <x:f>'Scenarios'!C6</x:f>
+        <x:v>366674.73333333334</x:v>
+      </x:c>
+      <x:c r="D5" s="49" t="n">
+        <x:f>'Scenarios'!D6</x:f>
+        <x:v>944852.922</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>Y1</x:v>
+      </x:c>
+      <x:c r="J5" s="49" t="n">
+        <x:f>B5</x:f>
+        <x:v>122363</x:v>
+      </x:c>
+      <x:c r="K5" s="49" t="n">
+        <x:f>B6</x:f>
+        <x:v>145134</x:v>
+      </x:c>
+      <x:c r="L5" s="49" t="n">
+        <x:f>B7</x:f>
+        <x:v>22771</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="110" t="str">
+        <x:v>Marketing-backed</x:v>
+      </x:c>
+      <x:c r="B6" s="111" t="n">
+        <x:f>'Scenarios'!B7</x:f>
+        <x:v>145134</x:v>
+      </x:c>
+      <x:c r="C6" s="111" t="n">
+        <x:f>'Scenarios'!C7</x:f>
+        <x:v>450255.11666666664</x:v>
+      </x:c>
+      <x:c r="D6" s="111" t="n">
+        <x:f>'Scenarios'!D7</x:f>
+        <x:v>1199682.4014</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Y2</x:v>
+      </x:c>
+      <x:c r="J6" s="49" t="n">
+        <x:f>C5</x:f>
+        <x:v>366674.73333333334</x:v>
+      </x:c>
+      <x:c r="K6" s="49" t="n">
+        <x:f>C6</x:f>
+        <x:v>450255.11666666664</x:v>
+      </x:c>
+      <x:c r="L6" s="49" t="n">
+        <x:f>C7</x:f>
+        <x:v>83580.3833333333</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Increment vs Base</x:v>
+      </x:c>
+      <x:c r="B7" s="49" t="n">
+        <x:f>B6-B5</x:f>
+        <x:v>22771</x:v>
+      </x:c>
+      <x:c r="C7" s="49" t="n">
+        <x:f>C6-C5</x:f>
+        <x:v>83580.3833333333</x:v>
+      </x:c>
+      <x:c r="D7" s="49" t="n">
+        <x:f>D6-D5</x:f>
+        <x:v>254829.47940000007</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>Y3</x:v>
+      </x:c>
+      <x:c r="J7" s="49" t="n">
+        <x:f>D5</x:f>
+        <x:v>944852.922</x:v>
+      </x:c>
+      <x:c r="K7" s="49" t="n">
+        <x:f>D6</x:f>
+        <x:v>1199682.4014</x:v>
+      </x:c>
+      <x:c r="L7" s="49" t="n">
+        <x:f>D7</x:f>
+        <x:v>254829.47940000007</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="A10" s="107" t="str">
+        <x:v>Gross-new acquisition</x:v>
+      </x:c>
+      <x:c r="B10" s="107" t="str">
+        <x:v>Base Y1</x:v>
+      </x:c>
+      <x:c r="C10" s="107" t="str">
+        <x:v>Plan Y1</x:v>
+      </x:c>
+      <x:c r="D10" s="107" t="str">
+        <x:v>Base Y2</x:v>
+      </x:c>
+      <x:c r="E10" s="107" t="str">
+        <x:v>Plan Y2</x:v>
+      </x:c>
+      <x:c r="F10" s="107" t="str">
+        <x:v>Base Y3</x:v>
+      </x:c>
+      <x:c r="G10" s="107" t="str">
+        <x:v>Plan Y3</x:v>
+      </x:c>
+      <x:c r="H10" s="107" t="str">
+        <x:v>Primary route</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>Individuals</x:v>
+      </x:c>
+      <x:c r="B11" s="112" t="n">
+        <x:f>'Assumptions'!B20</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C11" s="113" t="n">
+        <x:f>B11*'Scenarios'!C14</x:f>
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="D11" s="112" t="n">
+        <x:f>'Assumptions'!C20</x:f>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E11" s="113" t="n">
+        <x:f>D11*'Scenarios'!D14</x:f>
+        <x:v>312.5</x:v>
+      </x:c>
+      <x:c r="F11" s="112" t="n">
+        <x:f>'Assumptions'!D20</x:f>
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G11" s="113" t="n">
+        <x:f>F11*'Scenarios'!E14</x:f>
+        <x:v>650</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>PLG + proof content</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>Core team workspaces</x:v>
+      </x:c>
+      <x:c r="B12" s="112" t="n">
+        <x:f>'Assumptions'!B23</x:f>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C12" s="113" t="n">
+        <x:f>B12*'Scenarios'!C14</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="D12" s="112" t="n">
+        <x:f>'Assumptions'!C23</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E12" s="113" t="n">
+        <x:f>D12*'Scenarios'!D14</x:f>
+        <x:v>37.5</x:v>
+      </x:c>
+      <x:c r="F12" s="112" t="n">
+        <x:f>'Assumptions'!D23</x:f>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G12" s="113" t="n">
+        <x:f>F12*'Scenarios'!E14</x:f>
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Founder-led pilots + referrals</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>API active wallets</x:v>
+      </x:c>
+      <x:c r="B13" s="112" t="n">
+        <x:f>'Assumptions'!B29</x:f>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C13" s="113" t="n">
+        <x:f>B13*'Scenarios'!C14</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="D13" s="112" t="n">
+        <x:f>'Assumptions'!C29</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E13" s="113" t="n">
+        <x:f>D13*'Scenarios'!D14</x:f>
+        <x:v>62.5</x:v>
+      </x:c>
+      <x:c r="F13" s="112" t="n">
+        <x:f>'Assumptions'!D29</x:f>
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="G13" s="113" t="n">
+        <x:f>F13*'Scenarios'!E14</x:f>
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Developer docs + templates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>Engage workspaces</x:v>
+      </x:c>
+      <x:c r="B14" s="112" t="n">
+        <x:f>SUM('Assumptions'!B37,'Assumptions'!B39,'Assumptions'!B41,'Assumptions'!B43)</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C14" s="113" t="n">
+        <x:f>B14*'Scenarios'!C14</x:f>
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D14" s="112" t="n">
+        <x:f>SUM('Assumptions'!C37,'Assumptions'!C39,'Assumptions'!C41,'Assumptions'!C43)</x:f>
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E14" s="113" t="n">
+        <x:f>D14*'Scenarios'!D14</x:f>
+        <x:v>63.75</x:v>
+      </x:c>
+      <x:c r="F14" s="112" t="n">
+        <x:f>SUM('Assumptions'!D37,'Assumptions'!D39,'Assumptions'!D41,'Assumptions'!D43)</x:f>
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="G14" s="113" t="n">
+        <x:f>F14*'Scenarios'!E14</x:f>
+        <x:v>135.20000000000002</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>Vertical workflow campaigns</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="A17" s="107" t="str">
+        <x:v>Scale gate</x:v>
+      </x:c>
+      <x:c r="B17" s="107" t="str">
+        <x:v>Threshold</x:v>
+      </x:c>
+      <x:c r="C17" s="107" t="str">
+        <x:v>Why it matters</x:v>
+      </x:c>
+      <x:c r="D17" s="107" t="str">
+        <x:v>If it passes</x:v>
+      </x:c>
+      <x:c r="E17" s="107" t="str">
+        <x:v>If it misses</x:v>
+      </x:c>
+      <x:c r="F17" s="107" t="str">
+        <x:v>Evidence window</x:v>
+      </x:c>
+      <x:c r="G17" s="107" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="44" customHeight="1">
+      <x:c r="A18" s="130" t="str">
+        <x:v>Activated trial → paid</x:v>
+      </x:c>
+      <x:c r="B18" s="131" t="str">
+        <x:v>&gt;= 5%</x:v>
+      </x:c>
+      <x:c r="C18" s="130" t="str">
+        <x:v>Proves self-serve demand</x:v>
+      </x:c>
+      <x:c r="D18" s="130" t="str">
+        <x:v>Increase qualified traffic</x:v>
+      </x:c>
+      <x:c r="E18" s="130" t="str">
+        <x:v>Fix activation/onboarding</x:v>
+      </x:c>
+      <x:c r="F18" s="130" t="str">
+        <x:v>3 monthly cohorts</x:v>
+      </x:c>
+      <x:c r="G18" s="130" t="str">
+        <x:v>Growth + Product</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="44" customHeight="1">
+      <x:c r="A19" s="130" t="str">
+        <x:v>Team pilot → paid</x:v>
+      </x:c>
+      <x:c r="B19" s="131" t="str">
+        <x:v>&gt;= 20%</x:v>
+      </x:c>
+      <x:c r="C19" s="130" t="str">
+        <x:v>Validates founder-led sales</x:v>
+      </x:c>
+      <x:c r="D19" s="130" t="str">
+        <x:v>Expand target-account list</x:v>
+      </x:c>
+      <x:c r="E19" s="130" t="str">
+        <x:v>Narrow ICP and workflow</x:v>
+      </x:c>
+      <x:c r="F19" s="130" t="str">
+        <x:v>10+ completed pilots</x:v>
+      </x:c>
+      <x:c r="G19" s="130" t="str">
+        <x:v>Founder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="44" customHeight="1">
+      <x:c r="A20" s="130" t="str">
+        <x:v>90-day team retention</x:v>
+      </x:c>
+      <x:c r="B20" s="131" t="str">
+        <x:v>&gt;= 85%</x:v>
+      </x:c>
+      <x:c r="C20" s="130" t="str">
+        <x:v>Protects the 90% annual target</x:v>
+      </x:c>
+      <x:c r="D20" s="130" t="str">
+        <x:v>Add referral motion</x:v>
+      </x:c>
+      <x:c r="E20" s="130" t="str">
+        <x:v>Pause acquisition scaling</x:v>
+      </x:c>
+      <x:c r="F20" s="130" t="str">
+        <x:v>10+ paid teams</x:v>
+      </x:c>
+      <x:c r="G20" s="130" t="str">
+        <x:v>Product + CS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="44" customHeight="1">
+      <x:c r="A21" s="130" t="str">
+        <x:v>CAC payback</x:v>
+      </x:c>
+      <x:c r="B21" s="131" t="str">
+        <x:v>&lt;= 9 months</x:v>
+      </x:c>
+      <x:c r="C21" s="130" t="str">
+        <x:v>Protects cash efficiency</x:v>
+      </x:c>
+      <x:c r="D21" s="130" t="str">
+        <x:v>Scale winning channels</x:v>
+      </x:c>
+      <x:c r="E21" s="130" t="str">
+        <x:v>Cut channel or raise conversion</x:v>
+      </x:c>
+      <x:c r="F21" s="130" t="str">
+        <x:v>Two paid quarters</x:v>
+      </x:c>
+      <x:c r="G21" s="130" t="str">
+        <x:v>Finance + Growth</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="28" customHeight="1">
+      <x:c r="A24" s="107" t="str">
+        <x:v>Commercial year</x:v>
+      </x:c>
+      <x:c r="B24" s="107" t="str">
+        <x:v>Budget low</x:v>
+      </x:c>
+      <x:c r="C24" s="107" t="str">
+        <x:v>Budget high</x:v>
+      </x:c>
+      <x:c r="D24" s="107" t="str">
+        <x:v>Primary objective</x:v>
+      </x:c>
+      <x:c r="E24" s="107" t="str">
+        <x:v>Content / proof</x:v>
+      </x:c>
+      <x:c r="F24" s="107" t="str">
+        <x:v>Founder-led sales</x:v>
+      </x:c>
+      <x:c r="G24" s="107" t="str">
+        <x:v>Paid channel posture</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="46" customHeight="1">
+      <x:c r="A25" s="130" t="str">
+        <x:v>Y1</x:v>
+      </x:c>
+      <x:c r="B25" s="132" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="C25" s="132" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="D25" s="130" t="str">
+        <x:v>Validate repeatable acquisition</x:v>
+      </x:c>
+      <x:c r="E25" s="130" t="str">
+        <x:v>2 case studies + weekly proof</x:v>
+      </x:c>
+      <x:c r="F25" s="130" t="str">
+        <x:v>Core teams + design partners</x:v>
+      </x:c>
+      <x:c r="G25" s="130" t="str">
+        <x:v>Small tests only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="46" customHeight="1">
+      <x:c r="A26" s="130" t="str">
+        <x:v>Y2</x:v>
+      </x:c>
+      <x:c r="B26" s="132" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="C26" s="132" t="n">
+        <x:v>40000</x:v>
+      </x:c>
+      <x:c r="D26" s="130" t="str">
+        <x:v>Scale channels that pass gates</x:v>
+      </x:c>
+      <x:c r="E26" s="130" t="str">
+        <x:v>Vertical playbooks</x:v>
+      </x:c>
+      <x:c r="F26" s="130" t="str">
+        <x:v>Teams + early enterprise</x:v>
+      </x:c>
+      <x:c r="G26" s="130" t="str">
+        <x:v>Scale proven campaigns</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="46" customHeight="1">
+      <x:c r="A27" s="130" t="str">
+        <x:v>Y3</x:v>
+      </x:c>
+      <x:c r="B27" s="132" t="n">
+        <x:v>70000</x:v>
+      </x:c>
+      <x:c r="C27" s="132" t="n">
+        <x:v>90000</x:v>
+      </x:c>
+      <x:c r="D27" s="130" t="str">
+        <x:v>Compound portfolio distribution</x:v>
+      </x:c>
+      <x:c r="E27" s="130" t="str">
+        <x:v>Category + partner proof</x:v>
+      </x:c>
+      <x:c r="F27" s="130" t="str">
+        <x:v>Enterprise and expansion</x:v>
+      </x:c>
+      <x:c r="G27" s="130" t="str">
+        <x:v>Portfolio-level efficiency</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="28" customHeight="1">
+      <x:c r="A30" s="107" t="str">
+        <x:v>Phase</x:v>
+      </x:c>
+      <x:c r="B30" s="107" t="str">
+        <x:v>Timing</x:v>
+      </x:c>
+      <x:c r="C30" s="107" t="str">
+        <x:v>Goal</x:v>
+      </x:c>
+      <x:c r="D30" s="107" t="str">
+        <x:v>Individuals</x:v>
+      </x:c>
+      <x:c r="E30" s="107" t="str">
+        <x:v>Teams</x:v>
+      </x:c>
+      <x:c r="F30" s="107" t="str">
+        <x:v>Engage</x:v>
+      </x:c>
+      <x:c r="G30" s="107" t="str">
+        <x:v>Evidence produced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="48" customHeight="1">
+      <x:c r="A31" s="130" t="str">
+        <x:v>Close Beta</x:v>
+      </x:c>
+      <x:c r="B31" s="130" t="str">
+        <x:v>Now → access release</x:v>
+      </x:c>
+      <x:c r="C31" s="130" t="str">
+        <x:v>Sign the starting cohort</x:v>
+      </x:c>
+      <x:c r="D31" s="130" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E31" s="130" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F31" s="130" t="str">
+        <x:v>Design partners</x:v>
+      </x:c>
+      <x:c r="G31" s="130" t="str">
+        <x:v>Signed commitments + ICP notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="48" customHeight="1">
+      <x:c r="A32" s="130" t="str">
+        <x:v>Build + validate</x:v>
+      </x:c>
+      <x:c r="B32" s="130" t="str">
+        <x:v>Beta months 1–4</x:v>
+      </x:c>
+      <x:c r="C32" s="130" t="str">
+        <x:v>Prove recurring workflow value</x:v>
+      </x:c>
+      <x:c r="D32" s="130" t="str">
+        <x:v>12 active</x:v>
+      </x:c>
+      <x:c r="E32" s="130" t="str">
+        <x:v>2 active</x:v>
+      </x:c>
+      <x:c r="F32" s="130" t="str">
+        <x:v>Workflow interviews</x:v>
+      </x:c>
+      <x:c r="G32" s="130" t="str">
+        <x:v>Activation, usage, pilot feedback</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="48" customHeight="1">
+      <x:c r="A33" s="130" t="str">
+        <x:v>Expand Beta</x:v>
+      </x:c>
+      <x:c r="B33" s="130" t="str">
+        <x:v>Beta months 5–6</x:v>
+      </x:c>
+      <x:c r="C33" s="130" t="str">
+        <x:v>Test referrals and repeatability</x:v>
+      </x:c>
+      <x:c r="D33" s="130" t="str">
+        <x:v>30 active</x:v>
+      </x:c>
+      <x:c r="E33" s="130" t="str">
+        <x:v>5 active</x:v>
+      </x:c>
+      <x:c r="F33" s="130" t="str">
+        <x:v>First vertical shortlist</x:v>
+      </x:c>
+      <x:c r="G33" s="130" t="str">
+        <x:v>Case studies + retention leading indicators</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="48" customHeight="1">
+      <x:c r="A34" s="130" t="str">
+        <x:v>Commercial scale</x:v>
+      </x:c>
+      <x:c r="B34" s="130" t="str">
+        <x:v>From May 2027</x:v>
+      </x:c>
+      <x:c r="C34" s="130" t="str">
+        <x:v>Acquire only behind gates</x:v>
+      </x:c>
+      <x:c r="D34" s="130" t="str">
+        <x:v>120 Y1 new</x:v>
+      </x:c>
+      <x:c r="E34" s="130" t="str">
+        <x:v>24 Y1 new</x:v>
+      </x:c>
+      <x:c r="F34" s="130" t="str">
+        <x:v>36 Y1 new</x:v>
+      </x:c>
+      <x:c r="G34" s="130" t="str">
+        <x:v>Conversion, retention, CAC payback</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raad399a71d6b4c53"/>
 </x:worksheet>
 </file>
 
@@ -3505,7 +4499,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fdb9263f6374181"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde3b36c051cc46e6"/>
 </x:worksheet>
 </file>
 
@@ -10663,20 +11657,21 @@
       <x:c r="R6" s="29"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="29" t="str">
-        <x:v>Upside</x:v>
-      </x:c>
-      <x:c r="B7" s="62" t="n">
-        <x:f>R22</x:f>
-        <x:v>158029.61000000002</x:v>
-      </x:c>
-      <x:c r="C7" s="62" t="n">
-        <x:f>R23</x:f>
-        <x:v>497099.47079999995</x:v>
-      </x:c>
-      <x:c r="D7" s="62" t="n">
-        <x:f>R24</x:f>
-        <x:v>1335461.514858</x:v>
+      <x:c r="A7" s="86" t="str">
+        <x:f>$A$14</x:f>
+        <x:v>Marketing-backed</x:v>
+      </x:c>
+      <x:c r="B7" s="97" t="n">
+        <x:f>$R$25</x:f>
+        <x:v>145134</x:v>
+      </x:c>
+      <x:c r="C7" s="97" t="n">
+        <x:f>$R$26</x:f>
+        <x:v>450255.11666666664</x:v>
+      </x:c>
+      <x:c r="D7" s="97" t="n">
+        <x:f>$R$27</x:f>
+        <x:v>1199682.4014</x:v>
       </x:c>
       <x:c r="E7" s="29"/>
       <x:c r="F7" s="29"/>
@@ -10694,10 +11689,22 @@
       <x:c r="R7" s="29"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="29"/>
-      <x:c r="B8" s="29"/>
-      <x:c r="C8" s="29"/>
-      <x:c r="D8" s="29"/>
+      <x:c r="A8" s="29" t="str">
+        <x:f>$A$13</x:f>
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="B8" s="62" t="n">
+        <x:f>$R$22</x:f>
+        <x:v>158029.61000000002</x:v>
+      </x:c>
+      <x:c r="C8" s="62" t="n">
+        <x:f>$R$23</x:f>
+        <x:v>497099.47079999995</x:v>
+      </x:c>
+      <x:c r="D8" s="62" t="n">
+        <x:f>$R$24</x:f>
+        <x:v>1335461.514858</x:v>
+      </x:c>
       <x:c r="E8" s="29"/>
       <x:c r="F8" s="29"/>
       <x:c r="G8" s="29"/>
@@ -10878,14 +11885,30 @@
       <x:c r="R13" s="29"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="29"/>
-      <x:c r="B14" s="29"/>
-      <x:c r="C14" s="29"/>
-      <x:c r="D14" s="29"/>
-      <x:c r="E14" s="29"/>
-      <x:c r="F14" s="29"/>
-      <x:c r="G14" s="29"/>
-      <x:c r="H14" s="29"/>
+      <x:c r="A14" s="86" t="str">
+        <x:v>Marketing-backed</x:v>
+      </x:c>
+      <x:c r="B14" s="84" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C14" s="84" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="D14" s="84" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="E14" s="84" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="F14" s="84" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="G14" s="84" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="H14" s="84" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
       <x:c r="I14" s="29"/>
       <x:c r="J14" s="29"/>
       <x:c r="K14" s="29"/>
@@ -11617,6 +12640,228 @@
       <x:c r="R24" s="62" t="n">
         <x:f>N24+O24+P24+Q24</x:f>
         <x:v>1335461.514858</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="23" customHeight="1">
+      <x:c r="A25" s="88" t="str">
+        <x:f>$A$14</x:f>
+        <x:v>Marketing-backed</x:v>
+      </x:c>
+      <x:c r="B25" s="89" t="n">
+        <x:f>1</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C25" s="90" t="n">
+        <x:f>$B$14</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D25" s="90" t="n">
+        <x:f>$C$14</x:f>
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="E25" s="90" t="n">
+        <x:f>$F$14</x:f>
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="F25" s="90" t="n">
+        <x:f>$G$14</x:f>
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="G25" s="90" t="n">
+        <x:f>$H$14</x:f>
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="H25" s="91" t="n">
+        <x:f>$C25*(('Assumptions'!$B$8*(6*$E25^0+6*$E25^1)+'Assumptions'!$B$9*(10*$E25^0+2*$E25^1))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F25^0+6*$F25^1)+'Assumptions'!$B$12*(10*$F25^0+2*$F25^1))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
+        <x:v>8508</x:v>
+      </x:c>
+      <x:c r="I25" s="91" t="n">
+        <x:f>('Assumptions'!$B$20*$D25*6.5)*'Assumptions'!$B$22</x:f>
+        <x:v>12480</x:v>
+      </x:c>
+      <x:c r="J25" s="91" t="n">
+        <x:f>'Assumptions'!$B$23*$D25*6.5*'Assumptions'!$B$25*'Assumptions'!$B$26</x:f>
+        <x:v>24960</x:v>
+      </x:c>
+      <x:c r="K25" s="91" t="n">
+        <x:f>'Assumptions'!$B$27*$D25*6.5/12*'Assumptions'!$B$28</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L25" s="91" t="n">
+        <x:f>'Assumptions'!$B$29*$D25*6.5*'Assumptions'!$B$31</x:f>
+        <x:v>4680</x:v>
+      </x:c>
+      <x:c r="M25" s="91" t="n">
+        <x:f>('Assumptions'!$B$23+'Assumptions'!$B$27)*$D25*'Assumptions'!$B$32</x:f>
+        <x:v>24000</x:v>
+      </x:c>
+      <x:c r="N25" s="91" t="n">
+        <x:f>SUM(H25:M25)</x:f>
+        <x:v>74628</x:v>
+      </x:c>
+      <x:c r="O25" s="91" t="n">
+        <x:f>'Assumptions'!$B$37*$D25*6.5*'Assumptions'!$B$38+'Assumptions'!$B$39*$D25*6.5*'Assumptions'!$B$40+'Assumptions'!$B$41*$D25*6.5*'Assumptions'!$B$42+'Assumptions'!$B$43*$D25*6.5*'Assumptions'!$B$44</x:f>
+        <x:v>48905.99999999999</x:v>
+      </x:c>
+      <x:c r="P25" s="91" t="n">
+        <x:f>O25*'Assumptions'!$B$46</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q25" s="91" t="n">
+        <x:f>(('Assumptions'!$B$37+'Assumptions'!$B$39+'Assumptions'!$B$41)*'Assumptions'!$B$47+'Assumptions'!$B$43*'Assumptions'!$B$48)*$D25</x:f>
+        <x:v>21600</x:v>
+      </x:c>
+      <x:c r="R25" s="91" t="n">
+        <x:f>N25+O25+P25+Q25</x:f>
+        <x:v>145134</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="23" customHeight="1">
+      <x:c r="A26" s="88" t="str">
+        <x:f>$A$14</x:f>
+        <x:v>Marketing-backed</x:v>
+      </x:c>
+      <x:c r="B26" s="89" t="n">
+        <x:f>2</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C26" s="90" t="n">
+        <x:f>$B$14</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D26" s="90" t="n">
+        <x:f>$D$14</x:f>
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="E26" s="90" t="n">
+        <x:f>$F$14</x:f>
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="F26" s="90" t="n">
+        <x:f>$G$14</x:f>
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="G26" s="90" t="n">
+        <x:f>$H$14</x:f>
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="H26" s="91" t="n">
+        <x:f>$C26*(('Assumptions'!$B$8*(6*$E26^1+6*$E26^2)+'Assumptions'!$B$9*(10*$E26^1+2*$E26^2))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F26^1+6*$F26^2)+'Assumptions'!$B$12*(10*$F26^1+2*$F26^2))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
+        <x:v>6152.4000000000015</x:v>
+      </x:c>
+      <x:c r="I26" s="91" t="n">
+        <x:f>('Assumptions'!$B$20*$D25*$E26*12+'Assumptions'!$C$20*$D26*6.5)*'Assumptions'!$C$22</x:f>
+        <x:v>52114.5</x:v>
+      </x:c>
+      <x:c r="J26" s="91" t="n">
+        <x:f>('Assumptions'!$B$23*$D25*$F26*12+'Assumptions'!$C$23*$D26*6.5)*'Assumptions'!$C$25*'Assumptions'!$C$26</x:f>
+        <x:v>99584.1</x:v>
+      </x:c>
+      <x:c r="K26" s="91" t="n">
+        <x:f>('Assumptions'!$B$27*$D25*$F26*12+'Assumptions'!$C$27*$D26*6.5)/12*'Assumptions'!$C$28</x:f>
+        <x:v>13541.666666666668</x:v>
+      </x:c>
+      <x:c r="L26" s="91" t="n">
+        <x:f>('Assumptions'!$B$29*$D25*$G26*12+'Assumptions'!$C$29*$D26*6.5)*'Assumptions'!$C$31</x:f>
+        <x:v>27353.249999999996</x:v>
+      </x:c>
+      <x:c r="M26" s="91" t="n">
+        <x:f>('Assumptions'!$C$23+'Assumptions'!$C$27)*$D26*'Assumptions'!$C$32</x:f>
+        <x:v>34875</x:v>
+      </x:c>
+      <x:c r="N26" s="91" t="n">
+        <x:f>SUM(H26:M26)</x:f>
+        <x:v>233620.91666666666</x:v>
+      </x:c>
+      <x:c r="O26" s="91" t="n">
+        <x:f>('Assumptions'!$B$37*$D25*$F26*12+'Assumptions'!$C$37*$D26*6.5)*'Assumptions'!$C$38+('Assumptions'!$B$39*$D25*$F26*12+'Assumptions'!$C$39*$D26*6.5)*'Assumptions'!$C$40+('Assumptions'!$B$41*$D25*$F26*12+'Assumptions'!$C$41*$D26*6.5)*'Assumptions'!$C$42+('Assumptions'!$B$43*$D25*$F26*12+'Assumptions'!$C$43*$D26*6.5)*'Assumptions'!$C$44</x:f>
+        <x:v>180384.19999999998</x:v>
+      </x:c>
+      <x:c r="P26" s="91" t="n">
+        <x:f>O26*'Assumptions'!$C$46</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q26" s="91" t="n">
+        <x:f>(('Assumptions'!$C$37+'Assumptions'!$C$39+'Assumptions'!$C$41)*'Assumptions'!$C$47+'Assumptions'!$C$43*'Assumptions'!$C$48)*$D26</x:f>
+        <x:v>36250</x:v>
+      </x:c>
+      <x:c r="R26" s="91" t="n">
+        <x:f>N26+O26+P26+Q26</x:f>
+        <x:v>450255.11666666664</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="23" customHeight="1">
+      <x:c r="A27" s="92" t="str">
+        <x:f>$A$14</x:f>
+        <x:v>Marketing-backed</x:v>
+      </x:c>
+      <x:c r="B27" s="93" t="n">
+        <x:f>3</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C27" s="94" t="n">
+        <x:f>$B$14</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D27" s="94" t="n">
+        <x:f>$E$14</x:f>
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="E27" s="94" t="n">
+        <x:f>$F$14</x:f>
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="F27" s="94" t="n">
+        <x:f>$G$14</x:f>
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="G27" s="94" t="n">
+        <x:f>$H$14</x:f>
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="H27" s="95" t="n">
+        <x:f>$C27*(('Assumptions'!$B$8*(6*$E27^2+6*$E27^3)+'Assumptions'!$B$9*(10*$E27^2+2*$E27^3))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F27^2+6*$F27^3)+'Assumptions'!$B$12*(10*$F27^2+2*$F27^3))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
+        <x:v>4634.280000000001</x:v>
+      </x:c>
+      <x:c r="I27" s="95" t="n">
+        <x:f>('Assumptions'!$B$20*$D25*$E27^2*12+'Assumptions'!$C$20*$D26*$E27*12+'Assumptions'!$D$20*$D27*6.5)*'Assumptions'!$D$22</x:f>
+        <x:v>139868</x:v>
+      </x:c>
+      <x:c r="J27" s="95" t="n">
+        <x:f>('Assumptions'!$B$23*$D25*$F27^2*12+'Assumptions'!$C$23*$D26*$F27*12+'Assumptions'!$D$23*$D27*6.5)*'Assumptions'!$D$25*'Assumptions'!$D$26</x:f>
+        <x:v>274867.19999999995</x:v>
+      </x:c>
+      <x:c r="K27" s="95" t="n">
+        <x:f>('Assumptions'!$B$27*$D25*$F27^2*12+'Assumptions'!$C$27*$D26*$F27*12+'Assumptions'!$D$27*$D27*6.5)/12*'Assumptions'!$D$28</x:f>
+        <x:v>71225</x:v>
+      </x:c>
+      <x:c r="L27" s="95" t="n">
+        <x:f>('Assumptions'!$B$29*$D25*$G27^2*12+'Assumptions'!$C$29*$D26*$G27*12+'Assumptions'!$D$29*$D27*6.5)*'Assumptions'!$D$31</x:f>
+        <x:v>100807.2</x:v>
+      </x:c>
+      <x:c r="M27" s="95" t="n">
+        <x:f>('Assumptions'!$D$23+'Assumptions'!$D$27)*$D27*'Assumptions'!$D$32</x:f>
+        <x:v>61425.00000000001</x:v>
+      </x:c>
+      <x:c r="N27" s="95" t="n">
+        <x:f>SUM(H27:M27)</x:f>
+        <x:v>652826.6799999999</x:v>
+      </x:c>
+      <x:c r="O27" s="95" t="n">
+        <x:f>('Assumptions'!$B$37*$D25*$F27^2*12+'Assumptions'!$C$37*$D26*$F27*12+'Assumptions'!$D$37*$D27*6.5)*'Assumptions'!$D$38+('Assumptions'!$B$39*$D25*$F27^2*12+'Assumptions'!$C$39*$D26*$F27*12+'Assumptions'!$D$39*$D27*6.5)*'Assumptions'!$D$40+('Assumptions'!$B$41*$D25*$F27^2*12+'Assumptions'!$C$41*$D26*$F27*12+'Assumptions'!$D$41*$D27*6.5)*'Assumptions'!$D$42+('Assumptions'!$B$43*$D25*$F27^2*12+'Assumptions'!$C$43*$D26*$F27*12+'Assumptions'!$D$43*$D27*6.5)*'Assumptions'!$D$44</x:f>
+        <x:v>466811.38</x:v>
+      </x:c>
+      <x:c r="P27" s="95" t="n">
+        <x:f>O27*'Assumptions'!$D$46</x:f>
+        <x:v>14004.3414</x:v>
+      </x:c>
+      <x:c r="Q27" s="95" t="n">
+        <x:f>(('Assumptions'!$D$37+'Assumptions'!$D$39+'Assumptions'!$D$41)*'Assumptions'!$D$47+'Assumptions'!$D$43*'Assumptions'!$D$48)*$D27</x:f>
+        <x:v>66040</x:v>
+      </x:c>
+      <x:c r="R27" s="95" t="n">
+        <x:f>N27+O27+P27+Q27</x:f>
+        <x:v>1199682.4014</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11632,7 +12877,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="48" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="43" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
@@ -11949,16 +13194,15 @@
         <x:v>Scenario ordering — Y3</x:v>
       </x:c>
       <x:c r="B15" s="76" t="n">
-        <x:f>'Scenarios'!D7-'Scenarios'!D6</x:f>
-        <x:v>390608.59285799996</x:v>
+        <x:f>MIN('Scenarios'!D6-'Scenarios'!D5,'Scenarios'!D7-'Scenarios'!D6,'Scenarios'!D8-'Scenarios'!D7)</x:f>
+        <x:v>135779.1134579999</x:v>
       </x:c>
       <x:c r="C15" s="76" t="n">
-        <x:f>'Scenarios'!D6-'Scenarios'!D5</x:f>
-        <x:v>224445.84590000007</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D15" s="76" t="n">
-        <x:f>MIN(B15,C15)</x:f>
-        <x:v>224445.84590000007</x:v>
+        <x:f>B15-C15</x:f>
+        <x:v>135779.1134579999</x:v>
       </x:c>
       <x:c r="E15" s="29" t="str">
         <x:f>IF(D15&gt;0,"PASS","FAIL")</x:f>
@@ -11990,6 +13234,75 @@
       </x:c>
       <x:c r="F16" s="29" t="str">
         <x:v>Assumptions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="21" t="str">
+        <x:v>Marketing case keeps Base retention</x:v>
+      </x:c>
+      <x:c r="B17" s="60" t="n">
+        <x:f>ABS('Scenarios'!F14-'Scenarios'!F12)+ABS('Scenarios'!G14-'Scenarios'!G12)+ABS('Scenarios'!H14-'Scenarios'!H12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C17" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D17" s="60" t="n">
+        <x:f>B17-C17</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="122" t="str">
+        <x:f>IF(ABS(D17)&lt;0.0001,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F17" s="21" t="str">
+        <x:v>Scenarios</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="21" t="str">
+        <x:v>Marketing budget high exceeds low</x:v>
+      </x:c>
+      <x:c r="B18" s="55" t="n">
+        <x:f>MIN('GTM Plan'!C25-'GTM Plan'!B25,'GTM Plan'!C26-'GTM Plan'!B26,'GTM Plan'!C27-'GTM Plan'!B27)</x:f>
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="C18" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D18" s="55" t="n">
+        <x:f>B18-C18</x:f>
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="E18" s="122" t="str">
+        <x:f>IF(D18&gt;0,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F18" s="21" t="str">
+        <x:v>GTM Plan</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="24" customHeight="1">
+      <x:c r="A19" s="21" t="str">
+        <x:v>Marketing case changes acquisition</x:v>
+      </x:c>
+      <x:c r="B19" s="60" t="n">
+        <x:f>MIN('Scenarios'!C14-1,'Scenarios'!D14-1,'Scenarios'!E14-1)</x:f>
+        <x:v>0.19999999999999996</x:v>
+      </x:c>
+      <x:c r="C19" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D19" s="60" t="n">
+        <x:f>B19-C19</x:f>
+        <x:v>0.19999999999999996</x:v>
+      </x:c>
+      <x:c r="E19" s="122" t="str">
+        <x:f>IF(D19&gt;0,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F19" s="21" t="str">
+        <x:v>Scenarios</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12009,15 +13322,15 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="43" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="52" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="58" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="36" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="40" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="40" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -12379,6 +13692,93 @@
         <x:v>Replace with observed renewals</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="123" t="str">
+        <x:v>Trial conversion benchmark</x:v>
+      </x:c>
+      <x:c r="B14" s="123" t="str">
+        <x:v>Median trial-to-paid around 8%; good AI / B2B ranges roughly 6–10%</x:v>
+      </x:c>
+      <x:c r="C14" s="123" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="D14" s="123" t="str">
+        <x:v>Industry benchmark</x:v>
+      </x:c>
+      <x:c r="E14" s="123" t="str">
+        <x:v>ChartMogul</x:v>
+      </x:c>
+      <x:c r="F14" s="123" t="str">
+        <x:v>https://chartmogul.com/reports/saas-conversion-report/</x:v>
+      </x:c>
+      <x:c r="G14" s="123" t="str">
+        <x:v>GTM gates</x:v>
+      </x:c>
+      <x:c r="H14" s="123" t="str">
+        <x:v>Use &gt;=5% activated trial-to-paid as a conservative scale gate</x:v>
+      </x:c>
+      <x:c r="I14" s="123" t="str">
+        <x:v>Benchmark sample is not MIMAR cohort evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="123" t="str">
+        <x:v>GTM sequencing</x:v>
+      </x:c>
+      <x:c r="B15" s="123" t="str">
+        <x:v>Trial conversion concentrates early; PLG works best at low ASP with sales layered for larger contracts</x:v>
+      </x:c>
+      <x:c r="C15" s="123" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="D15" s="123" t="str">
+        <x:v>Industry benchmark</x:v>
+      </x:c>
+      <x:c r="E15" s="123" t="str">
+        <x:v>ChartMogul</x:v>
+      </x:c>
+      <x:c r="F15" s="123" t="str">
+        <x:v>https://chartmogul.com/reports/saas-go-to-market-report/</x:v>
+      </x:c>
+      <x:c r="G15" s="123" t="str">
+        <x:v>Individuals + teams</x:v>
+      </x:c>
+      <x:c r="H15" s="123" t="str">
+        <x:v>Combine PLG with founder-led sales</x:v>
+      </x:c>
+      <x:c r="I15" s="123" t="str">
+        <x:v>Operational guidance, not guaranteed performance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="123" t="str">
+        <x:v>CAC payback</x:v>
+      </x:c>
+      <x:c r="B16" s="123" t="str">
+        <x:v>Common SaaS benchmark is about 12 months; model uses a stricter &lt;=9-month scale gate</x:v>
+      </x:c>
+      <x:c r="C16" s="123" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="D16" s="123" t="str">
+        <x:v>Industry benchmark</x:v>
+      </x:c>
+      <x:c r="E16" s="123" t="str">
+        <x:v>Benchmarkit</x:v>
+      </x:c>
+      <x:c r="F16" s="123" t="str">
+        <x:v>https://www.benchmarkit.ai/2025benchmarks</x:v>
+      </x:c>
+      <x:c r="G16" s="123" t="str">
+        <x:v>Marketing budget</x:v>
+      </x:c>
+      <x:c r="H16" s="123" t="str">
+        <x:v>Scale only channels that protect cash efficiency</x:v>
+      </x:c>
+      <x:c r="I16" s="123" t="str">
+        <x:v>Survey population is more mature than MIMAR</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
Update paid beta to founding Team Pro target
</commit_message>
<xml_diff>
--- a/assets/MIMAR_Investor_Revenue_Model_2026-08-28.xlsx
+++ b/assets/MIMAR_Investor_Revenue_Model_2026-08-28.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R9ea471d298f14e5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beta Plan" sheetId="2" r:id="Rc4c7509d92e84482"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R13f17d7acc5144b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Bridge" sheetId="4" r:id="R12aeec3605984f07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Monthly" sheetId="5" r:id="R20da8b315e56467e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engage Monthly" sheetId="6" r:id="R8e127d1bf9544444"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="7" r:id="R66de412e2ae94a99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="Rddc47d5a6d944ee7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R327c7abce2c54d99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GTM Plan" sheetId="10" r:id="Rf58b19ae75234487"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rb826add9d2fe4f6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beta Plan" sheetId="2" r:id="R680a4d4f87db4a98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Redc221fc56254a71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Bridge" sheetId="4" r:id="R4a641a5adfed4dd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Monthly" sheetId="5" r:id="Re9fe6b8429104394"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engage Monthly" sheetId="6" r:id="Rcc8ae7cbc70a434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="7" r:id="R0defdef88ddb4610"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R6ecd0d23595b4839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Rd041fb77bd7d491e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GTM Plan" sheetId="10" r:id="R44b3c4a3791e4845"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -883,7 +883,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8f497707cb384624"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re373b63192f14e5f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -918,7 +918,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra793544cd1e24fbf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re900035a3ff24cdf"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1193,7 +1193,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>Paid Beta Nov 2026–Apr 2027 | Commercial forecast May 2027–Apr 2030 | Explicit cohorts and segmented retention</x:v>
+        <x:v>Paid Beta Nov 2026–Apr 2027 | 30 Individual Pro passes + 2 founding Team Pro workspaces | Commercial forecast May 2027–Apr 2030 | Explicit cohorts and segmented retention</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>Paid Beta Nov 2026–Apr 2027 | Commercial forecast May 2027–Apr 2030 | Explicit cohorts and segmented retention</x:v>
@@ -1264,15 +1264,15 @@
       </x:c>
       <x:c r="B5" s="62" t="n">
         <x:f>SUM('Core Monthly'!F5:F16)+SUM('Core Monthly'!J5:J16)</x:f>
-        <x:v>8508</x:v>
+        <x:v>6384</x:v>
       </x:c>
       <x:c r="C5" s="62" t="n">
         <x:f>SUM('Core Monthly'!F17:F28)+SUM('Core Monthly'!J17:J28)</x:f>
-        <x:v>6152.4</x:v>
+        <x:v>4240.800000000001</x:v>
       </x:c>
       <x:c r="D5" s="62" t="n">
         <x:f>SUM('Core Monthly'!F29:F40)+SUM('Core Monthly'!J29:J40)</x:f>
-        <x:v>4634.28</x:v>
+        <x:v>2913.8399999999992</x:v>
       </x:c>
       <x:c r="E5" s="29"/>
       <x:c r="F5" s="29" t="str">
@@ -1280,7 +1280,7 @@
       </x:c>
       <x:c r="G5" s="62" t="n">
         <x:f>B11</x:f>
-        <x:v>63608</x:v>
+        <x:v>61484</x:v>
       </x:c>
       <x:c r="H5" s="62" t="n">
         <x:f>B19</x:f>
@@ -1288,7 +1288,7 @@
       </x:c>
       <x:c r="I5" s="62" t="n">
         <x:f>B21</x:f>
-        <x:v>122363</x:v>
+        <x:v>120239</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1313,7 +1313,7 @@
       </x:c>
       <x:c r="G6" s="62" t="n">
         <x:f>C11</x:f>
-        <x:v>190658.73333333334</x:v>
+        <x:v>188747.13333333333</x:v>
       </x:c>
       <x:c r="H6" s="62" t="n">
         <x:f>C19</x:f>
@@ -1321,7 +1321,7 @@
       </x:c>
       <x:c r="I6" s="62" t="n">
         <x:f>C21</x:f>
-        <x:v>366674.73333333334</x:v>
+        <x:v>364763.1333333333</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1346,7 +1346,7 @@
       </x:c>
       <x:c r="G7" s="62" t="n">
         <x:f>D11</x:f>
-        <x:v>514146.28</x:v>
+        <x:v>512425.83999999997</x:v>
       </x:c>
       <x:c r="H7" s="62" t="n">
         <x:f>D19</x:f>
@@ -1354,7 +1354,7 @@
       </x:c>
       <x:c r="I7" s="62" t="n">
         <x:f>D21</x:f>
-        <x:v>944852.922</x:v>
+        <x:v>943132.482</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1429,15 +1429,15 @@
       </x:c>
       <x:c r="B11" s="64" t="n">
         <x:f>SUM(B5:B10)</x:f>
-        <x:v>63608</x:v>
+        <x:v>61484</x:v>
       </x:c>
       <x:c r="C11" s="64" t="n">
         <x:f>SUM(C5:C10)</x:f>
-        <x:v>190658.73333333334</x:v>
+        <x:v>188747.13333333333</x:v>
       </x:c>
       <x:c r="D11" s="64" t="n">
         <x:f>SUM(D5:D10)</x:f>
-        <x:v>514146.28</x:v>
+        <x:v>512425.83999999997</x:v>
       </x:c>
       <x:c r="E11" s="29"/>
       <x:c r="F11" s="29"/>
@@ -1627,15 +1627,15 @@
       </x:c>
       <x:c r="B21" s="66" t="n">
         <x:f>B11+B19</x:f>
-        <x:v>122363</x:v>
+        <x:v>120239</x:v>
       </x:c>
       <x:c r="C21" s="66" t="n">
         <x:f>C11+C19</x:f>
-        <x:v>366674.73333333334</x:v>
+        <x:v>364763.1333333333</x:v>
       </x:c>
       <x:c r="D21" s="66" t="n">
         <x:f>D11+D19</x:f>
-        <x:v>944852.922</x:v>
+        <x:v>943132.482</x:v>
       </x:c>
       <x:c r="E21" s="29"/>
       <x:c r="F21" s="29"/>
@@ -1649,15 +1649,15 @@
       </x:c>
       <x:c r="B22" s="62" t="n">
         <x:f>'Core Monthly'!S16-'Core Monthly'!R16+'Engage Monthly'!S16-'Engage Monthly'!R16</x:f>
-        <x:v>12225</x:v>
+        <x:v>12063</x:v>
       </x:c>
       <x:c r="C22" s="62" t="n">
         <x:f>'Core Monthly'!S28-'Core Monthly'!R28+'Engage Monthly'!S28-'Engage Monthly'!R28</x:f>
-        <x:v>37887.66666666667</x:v>
+        <x:v>37741.866666666676</x:v>
       </x:c>
       <x:c r="D22" s="62" t="n">
         <x:f>'Core Monthly'!S40-'Core Monthly'!R40+'Engage Monthly'!S40-'Engage Monthly'!R40</x:f>
-        <x:v>100298.70100000002</x:v>
+        <x:v>100167.48100000001</x:v>
       </x:c>
       <x:c r="E22" s="29"/>
       <x:c r="F22" s="29"/>
@@ -1671,15 +1671,15 @@
       </x:c>
       <x:c r="B23" s="62" t="n">
         <x:f>B22*12</x:f>
-        <x:v>146700</x:v>
+        <x:v>144756</x:v>
       </x:c>
       <x:c r="C23" s="62" t="n">
         <x:f>C22*12</x:f>
-        <x:v>454652.00000000006</x:v>
+        <x:v>452902.40000000014</x:v>
       </x:c>
       <x:c r="D23" s="62" t="n">
         <x:f>D22*12</x:f>
-        <x:v>1203584.4120000002</x:v>
+        <x:v>1202009.772</x:v>
       </x:c>
       <x:c r="E23" s="29"/>
       <x:c r="F23" s="29"/>
@@ -1693,15 +1693,15 @@
       </x:c>
       <x:c r="B24" s="67" t="n">
         <x:f>(B21-B10-B18)/B21</x:f>
-        <x:v>0.6894486078307985</x:v>
+        <x:v>0.6839627741415015</x:v>
       </x:c>
       <x:c r="C24" s="67" t="n">
         <x:f>(C21-C10-C18)/C21</x:f>
-        <x:v>0.8448215957430755</x:v>
+        <x:v>0.8440083583008298</x:v>
       </x:c>
       <x:c r="D24" s="67" t="n">
         <x:f>(D21-D10-D18)/D21</x:f>
-        <x:v>0.8962272352479427</x:v>
+        <x:v>0.8960379354212508</x:v>
       </x:c>
       <x:c r="E24" s="29"/>
       <x:c r="F24" s="29"/>
@@ -1715,15 +1715,15 @@
       </x:c>
       <x:c r="B25" s="67" t="n">
         <x:f>B11/B21</x:f>
-        <x:v>0.519830340871015</x:v>
+        <x:v>0.5113482314390505</x:v>
       </x:c>
       <x:c r="C25" s="67" t="n">
         <x:f>C11/C21</x:f>
-        <x:v>0.5199669243640276</x:v>
+        <x:v>0.5174512336498919</x:v>
       </x:c>
       <x:c r="D25" s="67" t="n">
         <x:f>D11/D21</x:f>
-        <x:v>0.5441548287872047</x:v>
+        <x:v>0.5433232867914308</x:v>
       </x:c>
       <x:c r="E25" s="29"/>
       <x:c r="F25" s="29"/>
@@ -1737,15 +1737,15 @@
       </x:c>
       <x:c r="B26" s="67" t="n">
         <x:f>B19/B21</x:f>
-        <x:v>0.48016965912898507</x:v>
+        <x:v>0.48865176856094944</x:v>
       </x:c>
       <x:c r="C26" s="67" t="n">
         <x:f>C19/C21</x:f>
-        <x:v>0.48003307563597236</x:v>
+        <x:v>0.4825487663501082</x:v>
       </x:c>
       <x:c r="D26" s="67" t="n">
         <x:f>D19/D21</x:f>
-        <x:v>0.4558451712127954</x:v>
+        <x:v>0.4566767132085692</x:v>
       </x:c>
       <x:c r="E26" s="29"/>
       <x:c r="F26" s="68" t="str">
@@ -1767,15 +1767,15 @@
       </x:c>
       <x:c r="B27" s="62" t="n">
         <x:f>SUM('Core Monthly'!U5:U16)+SUM('Engage Monthly'!U5:U16)</x:f>
-        <x:v>65650.95</x:v>
+        <x:v>64270.35</x:v>
       </x:c>
       <x:c r="C27" s="62" t="n">
         <x:f>SUM('Core Monthly'!U17:U28)+SUM('Engage Monthly'!U17:U28)</x:f>
-        <x:v>224832.7686666667</x:v>
+        <x:v>223532.88066666666</x:v>
       </x:c>
       <x:c r="D27" s="62" t="n">
         <x:f>SUM('Core Monthly'!U29:U40)+SUM('Engage Monthly'!U29:U40)</x:f>
-        <x:v>613164.9212</x:v>
+        <x:v>611960.6132</x:v>
       </x:c>
       <x:c r="E27" s="29"/>
       <x:c r="F27" s="68" t="str">
@@ -1797,15 +1797,15 @@
       </x:c>
       <x:c r="B28" s="67" t="n">
         <x:f>B27/B21</x:f>
-        <x:v>0.5365261557823852</x:v>
+        <x:v>0.534521661025125</x:v>
       </x:c>
       <x:c r="C28" s="67" t="n">
         <x:f>C27/C21</x:f>
-        <x:v>0.613166788512471</x:v>
+        <x:v>0.6128165382941662</x:v>
       </x:c>
       <x:c r="D28" s="67" t="n">
         <x:f>D27/D21</x:f>
-        <x:v>0.6489527702386678</x:v>
+        <x:v>0.6488596510877037</x:v>
       </x:c>
       <x:c r="E28" s="29"/>
       <x:c r="F28" s="68" t="str">
@@ -1869,15 +1869,15 @@
       </x:c>
       <x:c r="B31" s="62" t="n">
         <x:f>'Scenarios'!B5</x:f>
-        <x:v>85458.8</x:v>
+        <x:v>83997.2</x:v>
       </x:c>
       <x:c r="C31" s="62" t="n">
         <x:f>'Scenarios'!C5</x:f>
-        <x:v>268047.05666666664</x:v>
+        <x:v>266877.7766666666</x:v>
       </x:c>
       <x:c r="D31" s="62" t="n">
         <x:f>'Scenarios'!D5</x:f>
-        <x:v>720407.0761</x:v>
+        <x:v>719471.6521</x:v>
       </x:c>
       <x:c r="E31" s="29"/>
       <x:c r="F31" s="29"/>
@@ -1892,15 +1892,15 @@
       </x:c>
       <x:c r="B32" s="62" t="n">
         <x:f>'Scenarios'!B6</x:f>
-        <x:v>122363</x:v>
+        <x:v>120239</x:v>
       </x:c>
       <x:c r="C32" s="62" t="n">
         <x:f>'Scenarios'!C6</x:f>
-        <x:v>366674.73333333334</x:v>
+        <x:v>364763.1333333333</x:v>
       </x:c>
       <x:c r="D32" s="62" t="n">
         <x:f>'Scenarios'!D6</x:f>
-        <x:v>944852.922</x:v>
+        <x:v>943132.482</x:v>
       </x:c>
       <x:c r="E32" s="29"/>
       <x:c r="F32" s="29"/>
@@ -1915,15 +1915,15 @@
       </x:c>
       <x:c r="B33" s="97" t="n">
         <x:f>'Scenarios'!B7</x:f>
-        <x:v>145134</x:v>
+        <x:v>143010</x:v>
       </x:c>
       <x:c r="C33" s="97" t="n">
         <x:f>'Scenarios'!C7</x:f>
-        <x:v>450255.11666666664</x:v>
+        <x:v>448343.51666666666</x:v>
       </x:c>
       <x:c r="D33" s="97" t="n">
         <x:f>'Scenarios'!D7</x:f>
-        <x:v>1199682.4014</x:v>
+        <x:v>1197961.9614</x:v>
       </x:c>
       <x:c r="E33" s="29"/>
       <x:c r="F33" s="29"/>
@@ -1938,15 +1938,15 @@
       </x:c>
       <x:c r="B34" s="99" t="n">
         <x:f>'Scenarios'!B8</x:f>
-        <x:v>158029.61000000002</x:v>
+        <x:v>155574.59</x:v>
       </x:c>
       <x:c r="C34" s="99" t="n">
         <x:f>'Scenarios'!C8</x:f>
-        <x:v>497099.47079999995</x:v>
+        <x:v>494816.3022</x:v>
       </x:c>
       <x:c r="D34" s="99" t="n">
         <x:f>'Scenarios'!D8</x:f>
-        <x:v>1335461.514858</x:v>
+        <x:v>1333338.16806</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1956,7 +1956,7 @@
     <x:mergeCell ref="F26:I28"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd583ce6db775400b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1c3fce70e474fea"/>
 </x:worksheet>
 </file>
 
@@ -2042,26 +2042,26 @@
       </x:c>
       <x:c r="B5" s="49" t="n">
         <x:f>'Scenarios'!B6</x:f>
-        <x:v>122363</x:v>
+        <x:v>120239</x:v>
       </x:c>
       <x:c r="C5" s="49" t="n">
         <x:f>'Scenarios'!C6</x:f>
-        <x:v>366674.73333333334</x:v>
+        <x:v>364763.1333333333</x:v>
       </x:c>
       <x:c r="D5" s="49" t="n">
         <x:f>'Scenarios'!D6</x:f>
-        <x:v>944852.922</x:v>
+        <x:v>943132.482</x:v>
       </x:c>
       <x:c r="I5" t="str">
         <x:v>Y1</x:v>
       </x:c>
       <x:c r="J5" s="49" t="n">
         <x:f>B5</x:f>
-        <x:v>122363</x:v>
+        <x:v>120239</x:v>
       </x:c>
       <x:c r="K5" s="49" t="n">
         <x:f>B6</x:f>
-        <x:v>145134</x:v>
+        <x:v>143010</x:v>
       </x:c>
       <x:c r="L5" s="49" t="n">
         <x:f>B7</x:f>
@@ -2074,30 +2074,30 @@
       </x:c>
       <x:c r="B6" s="111" t="n">
         <x:f>'Scenarios'!B7</x:f>
-        <x:v>145134</x:v>
+        <x:v>143010</x:v>
       </x:c>
       <x:c r="C6" s="111" t="n">
         <x:f>'Scenarios'!C7</x:f>
-        <x:v>450255.11666666664</x:v>
+        <x:v>448343.51666666666</x:v>
       </x:c>
       <x:c r="D6" s="111" t="n">
         <x:f>'Scenarios'!D7</x:f>
-        <x:v>1199682.4014</x:v>
+        <x:v>1197961.9614</x:v>
       </x:c>
       <x:c r="I6" t="str">
         <x:v>Y2</x:v>
       </x:c>
       <x:c r="J6" s="49" t="n">
         <x:f>C5</x:f>
-        <x:v>366674.73333333334</x:v>
+        <x:v>364763.1333333333</x:v>
       </x:c>
       <x:c r="K6" s="49" t="n">
         <x:f>C6</x:f>
-        <x:v>450255.11666666664</x:v>
+        <x:v>448343.51666666666</x:v>
       </x:c>
       <x:c r="L6" s="49" t="n">
         <x:f>C7</x:f>
-        <x:v>83580.3833333333</x:v>
+        <x:v>83580.38333333336</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2110,26 +2110,26 @@
       </x:c>
       <x:c r="C7" s="49" t="n">
         <x:f>C6-C5</x:f>
-        <x:v>83580.3833333333</x:v>
+        <x:v>83580.38333333336</x:v>
       </x:c>
       <x:c r="D7" s="49" t="n">
         <x:f>D6-D5</x:f>
-        <x:v>254829.47940000007</x:v>
+        <x:v>254829.47939999995</x:v>
       </x:c>
       <x:c r="I7" t="str">
         <x:v>Y3</x:v>
       </x:c>
       <x:c r="J7" s="49" t="n">
         <x:f>D5</x:f>
-        <x:v>944852.922</x:v>
+        <x:v>943132.482</x:v>
       </x:c>
       <x:c r="K7" s="49" t="n">
         <x:f>D6</x:f>
-        <x:v>1199682.4014</x:v>
+        <x:v>1197961.9614</x:v>
       </x:c>
       <x:c r="L7" s="49" t="n">
         <x:f>D7</x:f>
-        <x:v>254829.47940000007</x:v>
+        <x:v>254829.47939999995</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
@@ -2576,13 +2576,13 @@
         <x:v>30 active</x:v>
       </x:c>
       <x:c r="E33" s="130" t="str">
-        <x:v>5 active</x:v>
+        <x:v>2 active</x:v>
       </x:c>
       <x:c r="F33" s="130" t="str">
         <x:v>First vertical shortlist</x:v>
       </x:c>
       <x:c r="G33" s="130" t="str">
-        <x:v>Case studies + retention leading indicators</x:v>
+        <x:v>Individual expansion, Team Pro workflow adoption, pilot feedback</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="48" customHeight="1">
@@ -2614,7 +2614,7 @@
     <x:mergeCell ref="A2:L2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raad399a71d6b4c53"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R853061ae7ba54e7a"/>
 </x:worksheet>
 </file>
 
@@ -2684,7 +2684,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>Recruit now, release access mid-Oct 2026, model six full months Nov 2026–Apr 2027, then commercial GA in May 2027.</x:v>
+        <x:v>Recruit now, release access mid-Oct 2026, model six full months Nov 2026–Apr 2027, then commercial GA. Beta target: 30 Individual Pro passes and two founding Team Pro workspaces.</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>Recruit now, release access mid-Oct 2026, model six full months Nov 2026–Apr 2027, then commercial GA in May 2027.</x:v>
@@ -3015,7 +3015,7 @@
         <x:v>46447</x:v>
       </x:c>
       <x:c r="B9" s="29" t="str">
-        <x:v>Expand cohort</x:v>
+        <x:v>Expand individuals</x:v>
       </x:c>
       <x:c r="C9" s="75" t="n">
         <x:f>'Assumptions'!$B$9</x:f>
@@ -3035,11 +3035,11 @@
       </x:c>
       <x:c r="G9" s="75" t="n">
         <x:f>'Assumptions'!$B$12</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H9" s="75" t="n">
         <x:f>H8+G9</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I9" s="75" t="n">
         <x:f>'Assumptions'!$B$13</x:f>
@@ -3047,23 +3047,23 @@
       </x:c>
       <x:c r="J9" s="76" t="n">
         <x:f>G9*I9*'Assumptions'!$B$14</x:f>
-        <x:v>2160</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K9" s="76" t="n">
         <x:f>H9*I9*'Assumptions'!$B$14/12</x:f>
-        <x:v>300</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="L9" s="76" t="n">
         <x:f>E9+J9</x:f>
-        <x:v>5580</x:v>
+        <x:v>3420</x:v>
       </x:c>
       <x:c r="M9" s="76" t="n">
         <x:f>F9+K9</x:f>
-        <x:v>775</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="N9" s="76" t="n">
         <x:f>D9*'Assumptions'!$B$10+H9*I9*'Assumptions'!$B$14</x:f>
-        <x:v>9300</x:v>
+        <x:v>7140</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -3071,7 +3071,7 @@
         <x:v>46478</x:v>
       </x:c>
       <x:c r="B10" s="29" t="str">
-        <x:v>Expand cohort</x:v>
+        <x:v>Expand individuals</x:v>
       </x:c>
       <x:c r="C10" s="75" t="n">
         <x:f>0</x:f>
@@ -3095,7 +3095,7 @@
       </x:c>
       <x:c r="H10" s="75" t="n">
         <x:f>H9+G10</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I10" s="75" t="n">
         <x:f>'Assumptions'!$B$13</x:f>
@@ -3107,7 +3107,7 @@
       </x:c>
       <x:c r="K10" s="76" t="n">
         <x:f>H10*I10*'Assumptions'!$B$14/12</x:f>
-        <x:v>300</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="L10" s="76" t="n">
         <x:f>E10+J10</x:f>
@@ -3115,11 +3115,11 @@
       </x:c>
       <x:c r="M10" s="76" t="n">
         <x:f>F10+K10</x:f>
-        <x:v>775</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="N10" s="76" t="n">
         <x:f>D10*'Assumptions'!$B$10+H10*I10*'Assumptions'!$B$14</x:f>
-        <x:v>9300</x:v>
+        <x:v>7140</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -3158,23 +3158,23 @@
       <x:c r="I12" s="77"/>
       <x:c r="J12" s="78" t="n">
         <x:f>SUM(J5:J10)</x:f>
-        <x:v>3600</x:v>
+        <x:v>1440</x:v>
       </x:c>
       <x:c r="K12" s="78" t="n">
         <x:f>SUM(K5:K10)</x:f>
-        <x:v>1080</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="L12" s="78" t="n">
         <x:f>SUM(L5:L10)</x:f>
-        <x:v>9300</x:v>
+        <x:v>7140</x:v>
       </x:c>
       <x:c r="M12" s="78" t="n">
         <x:f>SUM(M5:M10)</x:f>
-        <x:v>2790</x:v>
+        <x:v>2430</x:v>
       </x:c>
       <x:c r="N12" s="78" t="n">
         <x:f>N10</x:f>
-        <x:v>9300</x:v>
+        <x:v>7140</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -3508,7 +3508,7 @@
         <x:v>BETA — additional team cohort B</x:v>
       </x:c>
       <x:c r="B12" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="32"/>
       <x:c r="D12" s="32"/>
@@ -3519,10 +3519,10 @@
         <x:v>Management target</x:v>
       </x:c>
       <x:c r="G12" s="29" t="str">
-        <x:v>Recruit in Beta</x:v>
+        <x:v>Not targeted</x:v>
       </x:c>
       <x:c r="H12" s="36" t="str">
-        <x:v>Added in Beta month 5; five total at Beta exit</x:v>
+        <x:v>Team Beta target is two founding Team Pro workspaces.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
@@ -3549,7 +3549,7 @@
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="30" t="str">
-        <x:v>BETA — annual team price per seat</x:v>
+        <x:v>BETA — Founding Team Pro price</x:v>
       </x:c>
       <x:c r="B14" s="33" t="n">
         <x:v>240</x:v>
@@ -3560,13 +3560,13 @@
         <x:v>$/seat/year</x:v>
       </x:c>
       <x:c r="F14" s="29" t="str">
-        <x:v>Pricing assumption</x:v>
+        <x:v>Founder price</x:v>
       </x:c>
       <x:c r="G14" s="29" t="str">
-        <x:v>Validate in contracts</x:v>
+        <x:v>Management decision</x:v>
       </x:c>
       <x:c r="H14" s="36" t="str">
-        <x:v>$20 effective monthly price per paid seat</x:v>
+        <x:v>$240 / seat / year Team Pro Beta offer; three-seat minimum per team.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
@@ -3768,7 +3768,7 @@
         <x:v>Validate with pipeline</x:v>
       </x:c>
       <x:c r="H23" s="36" t="str">
-        <x:v>Commercial gross new workspaces; excludes five Beta teams</x:v>
+        <x:v>Commercial gross new workspaces; excludes two Beta teams</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
@@ -3799,7 +3799,7 @@
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
       <x:c r="A25" s="35" t="str">
-        <x:v>CORE — average active seats per team</x:v>
+        <x:v>CORE — avg. paid seats / team</x:v>
       </x:c>
       <x:c r="B25" s="32" t="n">
         <x:v>8</x:v>
@@ -4499,7 +4499,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde3b36c051cc46e6"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R530e210f6ba44b5e"/>
 </x:worksheet>
 </file>
 
@@ -4663,7 +4663,7 @@
       </x:c>
       <x:c r="C6" s="75" t="n">
         <x:f>'Assumptions'!B11+'Assumptions'!B12</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D6" s="75" t="n">
         <x:f>'Assumptions'!B23</x:f>
@@ -4671,7 +4671,7 @@
       </x:c>
       <x:c r="E6" s="75" t="n">
         <x:f>C6*B6+D6</x:f>
-        <x:v>24.5</x:v>
+        <x:v>21.8</x:v>
       </x:c>
       <x:c r="F6" s="75" t="n">
         <x:f>'Assumptions'!C23</x:f>
@@ -4679,7 +4679,7 @@
       </x:c>
       <x:c r="G6" s="75" t="n">
         <x:f>C6*B6^2+D6*B6+F6</x:f>
-        <x:v>52.05</x:v>
+        <x:v>49.620000000000005</x:v>
       </x:c>
       <x:c r="H6" s="75" t="n">
         <x:f>'Assumptions'!D23</x:f>
@@ -4687,7 +4687,7 @@
       </x:c>
       <x:c r="I6" s="75" t="n">
         <x:f>C6*B6^3+D6*B6^2+F6*B6+H6</x:f>
-        <x:v>106.845</x:v>
+        <x:v>104.658</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -5238,11 +5238,11 @@
       </x:c>
       <x:c r="I5" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D5+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D5+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J5" s="76" t="n">
         <x:f>I5*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>300</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="K5" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C5/12</x:f>
@@ -5278,15 +5278,15 @@
       </x:c>
       <x:c r="S5" s="76" t="n">
         <x:f>SUM(F5,H5,J5,L5,N5,P5,R5)</x:f>
-        <x:v>2891.666666666667</x:v>
+        <x:v>2711.666666666667</x:v>
       </x:c>
       <x:c r="T5" s="76" t="n">
         <x:f>(F5+H5+J5+L5+N5)*'Assumptions'!$B$33+P5*'Assumptions'!$B$34+R5*'Assumptions'!$B$35</x:f>
-        <x:v>1602.9166666666667</x:v>
+        <x:v>1539.9166666666667</x:v>
       </x:c>
       <x:c r="U5" s="76" t="n">
         <x:f>S5-T5</x:f>
-        <x:v>1288.7500000000002</x:v>
+        <x:v>1171.7500000000002</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -5320,11 +5320,11 @@
       </x:c>
       <x:c r="I6" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D6+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D6+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J6" s="76" t="n">
         <x:f>I6*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>300</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="K6" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C6/12</x:f>
@@ -5360,15 +5360,15 @@
       </x:c>
       <x:c r="S6" s="76" t="n">
         <x:f>SUM(F6,H6,J6,L6,N6,P6,R6)</x:f>
-        <x:v>3341.666666666667</x:v>
+        <x:v>3161.666666666667</x:v>
       </x:c>
       <x:c r="T6" s="76" t="n">
         <x:f>(F6+H6+J6+L6+N6)*'Assumptions'!$B$33+P6*'Assumptions'!$B$34+R6*'Assumptions'!$B$35</x:f>
-        <x:v>1767.9166666666667</x:v>
+        <x:v>1704.9166666666667</x:v>
       </x:c>
       <x:c r="U6" s="76" t="n">
         <x:f>S6-T6</x:f>
-        <x:v>1573.7500000000002</x:v>
+        <x:v>1456.7500000000002</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -5402,11 +5402,11 @@
       </x:c>
       <x:c r="I7" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D7+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D7+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J7" s="76" t="n">
         <x:f>I7*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>300</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="K7" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C7/12</x:f>
@@ -5442,15 +5442,15 @@
       </x:c>
       <x:c r="S7" s="76" t="n">
         <x:f>SUM(F7,H7,J7,L7,N7,P7,R7)</x:f>
-        <x:v>3791.666666666667</x:v>
+        <x:v>3611.666666666667</x:v>
       </x:c>
       <x:c r="T7" s="76" t="n">
         <x:f>(F7+H7+J7+L7+N7)*'Assumptions'!$B$33+P7*'Assumptions'!$B$34+R7*'Assumptions'!$B$35</x:f>
-        <x:v>1932.9166666666667</x:v>
+        <x:v>1869.9166666666667</x:v>
       </x:c>
       <x:c r="U7" s="76" t="n">
         <x:f>S7-T7</x:f>
-        <x:v>1858.7500000000002</x:v>
+        <x:v>1741.7500000000002</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5484,11 +5484,11 @@
       </x:c>
       <x:c r="I8" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D8+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D8+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J8" s="76" t="n">
         <x:f>I8*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>300</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="K8" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C8/12</x:f>
@@ -5524,15 +5524,15 @@
       </x:c>
       <x:c r="S8" s="76" t="n">
         <x:f>SUM(F8,H8,J8,L8,N8,P8,R8)</x:f>
-        <x:v>4241.666666666667</x:v>
+        <x:v>4061.666666666667</x:v>
       </x:c>
       <x:c r="T8" s="76" t="n">
         <x:f>(F8+H8+J8+L8+N8)*'Assumptions'!$B$33+P8*'Assumptions'!$B$34+R8*'Assumptions'!$B$35</x:f>
-        <x:v>2097.916666666667</x:v>
+        <x:v>2034.9166666666667</x:v>
       </x:c>
       <x:c r="U8" s="76" t="n">
         <x:f>S8-T8</x:f>
-        <x:v>2143.75</x:v>
+        <x:v>2026.7500000000002</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5566,11 +5566,11 @@
       </x:c>
       <x:c r="I9" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D9+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D9+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J9" s="76" t="n">
         <x:f>I9*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>300</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="K9" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C9/12</x:f>
@@ -5606,15 +5606,15 @@
       </x:c>
       <x:c r="S9" s="76" t="n">
         <x:f>SUM(F9,H9,J9,L9,N9,P9,R9)</x:f>
-        <x:v>4691.666666666667</x:v>
+        <x:v>4511.666666666667</x:v>
       </x:c>
       <x:c r="T9" s="76" t="n">
         <x:f>(F9+H9+J9+L9+N9)*'Assumptions'!$B$33+P9*'Assumptions'!$B$34+R9*'Assumptions'!$B$35</x:f>
-        <x:v>2262.916666666667</x:v>
+        <x:v>2199.916666666667</x:v>
       </x:c>
       <x:c r="U9" s="76" t="n">
         <x:f>S9-T9</x:f>
-        <x:v>2428.75</x:v>
+        <x:v>2311.75</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -5648,11 +5648,11 @@
       </x:c>
       <x:c r="I10" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D10+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D10+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J10" s="76" t="n">
         <x:f>I10*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>300</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="K10" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C10/12</x:f>
@@ -5688,15 +5688,15 @@
       </x:c>
       <x:c r="S10" s="76" t="n">
         <x:f>SUM(F10,H10,J10,L10,N10,P10,R10)</x:f>
-        <x:v>5141.666666666667</x:v>
+        <x:v>4961.666666666667</x:v>
       </x:c>
       <x:c r="T10" s="76" t="n">
         <x:f>(F10+H10+J10+L10+N10)*'Assumptions'!$B$33+P10*'Assumptions'!$B$34+R10*'Assumptions'!$B$35</x:f>
-        <x:v>2427.916666666667</x:v>
+        <x:v>2364.916666666667</x:v>
       </x:c>
       <x:c r="U10" s="76" t="n">
         <x:f>S10-T10</x:f>
-        <x:v>2713.75</x:v>
+        <x:v>2596.75</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -5730,11 +5730,11 @@
       </x:c>
       <x:c r="I11" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D11+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D11+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.8</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J11" s="76" t="n">
         <x:f>I11*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>287.99999999999994</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K11" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C11/12</x:f>
@@ -5770,15 +5770,15 @@
       </x:c>
       <x:c r="S11" s="76" t="n">
         <x:f>SUM(F11,H11,J11,L11,N11,P11,R11)</x:f>
-        <x:v>5503.666666666667</x:v>
+        <x:v>5323.666666666667</x:v>
       </x:c>
       <x:c r="T11" s="76" t="n">
         <x:f>(F11+H11+J11+L11+N11)*'Assumptions'!$B$33+P11*'Assumptions'!$B$34+R11*'Assumptions'!$B$35</x:f>
-        <x:v>2562.116666666667</x:v>
+        <x:v>2499.116666666667</x:v>
       </x:c>
       <x:c r="U11" s="76" t="n">
         <x:f>S11-T11</x:f>
-        <x:v>2941.55</x:v>
+        <x:v>2824.55</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -5812,11 +5812,11 @@
       </x:c>
       <x:c r="I12" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D12+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D12+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.8</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J12" s="76" t="n">
         <x:f>I12*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>287.99999999999994</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K12" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C12/12</x:f>
@@ -5852,15 +5852,15 @@
       </x:c>
       <x:c r="S12" s="76" t="n">
         <x:f>SUM(F12,H12,J12,L12,N12,P12,R12)</x:f>
-        <x:v>5953.666666666667</x:v>
+        <x:v>5773.666666666667</x:v>
       </x:c>
       <x:c r="T12" s="76" t="n">
         <x:f>(F12+H12+J12+L12+N12)*'Assumptions'!$B$33+P12*'Assumptions'!$B$34+R12*'Assumptions'!$B$35</x:f>
-        <x:v>2727.116666666667</x:v>
+        <x:v>2664.116666666667</x:v>
       </x:c>
       <x:c r="U12" s="76" t="n">
         <x:f>S12-T12</x:f>
-        <x:v>3226.55</x:v>
+        <x:v>3109.55</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -5894,11 +5894,11 @@
       </x:c>
       <x:c r="I13" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D13+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D13+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.8</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J13" s="76" t="n">
         <x:f>I13*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>287.99999999999994</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K13" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C13/12</x:f>
@@ -5934,15 +5934,15 @@
       </x:c>
       <x:c r="S13" s="76" t="n">
         <x:f>SUM(F13,H13,J13,L13,N13,P13,R13)</x:f>
-        <x:v>6403.666666666667</x:v>
+        <x:v>6223.666666666667</x:v>
       </x:c>
       <x:c r="T13" s="76" t="n">
         <x:f>(F13+H13+J13+L13+N13)*'Assumptions'!$B$33+P13*'Assumptions'!$B$34+R13*'Assumptions'!$B$35</x:f>
-        <x:v>2892.116666666667</x:v>
+        <x:v>2829.116666666667</x:v>
       </x:c>
       <x:c r="U13" s="76" t="n">
         <x:f>S13-T13</x:f>
-        <x:v>3511.55</x:v>
+        <x:v>3394.55</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -5976,11 +5976,11 @@
       </x:c>
       <x:c r="I14" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D14+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D14+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.8</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J14" s="76" t="n">
         <x:f>I14*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>287.99999999999994</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K14" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C14/12</x:f>
@@ -6016,15 +6016,15 @@
       </x:c>
       <x:c r="S14" s="76" t="n">
         <x:f>SUM(F14,H14,J14,L14,N14,P14,R14)</x:f>
-        <x:v>6853.666666666667</x:v>
+        <x:v>6673.666666666667</x:v>
       </x:c>
       <x:c r="T14" s="76" t="n">
         <x:f>(F14+H14+J14+L14+N14)*'Assumptions'!$B$33+P14*'Assumptions'!$B$34+R14*'Assumptions'!$B$35</x:f>
-        <x:v>3057.116666666667</x:v>
+        <x:v>2994.116666666667</x:v>
       </x:c>
       <x:c r="U14" s="76" t="n">
         <x:f>S14-T14</x:f>
-        <x:v>3796.55</x:v>
+        <x:v>3679.55</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -6058,11 +6058,11 @@
       </x:c>
       <x:c r="I15" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D15+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D15+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.5</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J15" s="76" t="n">
         <x:f>I15*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>270</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K15" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C15/12</x:f>
@@ -6098,15 +6098,15 @@
       </x:c>
       <x:c r="S15" s="76" t="n">
         <x:f>SUM(F15,H15,J15,L15,N15,P15,R15)</x:f>
-        <x:v>7171.666666666667</x:v>
+        <x:v>7009.666666666667</x:v>
       </x:c>
       <x:c r="T15" s="76" t="n">
         <x:f>(F15+H15+J15+L15+N15)*'Assumptions'!$B$33+P15*'Assumptions'!$B$34+R15*'Assumptions'!$B$35</x:f>
-        <x:v>3175.916666666667</x:v>
+        <x:v>3119.2166666666667</x:v>
       </x:c>
       <x:c r="U15" s="76" t="n">
         <x:f>S15-T15</x:f>
-        <x:v>3995.75</x:v>
+        <x:v>3890.4500000000003</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -6140,11 +6140,11 @@
       </x:c>
       <x:c r="I16" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D16+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D16+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.5</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J16" s="76" t="n">
         <x:f>I16*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>270</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K16" s="75" t="n">
         <x:f>'Assumptions'!$B$23*C16/12</x:f>
@@ -6180,15 +6180,15 @@
       </x:c>
       <x:c r="S16" s="76" t="n">
         <x:f>SUM(F16,H16,J16,L16,N16,P16,R16)</x:f>
-        <x:v>7621.666666666667</x:v>
+        <x:v>7459.666666666667</x:v>
       </x:c>
       <x:c r="T16" s="76" t="n">
         <x:f>(F16+H16+J16+L16+N16)*'Assumptions'!$B$33+P16*'Assumptions'!$B$34+R16*'Assumptions'!$B$35</x:f>
-        <x:v>3340.916666666667</x:v>
+        <x:v>3284.216666666667</x:v>
       </x:c>
       <x:c r="U16" s="76" t="n">
         <x:f>S16-T16</x:f>
-        <x:v>4280.75</x:v>
+        <x:v>4175.45</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -6222,11 +6222,11 @@
       </x:c>
       <x:c r="I17" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D17+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D17+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.5</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J17" s="76" t="n">
         <x:f>I17*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>270</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K17" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C17/12</x:f>
@@ -6262,15 +6262,15 @@
       </x:c>
       <x:c r="S17" s="76" t="n">
         <x:f>SUM(F17,H17,J17,L17,N17,P17,R17)</x:f>
-        <x:v>9350.388888888889</x:v>
+        <x:v>9188.388888888889</x:v>
       </x:c>
       <x:c r="T17" s="76" t="n">
         <x:f>(F17+H17+J17+L17+N17)*'Assumptions'!$C$33+P17*'Assumptions'!$C$34+R17*'Assumptions'!$C$35</x:f>
-        <x:v>3981.8994444444443</x:v>
+        <x:v>3930.059444444444</x:v>
       </x:c>
       <x:c r="U17" s="76" t="n">
         <x:f>S17-T17</x:f>
-        <x:v>5368.489444444444</x:v>
+        <x:v>5258.329444444445</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -6304,11 +6304,11 @@
       </x:c>
       <x:c r="I18" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D18+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D18+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.5</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J18" s="76" t="n">
         <x:f>I18*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>270</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K18" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C18/12</x:f>
@@ -6344,15 +6344,15 @@
       </x:c>
       <x:c r="S18" s="76" t="n">
         <x:f>SUM(F18,H18,J18,L18,N18,P18,R18)</x:f>
-        <x:v>10546.777777777777</x:v>
+        <x:v>10384.777777777777</x:v>
       </x:c>
       <x:c r="T18" s="76" t="n">
         <x:f>(F18+H18+J18+L18+N18)*'Assumptions'!$C$33+P18*'Assumptions'!$C$34+R18*'Assumptions'!$C$35</x:f>
-        <x:v>4389.118888888888</x:v>
+        <x:v>4337.278888888889</x:v>
       </x:c>
       <x:c r="U18" s="76" t="n">
         <x:f>S18-T18</x:f>
-        <x:v>6157.658888888889</x:v>
+        <x:v>6047.498888888888</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -6386,11 +6386,11 @@
       </x:c>
       <x:c r="I19" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D19+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D19+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.5</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J19" s="76" t="n">
         <x:f>I19*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>270</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K19" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C19/12</x:f>
@@ -6426,15 +6426,15 @@
       </x:c>
       <x:c r="S19" s="76" t="n">
         <x:f>SUM(F19,H19,J19,L19,N19,P19,R19)</x:f>
-        <x:v>11743.166666666666</x:v>
+        <x:v>11581.166666666668</x:v>
       </x:c>
       <x:c r="T19" s="76" t="n">
         <x:f>(F19+H19+J19+L19+N19)*'Assumptions'!$C$33+P19*'Assumptions'!$C$34+R19*'Assumptions'!$C$35</x:f>
-        <x:v>4796.338333333333</x:v>
+        <x:v>4744.498333333333</x:v>
       </x:c>
       <x:c r="U19" s="76" t="n">
         <x:f>S19-T19</x:f>
-        <x:v>6946.828333333333</x:v>
+        <x:v>6836.668333333335</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -6468,11 +6468,11 @@
       </x:c>
       <x:c r="I20" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D20+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D20+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.5</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J20" s="76" t="n">
         <x:f>I20*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>270</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K20" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C20/12</x:f>
@@ -6508,15 +6508,15 @@
       </x:c>
       <x:c r="S20" s="76" t="n">
         <x:f>SUM(F20,H20,J20,L20,N20,P20,R20)</x:f>
-        <x:v>12939.555555555555</x:v>
+        <x:v>12777.555555555555</x:v>
       </x:c>
       <x:c r="T20" s="76" t="n">
         <x:f>(F20+H20+J20+L20+N20)*'Assumptions'!$C$33+P20*'Assumptions'!$C$34+R20*'Assumptions'!$C$35</x:f>
-        <x:v>5203.557777777778</x:v>
+        <x:v>5151.717777777778</x:v>
       </x:c>
       <x:c r="U20" s="76" t="n">
         <x:f>S20-T20</x:f>
-        <x:v>7735.997777777777</x:v>
+        <x:v>7625.837777777777</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -6550,11 +6550,11 @@
       </x:c>
       <x:c r="I21" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D21+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D21+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.5</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J21" s="76" t="n">
         <x:f>I21*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>270</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K21" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C21/12</x:f>
@@ -6590,15 +6590,15 @@
       </x:c>
       <x:c r="S21" s="76" t="n">
         <x:f>SUM(F21,H21,J21,L21,N21,P21,R21)</x:f>
-        <x:v>14135.944444444445</x:v>
+        <x:v>13973.944444444445</x:v>
       </x:c>
       <x:c r="T21" s="76" t="n">
         <x:f>(F21+H21+J21+L21+N21)*'Assumptions'!$C$33+P21*'Assumptions'!$C$34+R21*'Assumptions'!$C$35</x:f>
-        <x:v>5610.777222222223</x:v>
+        <x:v>5558.937222222223</x:v>
       </x:c>
       <x:c r="U21" s="76" t="n">
         <x:f>S21-T21</x:f>
-        <x:v>8525.167222222222</x:v>
+        <x:v>8415.007222222222</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -6632,11 +6632,11 @@
       </x:c>
       <x:c r="I22" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D22+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D22+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.5</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J22" s="76" t="n">
         <x:f>I22*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>270</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K22" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C22/12</x:f>
@@ -6672,15 +6672,15 @@
       </x:c>
       <x:c r="S22" s="76" t="n">
         <x:f>SUM(F22,H22,J22,L22,N22,P22,R22)</x:f>
-        <x:v>15332.333333333334</x:v>
+        <x:v>15170.333333333334</x:v>
       </x:c>
       <x:c r="T22" s="76" t="n">
         <x:f>(F22+H22+J22+L22+N22)*'Assumptions'!$C$33+P22*'Assumptions'!$C$34+R22*'Assumptions'!$C$35</x:f>
-        <x:v>6017.996666666667</x:v>
+        <x:v>5966.156666666667</x:v>
       </x:c>
       <x:c r="U22" s="76" t="n">
         <x:f>S22-T22</x:f>
-        <x:v>9314.336666666666</x:v>
+        <x:v>9204.176666666666</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -6714,11 +6714,11 @@
       </x:c>
       <x:c r="I23" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D23+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D23+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.32</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J23" s="76" t="n">
         <x:f>I23*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>259.2</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K23" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C23/12</x:f>
@@ -6754,15 +6754,15 @@
       </x:c>
       <x:c r="S23" s="76" t="n">
         <x:f>SUM(F23,H23,J23,L23,N23,P23,R23)</x:f>
-        <x:v>16472.322222222225</x:v>
+        <x:v>16310.322222222223</x:v>
       </x:c>
       <x:c r="T23" s="76" t="n">
         <x:f>(F23+H23+J23+L23+N23)*'Assumptions'!$C$33+P23*'Assumptions'!$C$34+R23*'Assumptions'!$C$35</x:f>
-        <x:v>6407.168111111112</x:v>
+        <x:v>6355.328111111112</x:v>
       </x:c>
       <x:c r="U23" s="76" t="n">
         <x:f>S23-T23</x:f>
-        <x:v>10065.154111111113</x:v>
+        <x:v>9954.994111111111</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -6796,11 +6796,11 @@
       </x:c>
       <x:c r="I24" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D24+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D24+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.32</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J24" s="76" t="n">
         <x:f>I24*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>259.2</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K24" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C24/12</x:f>
@@ -6836,15 +6836,15 @@
       </x:c>
       <x:c r="S24" s="76" t="n">
         <x:f>SUM(F24,H24,J24,L24,N24,P24,R24)</x:f>
-        <x:v>17668.711111111108</x:v>
+        <x:v>17506.711111111108</x:v>
       </x:c>
       <x:c r="T24" s="76" t="n">
         <x:f>(F24+H24+J24+L24+N24)*'Assumptions'!$C$33+P24*'Assumptions'!$C$34+R24*'Assumptions'!$C$35</x:f>
-        <x:v>6814.387555555555</x:v>
+        <x:v>6762.547555555555</x:v>
       </x:c>
       <x:c r="U24" s="76" t="n">
         <x:f>S24-T24</x:f>
-        <x:v>10854.323555555553</x:v>
+        <x:v>10744.163555555553</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -6878,11 +6878,11 @@
       </x:c>
       <x:c r="I25" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D25+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D25+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.32</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J25" s="76" t="n">
         <x:f>I25*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>259.2</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K25" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C25/12</x:f>
@@ -6918,15 +6918,15 @@
       </x:c>
       <x:c r="S25" s="76" t="n">
         <x:f>SUM(F25,H25,J25,L25,N25,P25,R25)</x:f>
-        <x:v>18865.1</x:v>
+        <x:v>18703.1</x:v>
       </x:c>
       <x:c r="T25" s="76" t="n">
         <x:f>(F25+H25+J25+L25+N25)*'Assumptions'!$C$33+P25*'Assumptions'!$C$34+R25*'Assumptions'!$C$35</x:f>
-        <x:v>7221.607</x:v>
+        <x:v>7169.767</x:v>
       </x:c>
       <x:c r="U25" s="76" t="n">
         <x:f>S25-T25</x:f>
-        <x:v>11643.492999999999</x:v>
+        <x:v>11533.332999999999</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -6960,11 +6960,11 @@
       </x:c>
       <x:c r="I26" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D26+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D26+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.32</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J26" s="76" t="n">
         <x:f>I26*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>259.2</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K26" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C26/12</x:f>
@@ -7000,15 +7000,15 @@
       </x:c>
       <x:c r="S26" s="76" t="n">
         <x:f>SUM(F26,H26,J26,L26,N26,P26,R26)</x:f>
-        <x:v>20061.48888888889</x:v>
+        <x:v>19899.48888888889</x:v>
       </x:c>
       <x:c r="T26" s="76" t="n">
         <x:f>(F26+H26+J26+L26+N26)*'Assumptions'!$C$33+P26*'Assumptions'!$C$34+R26*'Assumptions'!$C$35</x:f>
-        <x:v>7628.826444444445</x:v>
+        <x:v>7576.986444444445</x:v>
       </x:c>
       <x:c r="U26" s="76" t="n">
         <x:f>S26-T26</x:f>
-        <x:v>12432.662444444444</x:v>
+        <x:v>12322.502444444444</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -7042,11 +7042,11 @@
       </x:c>
       <x:c r="I27" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D27+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D27+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.050000000000001</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J27" s="76" t="n">
         <x:f>I27*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>243.00000000000003</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K27" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C27/12</x:f>
@@ -7082,15 +7082,15 @@
       </x:c>
       <x:c r="S27" s="76" t="n">
         <x:f>SUM(F27,H27,J27,L27,N27,P27,R27)</x:f>
-        <x:v>21173.277777777777</x:v>
+        <x:v>21027.477777777778</x:v>
       </x:c>
       <x:c r="T27" s="76" t="n">
         <x:f>(F27+H27+J27+L27+N27)*'Assumptions'!$C$33+P27*'Assumptions'!$C$34+R27*'Assumptions'!$C$35</x:f>
-        <x:v>8008.973888888889</x:v>
+        <x:v>7962.317888888889</x:v>
       </x:c>
       <x:c r="U27" s="76" t="n">
         <x:f>S27-T27</x:f>
-        <x:v>13164.303888888888</x:v>
+        <x:v>13065.15988888889</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -7124,11 +7124,11 @@
       </x:c>
       <x:c r="I28" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D28+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D28+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.050000000000001</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J28" s="76" t="n">
         <x:f>I28*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>243.00000000000003</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K28" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24+'Assumptions'!$C$23*C28/12</x:f>
@@ -7164,15 +7164,15 @@
       </x:c>
       <x:c r="S28" s="76" t="n">
         <x:f>SUM(F28,H28,J28,L28,N28,P28,R28)</x:f>
-        <x:v>22369.666666666668</x:v>
+        <x:v>22223.86666666667</x:v>
       </x:c>
       <x:c r="T28" s="76" t="n">
         <x:f>(F28+H28+J28+L28+N28)*'Assumptions'!$C$33+P28*'Assumptions'!$C$34+R28*'Assumptions'!$C$35</x:f>
-        <x:v>8416.193333333333</x:v>
+        <x:v>8369.537333333334</x:v>
       </x:c>
       <x:c r="U28" s="76" t="n">
         <x:f>S28-T28</x:f>
-        <x:v>13953.473333333335</x:v>
+        <x:v>13854.329333333335</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -7206,11 +7206,11 @@
       </x:c>
       <x:c r="I29" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D29+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D29+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.050000000000001</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J29" s="76" t="n">
         <x:f>I29*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>243.00000000000003</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K29" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C29/12</x:f>
@@ -7246,15 +7246,15 @@
       </x:c>
       <x:c r="S29" s="76" t="n">
         <x:f>SUM(F29,H29,J29,L29,N29,P29,R29)</x:f>
-        <x:v>25869.166666666664</x:v>
+        <x:v>25723.366666666665</x:v>
       </x:c>
       <x:c r="T29" s="76" t="n">
         <x:f>(F29+H29+J29+L29+N29)*'Assumptions'!$D$33+P29*'Assumptions'!$D$34+R29*'Assumptions'!$D$35</x:f>
-        <x:v>9664.55</x:v>
+        <x:v>9620.81</x:v>
       </x:c>
       <x:c r="U29" s="76" t="n">
         <x:f>S29-T29</x:f>
-        <x:v>16204.616666666665</x:v>
+        <x:v>16102.556666666665</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -7288,11 +7288,11 @@
       </x:c>
       <x:c r="I30" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D30+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D30+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.050000000000001</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J30" s="76" t="n">
         <x:f>I30*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>243.00000000000003</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K30" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C30/12</x:f>
@@ -7328,15 +7328,15 @@
       </x:c>
       <x:c r="S30" s="76" t="n">
         <x:f>SUM(F30,H30,J30,L30,N30,P30,R30)</x:f>
-        <x:v>28960.833333333332</x:v>
+        <x:v>28815.033333333333</x:v>
       </x:c>
       <x:c r="T30" s="76" t="n">
         <x:f>(F30+H30+J30+L30+N30)*'Assumptions'!$D$33+P30*'Assumptions'!$D$34+R30*'Assumptions'!$D$35</x:f>
-        <x:v>10652.05</x:v>
+        <x:v>10608.31</x:v>
       </x:c>
       <x:c r="U30" s="76" t="n">
         <x:f>S30-T30</x:f>
-        <x:v>18308.783333333333</x:v>
+        <x:v>18206.723333333335</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -7370,11 +7370,11 @@
       </x:c>
       <x:c r="I31" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D31+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D31+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.050000000000001</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J31" s="76" t="n">
         <x:f>I31*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>243.00000000000003</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K31" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C31/12</x:f>
@@ -7410,15 +7410,15 @@
       </x:c>
       <x:c r="S31" s="76" t="n">
         <x:f>SUM(F31,H31,J31,L31,N31,P31,R31)</x:f>
-        <x:v>32052.5</x:v>
+        <x:v>31906.7</x:v>
       </x:c>
       <x:c r="T31" s="76" t="n">
         <x:f>(F31+H31+J31+L31+N31)*'Assumptions'!$D$33+P31*'Assumptions'!$D$34+R31*'Assumptions'!$D$35</x:f>
-        <x:v>11639.55</x:v>
+        <x:v>11595.81</x:v>
       </x:c>
       <x:c r="U31" s="76" t="n">
         <x:f>S31-T31</x:f>
-        <x:v>20412.95</x:v>
+        <x:v>20310.89</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -7452,11 +7452,11 @@
       </x:c>
       <x:c r="I32" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D32+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D32+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.050000000000001</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J32" s="76" t="n">
         <x:f>I32*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>243.00000000000003</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K32" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C32/12</x:f>
@@ -7492,15 +7492,15 @@
       </x:c>
       <x:c r="S32" s="76" t="n">
         <x:f>SUM(F32,H32,J32,L32,N32,P32,R32)</x:f>
-        <x:v>35144.166666666664</x:v>
+        <x:v>34998.36666666667</x:v>
       </x:c>
       <x:c r="T32" s="76" t="n">
         <x:f>(F32+H32+J32+L32+N32)*'Assumptions'!$D$33+P32*'Assumptions'!$D$34+R32*'Assumptions'!$D$35</x:f>
-        <x:v>12627.05</x:v>
+        <x:v>12583.31</x:v>
       </x:c>
       <x:c r="U32" s="76" t="n">
         <x:f>S32-T32</x:f>
-        <x:v>22517.116666666665</x:v>
+        <x:v>22415.05666666667</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -7534,11 +7534,11 @@
       </x:c>
       <x:c r="I33" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D33+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D33+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.050000000000001</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J33" s="76" t="n">
         <x:f>I33*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>243.00000000000003</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K33" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C33/12</x:f>
@@ -7574,15 +7574,15 @@
       </x:c>
       <x:c r="S33" s="76" t="n">
         <x:f>SUM(F33,H33,J33,L33,N33,P33,R33)</x:f>
-        <x:v>38235.833333333336</x:v>
+        <x:v>38090.03333333334</x:v>
       </x:c>
       <x:c r="T33" s="76" t="n">
         <x:f>(F33+H33+J33+L33+N33)*'Assumptions'!$D$33+P33*'Assumptions'!$D$34+R33*'Assumptions'!$D$35</x:f>
-        <x:v>13614.550000000001</x:v>
+        <x:v>13570.810000000001</x:v>
       </x:c>
       <x:c r="U33" s="76" t="n">
         <x:f>S33-T33</x:f>
-        <x:v>24621.283333333333</x:v>
+        <x:v>24519.22333333334</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -7616,11 +7616,11 @@
       </x:c>
       <x:c r="I34" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D34+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D34+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>4.050000000000001</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J34" s="76" t="n">
         <x:f>I34*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>243.00000000000003</x:v>
+        <x:v>97.2</x:v>
       </x:c>
       <x:c r="K34" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C34/12</x:f>
@@ -7656,15 +7656,15 @@
       </x:c>
       <x:c r="S34" s="76" t="n">
         <x:f>SUM(F34,H34,J34,L34,N34,P34,R34)</x:f>
-        <x:v>41327.5</x:v>
+        <x:v>41181.7</x:v>
       </x:c>
       <x:c r="T34" s="76" t="n">
         <x:f>(F34+H34+J34+L34+N34)*'Assumptions'!$D$33+P34*'Assumptions'!$D$34+R34*'Assumptions'!$D$35</x:f>
-        <x:v>14602.050000000001</x:v>
+        <x:v>14558.310000000001</x:v>
       </x:c>
       <x:c r="U34" s="76" t="n">
         <x:f>S34-T34</x:f>
-        <x:v>26725.449999999997</x:v>
+        <x:v>26623.389999999996</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -7698,11 +7698,11 @@
       </x:c>
       <x:c r="I35" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D35+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D35+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>3.8880000000000003</x:v>
+        <x:v>1.4580000000000002</x:v>
       </x:c>
       <x:c r="J35" s="76" t="n">
         <x:f>I35*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>233.28000000000006</x:v>
+        <x:v>87.48000000000002</x:v>
       </x:c>
       <x:c r="K35" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C35/12</x:f>
@@ -7738,15 +7738,15 @@
       </x:c>
       <x:c r="S35" s="76" t="n">
         <x:f>SUM(F35,H35,J35,L35,N35,P35,R35)</x:f>
-        <x:v>44382.08666666667</x:v>
+        <x:v>44236.28666666667</x:v>
       </x:c>
       <x:c r="T35" s="76" t="n">
         <x:f>(F35+H35+J35+L35+N35)*'Assumptions'!$D$33+P35*'Assumptions'!$D$34+R35*'Assumptions'!$D$35</x:f>
-        <x:v>15578.426000000001</x:v>
+        <x:v>15534.686</x:v>
       </x:c>
       <x:c r="U35" s="76" t="n">
         <x:f>S35-T35</x:f>
-        <x:v>28803.66066666667</x:v>
+        <x:v>28701.600666666665</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -7780,11 +7780,11 @@
       </x:c>
       <x:c r="I36" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D36+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D36+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>3.8880000000000003</x:v>
+        <x:v>1.4580000000000002</x:v>
       </x:c>
       <x:c r="J36" s="76" t="n">
         <x:f>I36*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>233.28000000000006</x:v>
+        <x:v>87.48000000000002</x:v>
       </x:c>
       <x:c r="K36" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C36/12</x:f>
@@ -7820,15 +7820,15 @@
       </x:c>
       <x:c r="S36" s="76" t="n">
         <x:f>SUM(F36,H36,J36,L36,N36,P36,R36)</x:f>
-        <x:v>47473.75333333333</x:v>
+        <x:v>47327.95333333333</x:v>
       </x:c>
       <x:c r="T36" s="76" t="n">
         <x:f>(F36+H36+J36+L36+N36)*'Assumptions'!$D$33+P36*'Assumptions'!$D$34+R36*'Assumptions'!$D$35</x:f>
-        <x:v>16565.926</x:v>
+        <x:v>16522.186</x:v>
       </x:c>
       <x:c r="U36" s="76" t="n">
         <x:f>S36-T36</x:f>
-        <x:v>30907.827333333327</x:v>
+        <x:v>30805.76733333333</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -7862,11 +7862,11 @@
       </x:c>
       <x:c r="I37" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D37+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D37+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>3.8880000000000003</x:v>
+        <x:v>1.4580000000000002</x:v>
       </x:c>
       <x:c r="J37" s="76" t="n">
         <x:f>I37*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>233.28000000000006</x:v>
+        <x:v>87.48000000000002</x:v>
       </x:c>
       <x:c r="K37" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C37/12</x:f>
@@ -7902,15 +7902,15 @@
       </x:c>
       <x:c r="S37" s="76" t="n">
         <x:f>SUM(F37,H37,J37,L37,N37,P37,R37)</x:f>
-        <x:v>50565.42</x:v>
+        <x:v>50419.619999999995</x:v>
       </x:c>
       <x:c r="T37" s="76" t="n">
         <x:f>(F37+H37+J37+L37+N37)*'Assumptions'!$D$33+P37*'Assumptions'!$D$34+R37*'Assumptions'!$D$35</x:f>
-        <x:v>17553.426</x:v>
+        <x:v>17509.686</x:v>
       </x:c>
       <x:c r="U37" s="76" t="n">
         <x:f>S37-T37</x:f>
-        <x:v>33011.994</x:v>
+        <x:v>32909.933999999994</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -7944,11 +7944,11 @@
       </x:c>
       <x:c r="I38" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D38+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D38+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>3.8880000000000003</x:v>
+        <x:v>1.4580000000000002</x:v>
       </x:c>
       <x:c r="J38" s="76" t="n">
         <x:f>I38*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>233.28000000000006</x:v>
+        <x:v>87.48000000000002</x:v>
       </x:c>
       <x:c r="K38" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C38/12</x:f>
@@ -7984,15 +7984,15 @@
       </x:c>
       <x:c r="S38" s="76" t="n">
         <x:f>SUM(F38,H38,J38,L38,N38,P38,R38)</x:f>
-        <x:v>53657.08666666667</x:v>
+        <x:v>53511.286666666674</x:v>
       </x:c>
       <x:c r="T38" s="76" t="n">
         <x:f>(F38+H38+J38+L38+N38)*'Assumptions'!$D$33+P38*'Assumptions'!$D$34+R38*'Assumptions'!$D$35</x:f>
-        <x:v>18540.926</x:v>
+        <x:v>18497.186</x:v>
       </x:c>
       <x:c r="U38" s="76" t="n">
         <x:f>S38-T38</x:f>
-        <x:v>35116.16066666667</x:v>
+        <x:v>35014.10066666667</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -8026,11 +8026,11 @@
       </x:c>
       <x:c r="I39" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D39+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D39+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>3.6450000000000005</x:v>
+        <x:v>1.4580000000000002</x:v>
       </x:c>
       <x:c r="J39" s="76" t="n">
         <x:f>I39*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>218.70000000000005</x:v>
+        <x:v>87.48000000000002</x:v>
       </x:c>
       <x:c r="K39" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C39/12</x:f>
@@ -8066,15 +8066,15 @@
       </x:c>
       <x:c r="S39" s="76" t="n">
         <x:f>SUM(F39,H39,J39,L39,N39,P39,R39)</x:f>
-        <x:v>56693.13333333333</x:v>
+        <x:v>56561.91333333333</x:v>
       </x:c>
       <x:c r="T39" s="76" t="n">
         <x:f>(F39+H39+J39+L39+N39)*'Assumptions'!$D$33+P39*'Assumptions'!$D$34+R39*'Assumptions'!$D$35</x:f>
-        <x:v>19511.739999999998</x:v>
+        <x:v>19472.374</x:v>
       </x:c>
       <x:c r="U39" s="76" t="n">
         <x:f>S39-T39</x:f>
-        <x:v>37181.39333333333</x:v>
+        <x:v>37089.539333333334</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -8108,11 +8108,11 @@
       </x:c>
       <x:c r="I40" s="75" t="n">
         <x:f>'Assumptions'!$B$11*POWER('Assumptions'!$B$16,INT((D40+11-'Assumptions'!$B$17)/12))+'Assumptions'!$B$12*POWER('Assumptions'!$B$16,INT((D40+11-'Assumptions'!$B$18)/12))</x:f>
-        <x:v>3.6450000000000005</x:v>
+        <x:v>1.4580000000000002</x:v>
       </x:c>
       <x:c r="J40" s="76" t="n">
         <x:f>I40*'Assumptions'!$B$13*'Assumptions'!$B$14/12</x:f>
-        <x:v>218.70000000000005</x:v>
+        <x:v>87.48000000000002</x:v>
       </x:c>
       <x:c r="K40" s="75" t="n">
         <x:f>'Assumptions'!$B$23*'Assumptions'!$B$24^2+'Assumptions'!$C$23*'Assumptions'!$C$24+'Assumptions'!$D$23*C40/12</x:f>
@@ -8148,15 +8148,15 @@
       </x:c>
       <x:c r="S40" s="76" t="n">
         <x:f>SUM(F40,H40,J40,L40,N40,P40,R40)</x:f>
-        <x:v>59784.8</x:v>
+        <x:v>59653.58</x:v>
       </x:c>
       <x:c r="T40" s="76" t="n">
         <x:f>(F40+H40+J40+L40+N40)*'Assumptions'!$D$33+P40*'Assumptions'!$D$34+R40*'Assumptions'!$D$35</x:f>
-        <x:v>20499.24</x:v>
+        <x:v>20459.874</x:v>
       </x:c>
       <x:c r="U40" s="76" t="n">
         <x:f>S40-T40</x:f>
-        <x:v>39285.56</x:v>
+        <x:v>39193.706000000006</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11600,15 +11600,15 @@
       </x:c>
       <x:c r="B5" s="62" t="n">
         <x:f>R16</x:f>
-        <x:v>85458.8</x:v>
+        <x:v>83997.2</x:v>
       </x:c>
       <x:c r="C5" s="62" t="n">
         <x:f>R17</x:f>
-        <x:v>268047.05666666664</x:v>
+        <x:v>266877.7766666666</x:v>
       </x:c>
       <x:c r="D5" s="62" t="n">
         <x:f>R18</x:f>
-        <x:v>720407.0761</x:v>
+        <x:v>719471.6521</x:v>
       </x:c>
       <x:c r="E5" s="29"/>
       <x:c r="F5" s="29"/>
@@ -11631,15 +11631,15 @@
       </x:c>
       <x:c r="B6" s="62" t="n">
         <x:f>R19</x:f>
-        <x:v>122363</x:v>
+        <x:v>120239</x:v>
       </x:c>
       <x:c r="C6" s="62" t="n">
         <x:f>R20</x:f>
-        <x:v>366674.73333333334</x:v>
+        <x:v>364763.1333333333</x:v>
       </x:c>
       <x:c r="D6" s="62" t="n">
         <x:f>R21</x:f>
-        <x:v>944852.922</x:v>
+        <x:v>943132.482</x:v>
       </x:c>
       <x:c r="E6" s="29"/>
       <x:c r="F6" s="29"/>
@@ -11663,15 +11663,15 @@
       </x:c>
       <x:c r="B7" s="97" t="n">
         <x:f>$R$25</x:f>
-        <x:v>145134</x:v>
+        <x:v>143010</x:v>
       </x:c>
       <x:c r="C7" s="97" t="n">
         <x:f>$R$26</x:f>
-        <x:v>450255.11666666664</x:v>
+        <x:v>448343.51666666666</x:v>
       </x:c>
       <x:c r="D7" s="97" t="n">
         <x:f>$R$27</x:f>
-        <x:v>1199682.4014</x:v>
+        <x:v>1197961.9614</x:v>
       </x:c>
       <x:c r="E7" s="29"/>
       <x:c r="F7" s="29"/>
@@ -11695,15 +11695,15 @@
       </x:c>
       <x:c r="B8" s="62" t="n">
         <x:f>$R$22</x:f>
-        <x:v>158029.61000000002</x:v>
+        <x:v>155574.59</x:v>
       </x:c>
       <x:c r="C8" s="62" t="n">
         <x:f>$R$23</x:f>
-        <x:v>497099.47079999995</x:v>
+        <x:v>494816.3022</x:v>
       </x:c>
       <x:c r="D8" s="62" t="n">
         <x:f>$R$24</x:f>
-        <x:v>1335461.514858</x:v>
+        <x:v>1333338.16806</x:v>
       </x:c>
       <x:c r="E8" s="29"/>
       <x:c r="F8" s="29"/>
@@ -12007,7 +12007,7 @@
       </x:c>
       <x:c r="H16" s="62" t="n">
         <x:f>$C16*(('Assumptions'!$B$8*(6*$E16^0+6*$E16^1)+'Assumptions'!$B$9*(10*$E16^0+2*$E16^1))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F16^0+6*$F16^1)+'Assumptions'!$B$12*(10*$F16^0+2*$F16^1))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>5760.299999999999</x:v>
+        <x:v>4298.7</x:v>
       </x:c>
       <x:c r="I16" s="62" t="n">
         <x:f>('Assumptions'!$B$20*$D16*6.5)*'Assumptions'!$B$22</x:f>
@@ -12031,7 +12031,7 @@
       </x:c>
       <x:c r="N16" s="62" t="n">
         <x:f>SUM(H16:M16)</x:f>
-        <x:v>44330.3</x:v>
+        <x:v>42868.7</x:v>
       </x:c>
       <x:c r="O16" s="62" t="n">
         <x:f>'Assumptions'!$B$37*$D16*6.5*'Assumptions'!$B$38+'Assumptions'!$B$39*$D16*6.5*'Assumptions'!$B$40+'Assumptions'!$B$41*$D16*6.5*'Assumptions'!$B$42+'Assumptions'!$B$43*$D16*6.5*'Assumptions'!$B$44</x:f>
@@ -12047,7 +12047,7 @@
       </x:c>
       <x:c r="R16" s="62" t="n">
         <x:f>N16+O16+P16+Q16</x:f>
-        <x:v>85458.8</x:v>
+        <x:v>83997.2</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -12081,7 +12081,7 @@
       </x:c>
       <x:c r="H17" s="62" t="n">
         <x:f>$C17*(('Assumptions'!$B$8*(6*$E17^1+6*$E17^2)+'Assumptions'!$B$9*(10*$E17^1+2*$E17^2))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F17^1+6*$F17^2)+'Assumptions'!$B$12*(10*$F17^1+2*$F17^2))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>3590.7900000000004</x:v>
+        <x:v>2421.5099999999998</x:v>
       </x:c>
       <x:c r="I17" s="62" t="n">
         <x:f>('Assumptions'!$B$20*$D16*$E17*12+'Assumptions'!$C$20*$D17*6.5)*'Assumptions'!$C$22</x:f>
@@ -12105,7 +12105,7 @@
       </x:c>
       <x:c r="N17" s="62" t="n">
         <x:f>SUM(H17:M17)</x:f>
-        <x:v>139272.65666666668</x:v>
+        <x:v>138103.37666666665</x:v>
       </x:c>
       <x:c r="O17" s="62" t="n">
         <x:f>('Assumptions'!$B$37*$D16*$F17*12+'Assumptions'!$C$37*$D17*6.5)*'Assumptions'!$C$38+('Assumptions'!$B$39*$D16*$F17*12+'Assumptions'!$C$39*$D17*6.5)*'Assumptions'!$C$40+('Assumptions'!$B$41*$D16*$F17*12+'Assumptions'!$C$41*$D17*6.5)*'Assumptions'!$C$42+('Assumptions'!$B$43*$D16*$F17*12+'Assumptions'!$C$43*$D17*6.5)*'Assumptions'!$C$44</x:f>
@@ -12121,7 +12121,7 @@
       </x:c>
       <x:c r="R17" s="62" t="n">
         <x:f>N17+O17+P17+Q17</x:f>
-        <x:v>268047.05666666664</x:v>
+        <x:v>266877.7766666666</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -12155,7 +12155,7 @@
       </x:c>
       <x:c r="H18" s="62" t="n">
         <x:f>$C18*(('Assumptions'!$B$8*(6*$E18^2+6*$E18^3)+'Assumptions'!$B$9*(10*$E18^2+2*$E18^3))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F18^2+6*$F18^3)+'Assumptions'!$B$12*(10*$F18^2+2*$F18^3))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>2363.907</x:v>
+        <x:v>1428.483</x:v>
       </x:c>
       <x:c r="I18" s="62" t="n">
         <x:f>('Assumptions'!$B$20*$D16*$E18^2*12+'Assumptions'!$C$20*$D17*$E18*12+'Assumptions'!$D$20*$D18*6.5)*'Assumptions'!$D$22</x:f>
@@ -12179,7 +12179,7 @@
       </x:c>
       <x:c r="N18" s="62" t="n">
         <x:f>SUM(H18:M18)</x:f>
-        <x:v>391793.50700000004</x:v>
+        <x:v>390858.083</x:v>
       </x:c>
       <x:c r="O18" s="62" t="n">
         <x:f>('Assumptions'!$B$37*$D16*$F18^2*12+'Assumptions'!$C$37*$D17*$F18*12+'Assumptions'!$D$37*$D18*6.5)*'Assumptions'!$D$38+('Assumptions'!$B$39*$D16*$F18^2*12+'Assumptions'!$C$39*$D17*$F18*12+'Assumptions'!$D$39*$D18*6.5)*'Assumptions'!$D$40+('Assumptions'!$B$41*$D16*$F18^2*12+'Assumptions'!$C$41*$D17*$F18*12+'Assumptions'!$D$41*$D18*6.5)*'Assumptions'!$D$42+('Assumptions'!$B$43*$D16*$F18^2*12+'Assumptions'!$C$43*$D17*$F18*12+'Assumptions'!$D$43*$D18*6.5)*'Assumptions'!$D$44</x:f>
@@ -12195,7 +12195,7 @@
       </x:c>
       <x:c r="R18" s="62" t="n">
         <x:f>N18+O18+P18+Q18</x:f>
-        <x:v>720407.0761</x:v>
+        <x:v>719471.6521</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -12229,7 +12229,7 @@
       </x:c>
       <x:c r="H19" s="62" t="n">
         <x:f>$C19*(('Assumptions'!$B$8*(6*$E19^0+6*$E19^1)+'Assumptions'!$B$9*(10*$E19^0+2*$E19^1))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F19^0+6*$F19^1)+'Assumptions'!$B$12*(10*$F19^0+2*$F19^1))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>8508</x:v>
+        <x:v>6383.999999999999</x:v>
       </x:c>
       <x:c r="I19" s="62" t="n">
         <x:f>('Assumptions'!$B$20*$D19*6.5)*'Assumptions'!$B$22</x:f>
@@ -12253,7 +12253,7 @@
       </x:c>
       <x:c r="N19" s="62" t="n">
         <x:f>SUM(H19:M19)</x:f>
-        <x:v>63608</x:v>
+        <x:v>61484</x:v>
       </x:c>
       <x:c r="O19" s="62" t="n">
         <x:f>'Assumptions'!$B$37*$D19*6.5*'Assumptions'!$B$38+'Assumptions'!$B$39*$D19*6.5*'Assumptions'!$B$40+'Assumptions'!$B$41*$D19*6.5*'Assumptions'!$B$42+'Assumptions'!$B$43*$D19*6.5*'Assumptions'!$B$44</x:f>
@@ -12269,7 +12269,7 @@
       </x:c>
       <x:c r="R19" s="62" t="n">
         <x:f>N19+O19+P19+Q19</x:f>
-        <x:v>122363</x:v>
+        <x:v>120239</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -12303,7 +12303,7 @@
       </x:c>
       <x:c r="H20" s="62" t="n">
         <x:f>$C20*(('Assumptions'!$B$8*(6*$E20^1+6*$E20^2)+'Assumptions'!$B$9*(10*$E20^1+2*$E20^2))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F20^1+6*$F20^2)+'Assumptions'!$B$12*(10*$F20^1+2*$F20^2))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>6152.4000000000015</x:v>
+        <x:v>4240.8</x:v>
       </x:c>
       <x:c r="I20" s="62" t="n">
         <x:f>('Assumptions'!$B$20*$D19*$E20*12+'Assumptions'!$C$20*$D20*6.5)*'Assumptions'!$C$22</x:f>
@@ -12327,7 +12327,7 @@
       </x:c>
       <x:c r="N20" s="62" t="n">
         <x:f>SUM(H20:M20)</x:f>
-        <x:v>190658.73333333334</x:v>
+        <x:v>188747.13333333333</x:v>
       </x:c>
       <x:c r="O20" s="62" t="n">
         <x:f>('Assumptions'!$B$37*$D19*$F20*12+'Assumptions'!$C$37*$D20*6.5)*'Assumptions'!$C$38+('Assumptions'!$B$39*$D19*$F20*12+'Assumptions'!$C$39*$D20*6.5)*'Assumptions'!$C$40+('Assumptions'!$B$41*$D19*$F20*12+'Assumptions'!$C$41*$D20*6.5)*'Assumptions'!$C$42+('Assumptions'!$B$43*$D19*$F20*12+'Assumptions'!$C$43*$D20*6.5)*'Assumptions'!$C$44</x:f>
@@ -12343,7 +12343,7 @@
       </x:c>
       <x:c r="R20" s="62" t="n">
         <x:f>N20+O20+P20+Q20</x:f>
-        <x:v>366674.73333333334</x:v>
+        <x:v>364763.1333333333</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -12377,7 +12377,7 @@
       </x:c>
       <x:c r="H21" s="62" t="n">
         <x:f>$C21*(('Assumptions'!$B$8*(6*$E21^2+6*$E21^3)+'Assumptions'!$B$9*(10*$E21^2+2*$E21^3))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F21^2+6*$F21^3)+'Assumptions'!$B$12*(10*$F21^2+2*$F21^3))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>4634.280000000001</x:v>
+        <x:v>2913.84</x:v>
       </x:c>
       <x:c r="I21" s="62" t="n">
         <x:f>('Assumptions'!$B$20*$D19*$E21^2*12+'Assumptions'!$C$20*$D20*$E21*12+'Assumptions'!$D$20*$D21*6.5)*'Assumptions'!$D$22</x:f>
@@ -12401,7 +12401,7 @@
       </x:c>
       <x:c r="N21" s="62" t="n">
         <x:f>SUM(H21:M21)</x:f>
-        <x:v>514146.28</x:v>
+        <x:v>512425.83999999997</x:v>
       </x:c>
       <x:c r="O21" s="62" t="n">
         <x:f>('Assumptions'!$B$37*$D19*$F21^2*12+'Assumptions'!$C$37*$D20*$F21*12+'Assumptions'!$D$37*$D21*6.5)*'Assumptions'!$D$38+('Assumptions'!$B$39*$D19*$F21^2*12+'Assumptions'!$C$39*$D20*$F21*12+'Assumptions'!$D$39*$D21*6.5)*'Assumptions'!$D$40+('Assumptions'!$B$41*$D19*$F21^2*12+'Assumptions'!$C$41*$D20*$F21*12+'Assumptions'!$D$41*$D21*6.5)*'Assumptions'!$D$42+('Assumptions'!$B$43*$D19*$F21^2*12+'Assumptions'!$C$43*$D20*$F21*12+'Assumptions'!$D$43*$D21*6.5)*'Assumptions'!$D$44</x:f>
@@ -12417,7 +12417,7 @@
       </x:c>
       <x:c r="R21" s="62" t="n">
         <x:f>N21+O21+P21+Q21</x:f>
-        <x:v>944852.922</x:v>
+        <x:v>943132.482</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -12451,7 +12451,7 @@
       </x:c>
       <x:c r="H22" s="62" t="n">
         <x:f>$C22*(('Assumptions'!$B$8*(6*$E22^0+6*$E22^1)+'Assumptions'!$B$9*(10*$E22^0+2*$E22^1))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F22^0+6*$F22^1)+'Assumptions'!$B$12*(10*$F22^0+2*$F22^1))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>10018.11</x:v>
+        <x:v>7563.090000000001</x:v>
       </x:c>
       <x:c r="I22" s="62" t="n">
         <x:f>('Assumptions'!$B$20*$D22*6.5)*'Assumptions'!$B$22</x:f>
@@ -12475,7 +12475,7 @@
       </x:c>
       <x:c r="N22" s="62" t="n">
         <x:f>SUM(H22:M22)</x:f>
-        <x:v>81648.11</x:v>
+        <x:v>79193.09</x:v>
       </x:c>
       <x:c r="O22" s="62" t="n">
         <x:f>'Assumptions'!$B$37*$D22*6.5*'Assumptions'!$B$38+'Assumptions'!$B$39*$D22*6.5*'Assumptions'!$B$40+'Assumptions'!$B$41*$D22*6.5*'Assumptions'!$B$42+'Assumptions'!$B$43*$D22*6.5*'Assumptions'!$B$44</x:f>
@@ -12491,7 +12491,7 @@
       </x:c>
       <x:c r="R22" s="62" t="n">
         <x:f>N22+O22+P22+Q22</x:f>
-        <x:v>158029.61000000002</x:v>
+        <x:v>155574.59</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -12525,7 +12525,7 @@
       </x:c>
       <x:c r="H23" s="62" t="n">
         <x:f>$C23*(('Assumptions'!$B$8*(6*$E23^1+6*$E23^2)+'Assumptions'!$B$9*(10*$E23^1+2*$E23^2))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F23^1+6*$F23^2)+'Assumptions'!$B$12*(10*$F23^1+2*$F23^2))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>7944.8808</x:v>
+        <x:v>5661.712199999999</x:v>
       </x:c>
       <x:c r="I23" s="62" t="n">
         <x:f>('Assumptions'!$B$20*$D22*$E23*12+'Assumptions'!$C$20*$D23*6.5)*'Assumptions'!$C$22</x:f>
@@ -12549,7 +12549,7 @@
       </x:c>
       <x:c r="N23" s="62" t="n">
         <x:f>SUM(H23:M23)</x:f>
-        <x:v>259929.31079999998</x:v>
+        <x:v>257646.1422</x:v>
       </x:c>
       <x:c r="O23" s="62" t="n">
         <x:f>('Assumptions'!$B$37*$D22*$F23*12+'Assumptions'!$C$37*$D23*6.5)*'Assumptions'!$C$38+('Assumptions'!$B$39*$D22*$F23*12+'Assumptions'!$C$39*$D23*6.5)*'Assumptions'!$C$40+('Assumptions'!$B$41*$D22*$F23*12+'Assumptions'!$C$41*$D23*6.5)*'Assumptions'!$C$42+('Assumptions'!$B$43*$D22*$F23*12+'Assumptions'!$C$43*$D23*6.5)*'Assumptions'!$C$44</x:f>
@@ -12565,7 +12565,7 @@
       </x:c>
       <x:c r="R23" s="62" t="n">
         <x:f>N23+O23+P23+Q23</x:f>
-        <x:v>497099.47079999995</x:v>
+        <x:v>494816.3022</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -12599,7 +12599,7 @@
       </x:c>
       <x:c r="H24" s="62" t="n">
         <x:f>$C24*(('Assumptions'!$B$8*(6*$E24^2+6*$E24^3)+'Assumptions'!$B$9*(10*$E24^2+2*$E24^3))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F24^2+6*$F24^3)+'Assumptions'!$B$12*(10*$F24^2+2*$F24^3))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>6428.366094</x:v>
+        <x:v>4305.0192959999995</x:v>
       </x:c>
       <x:c r="I24" s="62" t="n">
         <x:f>('Assumptions'!$B$20*$D22*$E24^2*12+'Assumptions'!$C$20*$D23*$E24*12+'Assumptions'!$D$20*$D24*6.5)*'Assumptions'!$D$22</x:f>
@@ -12623,7 +12623,7 @@
       </x:c>
       <x:c r="N24" s="62" t="n">
         <x:f>SUM(H24:M24)</x:f>
-        <x:v>733897.078094</x:v>
+        <x:v>731773.7312960001</x:v>
       </x:c>
       <x:c r="O24" s="62" t="n">
         <x:f>('Assumptions'!$B$37*$D22*$F24^2*12+'Assumptions'!$C$37*$D23*$F24*12+'Assumptions'!$D$37*$D24*6.5)*'Assumptions'!$D$38+('Assumptions'!$B$39*$D22*$F24^2*12+'Assumptions'!$C$39*$D23*$F24*12+'Assumptions'!$D$39*$D24*6.5)*'Assumptions'!$D$40+('Assumptions'!$B$41*$D22*$F24^2*12+'Assumptions'!$C$41*$D23*$F24*12+'Assumptions'!$D$41*$D24*6.5)*'Assumptions'!$D$42+('Assumptions'!$B$43*$D22*$F24^2*12+'Assumptions'!$C$43*$D23*$F24*12+'Assumptions'!$D$43*$D24*6.5)*'Assumptions'!$D$44</x:f>
@@ -12639,7 +12639,7 @@
       </x:c>
       <x:c r="R24" s="62" t="n">
         <x:f>N24+O24+P24+Q24</x:f>
-        <x:v>1335461.514858</x:v>
+        <x:v>1333338.16806</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
@@ -12673,7 +12673,7 @@
       </x:c>
       <x:c r="H25" s="91" t="n">
         <x:f>$C25*(('Assumptions'!$B$8*(6*$E25^0+6*$E25^1)+'Assumptions'!$B$9*(10*$E25^0+2*$E25^1))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F25^0+6*$F25^1)+'Assumptions'!$B$12*(10*$F25^0+2*$F25^1))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>8508</x:v>
+        <x:v>6383.999999999999</x:v>
       </x:c>
       <x:c r="I25" s="91" t="n">
         <x:f>('Assumptions'!$B$20*$D25*6.5)*'Assumptions'!$B$22</x:f>
@@ -12697,7 +12697,7 @@
       </x:c>
       <x:c r="N25" s="91" t="n">
         <x:f>SUM(H25:M25)</x:f>
-        <x:v>74628</x:v>
+        <x:v>72504</x:v>
       </x:c>
       <x:c r="O25" s="91" t="n">
         <x:f>'Assumptions'!$B$37*$D25*6.5*'Assumptions'!$B$38+'Assumptions'!$B$39*$D25*6.5*'Assumptions'!$B$40+'Assumptions'!$B$41*$D25*6.5*'Assumptions'!$B$42+'Assumptions'!$B$43*$D25*6.5*'Assumptions'!$B$44</x:f>
@@ -12713,7 +12713,7 @@
       </x:c>
       <x:c r="R25" s="91" t="n">
         <x:f>N25+O25+P25+Q25</x:f>
-        <x:v>145134</x:v>
+        <x:v>143010</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
@@ -12747,7 +12747,7 @@
       </x:c>
       <x:c r="H26" s="91" t="n">
         <x:f>$C26*(('Assumptions'!$B$8*(6*$E26^1+6*$E26^2)+'Assumptions'!$B$9*(10*$E26^1+2*$E26^2))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F26^1+6*$F26^2)+'Assumptions'!$B$12*(10*$F26^1+2*$F26^2))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>6152.4000000000015</x:v>
+        <x:v>4240.8</x:v>
       </x:c>
       <x:c r="I26" s="91" t="n">
         <x:f>('Assumptions'!$B$20*$D25*$E26*12+'Assumptions'!$C$20*$D26*6.5)*'Assumptions'!$C$22</x:f>
@@ -12771,7 +12771,7 @@
       </x:c>
       <x:c r="N26" s="91" t="n">
         <x:f>SUM(H26:M26)</x:f>
-        <x:v>233620.91666666666</x:v>
+        <x:v>231709.31666666668</x:v>
       </x:c>
       <x:c r="O26" s="91" t="n">
         <x:f>('Assumptions'!$B$37*$D25*$F26*12+'Assumptions'!$C$37*$D26*6.5)*'Assumptions'!$C$38+('Assumptions'!$B$39*$D25*$F26*12+'Assumptions'!$C$39*$D26*6.5)*'Assumptions'!$C$40+('Assumptions'!$B$41*$D25*$F26*12+'Assumptions'!$C$41*$D26*6.5)*'Assumptions'!$C$42+('Assumptions'!$B$43*$D25*$F26*12+'Assumptions'!$C$43*$D26*6.5)*'Assumptions'!$C$44</x:f>
@@ -12787,7 +12787,7 @@
       </x:c>
       <x:c r="R26" s="91" t="n">
         <x:f>N26+O26+P26+Q26</x:f>
-        <x:v>450255.11666666664</x:v>
+        <x:v>448343.51666666666</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
@@ -12821,7 +12821,7 @@
       </x:c>
       <x:c r="H27" s="95" t="n">
         <x:f>$C27*(('Assumptions'!$B$8*(6*$E27^2+6*$E27^3)+'Assumptions'!$B$9*(10*$E27^2+2*$E27^3))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F27^2+6*$F27^3)+'Assumptions'!$B$12*(10*$F27^2+2*$F27^3))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
-        <x:v>4634.280000000001</x:v>
+        <x:v>2913.84</x:v>
       </x:c>
       <x:c r="I27" s="95" t="n">
         <x:f>('Assumptions'!$B$20*$D25*$E27^2*12+'Assumptions'!$C$20*$D26*$E27*12+'Assumptions'!$D$20*$D27*6.5)*'Assumptions'!$D$22</x:f>
@@ -12845,7 +12845,7 @@
       </x:c>
       <x:c r="N27" s="95" t="n">
         <x:f>SUM(H27:M27)</x:f>
-        <x:v>652826.6799999999</x:v>
+        <x:v>651106.2399999999</x:v>
       </x:c>
       <x:c r="O27" s="95" t="n">
         <x:f>('Assumptions'!$B$37*$D25*$F27^2*12+'Assumptions'!$C$37*$D26*$F27*12+'Assumptions'!$D$37*$D27*6.5)*'Assumptions'!$D$38+('Assumptions'!$B$39*$D25*$F27^2*12+'Assumptions'!$C$39*$D26*$F27*12+'Assumptions'!$D$39*$D27*6.5)*'Assumptions'!$D$40+('Assumptions'!$B$41*$D25*$F27^2*12+'Assumptions'!$C$41*$D26*$F27*12+'Assumptions'!$D$41*$D27*6.5)*'Assumptions'!$D$42+('Assumptions'!$B$43*$D25*$F27^2*12+'Assumptions'!$C$43*$D26*$F27*12+'Assumptions'!$D$43*$D27*6.5)*'Assumptions'!$D$44</x:f>
@@ -12861,7 +12861,7 @@
       </x:c>
       <x:c r="R27" s="95" t="n">
         <x:f>N27+O27+P27+Q27</x:f>
-        <x:v>1199682.4014</x:v>
+        <x:v>1197961.9614</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12982,10 +12982,10 @@
       </x:c>
       <x:c r="B6" s="75" t="n">
         <x:f>'Beta Plan'!H10</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C6" s="75" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D6" s="75" t="n">
         <x:f>B6-C6</x:f>
@@ -13005,10 +13005,10 @@
       </x:c>
       <x:c r="B7" s="76" t="n">
         <x:f>'Beta Plan'!L12</x:f>
-        <x:v>9300</x:v>
+        <x:v>7140</x:v>
       </x:c>
       <x:c r="C7" s="76" t="n">
-        <x:v>9300</x:v>
+        <x:v>7140</x:v>
       </x:c>
       <x:c r="D7" s="76" t="n">
         <x:f>B7-C7</x:f>
@@ -13028,10 +13028,10 @@
       </x:c>
       <x:c r="B8" s="76" t="n">
         <x:f>'Beta Plan'!M12</x:f>
-        <x:v>2790</x:v>
+        <x:v>2430</x:v>
       </x:c>
       <x:c r="C8" s="76" t="n">
-        <x:v>2790</x:v>
+        <x:v>2430</x:v>
       </x:c>
       <x:c r="D8" s="76" t="n">
         <x:f>B8-C8</x:f>
@@ -13051,11 +13051,11 @@
       </x:c>
       <x:c r="B9" s="76" t="n">
         <x:f>'Executive Summary'!B21</x:f>
-        <x:v>122363</x:v>
+        <x:v>120239</x:v>
       </x:c>
       <x:c r="C9" s="76" t="n">
         <x:f>'Executive Summary'!B11+'Executive Summary'!B19</x:f>
-        <x:v>122363</x:v>
+        <x:v>120239</x:v>
       </x:c>
       <x:c r="D9" s="76" t="n">
         <x:f>B9-C9</x:f>
@@ -13075,11 +13075,11 @@
       </x:c>
       <x:c r="B10" s="76" t="n">
         <x:f>'Executive Summary'!C21</x:f>
-        <x:v>366674.73333333334</x:v>
+        <x:v>364763.1333333333</x:v>
       </x:c>
       <x:c r="C10" s="76" t="n">
         <x:f>'Executive Summary'!C11+'Executive Summary'!C19</x:f>
-        <x:v>366674.73333333334</x:v>
+        <x:v>364763.1333333333</x:v>
       </x:c>
       <x:c r="D10" s="76" t="n">
         <x:f>B10-C10</x:f>
@@ -13099,11 +13099,11 @@
       </x:c>
       <x:c r="B11" s="76" t="n">
         <x:f>'Executive Summary'!D21</x:f>
-        <x:v>944852.922</x:v>
+        <x:v>943132.482</x:v>
       </x:c>
       <x:c r="C11" s="76" t="n">
         <x:f>'Executive Summary'!D11+'Executive Summary'!D19</x:f>
-        <x:v>944852.922</x:v>
+        <x:v>943132.482</x:v>
       </x:c>
       <x:c r="D11" s="76" t="n">
         <x:f>B11-C11</x:f>
@@ -13123,11 +13123,11 @@
       </x:c>
       <x:c r="B12" s="76" t="n">
         <x:f>'Cohort Bridge'!E6</x:f>
-        <x:v>24.5</x:v>
+        <x:v>21.8</x:v>
       </x:c>
       <x:c r="C12" s="76" t="n">
         <x:f>'Cohort Bridge'!C6*'Cohort Bridge'!B6+'Cohort Bridge'!D6</x:f>
-        <x:v>24.5</x:v>
+        <x:v>21.8</x:v>
       </x:c>
       <x:c r="D12" s="76" t="n">
         <x:f>B12-C12</x:f>
@@ -13147,11 +13147,11 @@
       </x:c>
       <x:c r="B13" s="76" t="n">
         <x:f>'Cohort Bridge'!I6</x:f>
-        <x:v>106.845</x:v>
+        <x:v>104.658</x:v>
       </x:c>
       <x:c r="C13" s="76" t="n">
         <x:f>'Cohort Bridge'!C6*'Cohort Bridge'!B6^3+'Cohort Bridge'!D6*'Cohort Bridge'!B6^2+'Cohort Bridge'!F6*'Cohort Bridge'!B6+'Cohort Bridge'!H6</x:f>
-        <x:v>106.845</x:v>
+        <x:v>104.658</x:v>
       </x:c>
       <x:c r="D13" s="76" t="n">
         <x:f>B13-C13</x:f>
@@ -13171,11 +13171,11 @@
       </x:c>
       <x:c r="B14" s="76" t="n">
         <x:f>'Executive Summary'!D23</x:f>
-        <x:v>1203584.4120000002</x:v>
+        <x:v>1202009.772</x:v>
       </x:c>
       <x:c r="C14" s="76" t="n">
         <x:f>'Executive Summary'!D22*12</x:f>
-        <x:v>1203584.4120000002</x:v>
+        <x:v>1202009.772</x:v>
       </x:c>
       <x:c r="D14" s="76" t="n">
         <x:f>B14-C14</x:f>
@@ -13195,14 +13195,14 @@
       </x:c>
       <x:c r="B15" s="76" t="n">
         <x:f>MIN('Scenarios'!D6-'Scenarios'!D5,'Scenarios'!D7-'Scenarios'!D6,'Scenarios'!D8-'Scenarios'!D7)</x:f>
-        <x:v>135779.1134579999</x:v>
+        <x:v>135376.20666000014</x:v>
       </x:c>
       <x:c r="C15" s="76" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D15" s="76" t="n">
         <x:f>B15-C15</x:f>
-        <x:v>135779.1134579999</x:v>
+        <x:v>135376.20666000014</x:v>
       </x:c>
       <x:c r="E15" s="29" t="str">
         <x:f>IF(D15&gt;0,"PASS","FAIL")</x:f>
@@ -13436,7 +13436,7 @@
         <x:v>Beta timeline and targets</x:v>
       </x:c>
       <x:c r="B5" s="36" t="str">
-        <x:v>6 months; 12 then 30 individuals; 2 then 5 teams</x:v>
+        <x:v>6 months; 12 then 30 individuals; 2 founding Team Pro workspaces</x:v>
       </x:c>
       <x:c r="C5" s="81" t="str">
         <x:v>2026-08-28</x:v>
@@ -13494,13 +13494,13 @@
         <x:v>Beta team price</x:v>
       </x:c>
       <x:c r="B7" s="36" t="str">
-        <x:v>$240/seat/year; 3-seat minimum</x:v>
+        <x:v>Founding Team Pro Beta: $240/seat/year; 3-seat minimum; 2 workspaces</x:v>
       </x:c>
       <x:c r="C7" s="81" t="str">
-        <x:v>2026-08-28</x:v>
+        <x:v>2026-08-29</x:v>
       </x:c>
       <x:c r="D7" s="36" t="str">
-        <x:v>Planning assumption</x:v>
+        <x:v>Management decision</x:v>
       </x:c>
       <x:c r="E7" s="36" t="str">
         <x:v>MIMAR underwriting</x:v>
@@ -13515,7 +13515,7 @@
         <x:v>$720 minimum annual workspace booking</x:v>
       </x:c>
       <x:c r="I7" s="36" t="str">
-        <x:v>Pending management confirmation</x:v>
+        <x:v>Confirm signed Beta commitments</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="35" customHeight="1">

</xml_diff>

<commit_message>
Clarify MIMAR product suite architecture
</commit_message>
<xml_diff>
--- a/assets/MIMAR_Investor_Revenue_Model_2026-08-28.xlsx
+++ b/assets/MIMAR_Investor_Revenue_Model_2026-08-28.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rb826add9d2fe4f6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beta Plan" sheetId="2" r:id="R680a4d4f87db4a98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Redc221fc56254a71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Bridge" sheetId="4" r:id="R4a641a5adfed4dd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Monthly" sheetId="5" r:id="Re9fe6b8429104394"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engage Monthly" sheetId="6" r:id="Rcc8ae7cbc70a434e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="7" r:id="R0defdef88ddb4610"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R6ecd0d23595b4839"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Rd041fb77bd7d491e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GTM Plan" sheetId="10" r:id="R44b3c4a3791e4845"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R036bf00595594bfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beta Plan" sheetId="2" r:id="R4dbb017d1bed464e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Re0fd07692c77422e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Bridge" sheetId="4" r:id="Rc714ecd52be34a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Monthly" sheetId="5" r:id="Rb585e47fdec6444c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engage Monthly" sheetId="6" r:id="Ra2d4e18647b94517"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="7" r:id="R4c8e31abc310448b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R7bb756c73fd741bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Rc5f93fae2f954816"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GTM Plan" sheetId="10" r:id="Rb257c80f95b74df6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -883,7 +883,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re373b63192f14e5f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R084be8463b984317"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -918,7 +918,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re900035a3ff24cdf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf6098a4bd9184462"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1164,7 +1164,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>MIMAR Portfolio — Investor Revenue Model</x:v>
+        <x:v>MIMAR Product Suite — Investor Revenue Model</x:v>
       </x:c>
       <x:c r="B1" s="19" t="str">
         <x:v>MIMAR Portfolio — Investor Revenue Model</x:v>
@@ -1193,7 +1193,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>Paid Beta Nov 2026–Apr 2027 | 30 Individual Pro passes + 2 founding Team Pro workspaces | Commercial forecast May 2027–Apr 2030 | Explicit cohorts and segmented retention</x:v>
+        <x:v>Paid Beta Nov 2026–Apr 2027 | Commercial forecast May 2027–Apr 2030 | Core + Engage: one platform, separate commercial models</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>Paid Beta Nov 2026–Apr 2027 | Commercial forecast May 2027–Apr 2030 | Explicit cohorts and segmented retention</x:v>
@@ -1255,7 +1255,7 @@
         <x:v>Engage</x:v>
       </x:c>
       <x:c r="I4" s="22" t="str">
-        <x:v>Portfolio</x:v>
+        <x:v>Total MIMAR</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1381,7 +1381,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>CORE — API wallet</x:v>
+        <x:v>CORE — Metered usage</x:v>
       </x:c>
       <x:c r="B9" s="62" t="n">
         <x:f>SUM('Core Monthly'!P5:P16)</x:f>
@@ -1623,7 +1623,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="65" t="str">
-        <x:v>PORTFOLIO REVENUE</x:v>
+        <x:v>TOTAL MIMAR REVENUE</x:v>
       </x:c>
       <x:c r="B21" s="66" t="n">
         <x:f>B11+B19</x:f>
@@ -1956,7 +1956,7 @@
     <x:mergeCell ref="F26:I28"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1c3fce70e474fea"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c4b02dc3896495e"/>
 </x:worksheet>
 </file>
 
@@ -2224,7 +2224,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>API active wallets</x:v>
+        <x:v>Core metered usage accounts</x:v>
       </x:c>
       <x:c r="B13" s="112" t="n">
         <x:f>'Assumptions'!B29</x:f>
@@ -2481,7 +2481,7 @@
         <x:v>90000</x:v>
       </x:c>
       <x:c r="D27" s="130" t="str">
-        <x:v>Compound portfolio distribution</x:v>
+        <x:v>Compound product-suite distribution</x:v>
       </x:c>
       <x:c r="E27" s="130" t="str">
         <x:v>Category + partner proof</x:v>
@@ -2490,7 +2490,7 @@
         <x:v>Enterprise and expansion</x:v>
       </x:c>
       <x:c r="G27" s="130" t="str">
-        <x:v>Portfolio-level efficiency</x:v>
+        <x:v>Product-suite efficiency</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
@@ -2614,7 +2614,7 @@
     <x:mergeCell ref="A2:L2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R853061ae7ba54e7a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raff36639ceb24aee"/>
 </x:worksheet>
 </file>
 
@@ -4499,7 +4499,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R530e210f6ba44b5e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabf7071656294ef5"/>
 </x:worksheet>
 </file>
 
@@ -11973,7 +11973,7 @@
         <x:v>Engage onboarding</x:v>
       </x:c>
       <x:c r="R15" s="22" t="str">
-        <x:v>PORTFOLIO</x:v>
+        <x:v>TOTAL MIMAR</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -13047,7 +13047,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>Portfolio equals Core + Engage — Y1</x:v>
+        <x:v>Total MIMAR revenue equals Core + Engage — Y1</x:v>
       </x:c>
       <x:c r="B9" s="76" t="n">
         <x:f>'Executive Summary'!B21</x:f>
@@ -13071,7 +13071,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>Portfolio equals Core + Engage — Y2</x:v>
+        <x:v>Total MIMAR revenue equals Core + Engage — Y2</x:v>
       </x:c>
       <x:c r="B10" s="76" t="n">
         <x:f>'Executive Summary'!C21</x:f>
@@ -13095,7 +13095,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>Portfolio equals Core + Engage — Y3</x:v>
+        <x:v>Total MIMAR revenue equals Core + Engage — Y3</x:v>
       </x:c>
       <x:c r="B11" s="76" t="n">
         <x:f>'Executive Summary'!D21</x:f>

</xml_diff>

<commit_message>
Simplify investor revenue workbook
</commit_message>
<xml_diff>
--- a/assets/MIMAR_Investor_Revenue_Model_2026-08-28.xlsx
+++ b/assets/MIMAR_Investor_Revenue_Model_2026-08-28.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R036bf00595594bfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beta Plan" sheetId="2" r:id="R4dbb017d1bed464e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Re0fd07692c77422e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Bridge" sheetId="4" r:id="Rc714ecd52be34a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Monthly" sheetId="5" r:id="Rb585e47fdec6444c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engage Monthly" sheetId="6" r:id="Ra2d4e18647b94517"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="7" r:id="R4c8e31abc310448b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R7bb756c73fd741bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Rc5f93fae2f954816"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GTM Plan" sheetId="10" r:id="Rb257c80f95b74df6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R5cdd590212534941"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beta Plan" sheetId="2" r:id="Rdbf76da2ac2d467a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Rf2032615004d45d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Bridge" sheetId="4" r:id="Re5f1cb76283546d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Monthly" sheetId="5" r:id="R325712292b8342fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engage Monthly" sheetId="6" r:id="R3faca3d41f214cd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="7" r:id="R495a339825ac490d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R1de9b3f933724736"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Rceedbf1003e8424f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GTM Plan" sheetId="10" r:id="R4cf2c1c4e6244c85"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -108,7 +108,7 @@
     <x:numFmt numFmtId="207" formatCode="0"/>
     <x:numFmt numFmtId="208" formatCode="#,##0;[Red](#,##0);-"/>
   </x:numFmts>
-  <x:fonts count="23">
+  <x:fonts count="26">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -236,8 +236,25 @@
       <x:color rgb="FF166534"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="1"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="1"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="1"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -294,8 +311,13 @@
         <x:fgColor rgb="FF0B1016"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="4">
+  <x:borders count="26">
     <x:border/>
     <x:border>
       <x:bottom style="medium">
@@ -312,11 +334,118 @@
         <x:color rgb="FF4CD6E5"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="none"/>
+      <x:top style="none"/>
+    </x:border>
+    <x:border>
+      <x:top style="none"/>
+    </x:border>
+    <x:border>
+      <x:right style="none"/>
+      <x:top style="none"/>
+    </x:border>
+    <x:border>
+      <x:left style="none"/>
+    </x:border>
+    <x:border>
+      <x:right style="none"/>
+    </x:border>
+    <x:border>
+      <x:left style="none"/>
+      <x:bottom style="none"/>
+    </x:border>
+    <x:border>
+      <x:bottom style="none"/>
+    </x:border>
+    <x:border>
+      <x:right style="none"/>
+      <x:bottom style="none"/>
+    </x:border>
+    <x:border>
+      <x:left style="none"/>
+      <x:top style="none"/>
+      <x:bottom style="none"/>
+    </x:border>
+    <x:border>
+      <x:top style="none"/>
+      <x:bottom style="none"/>
+    </x:border>
+    <x:border>
+      <x:right style="none"/>
+      <x:top style="none"/>
+      <x:bottom style="none"/>
+    </x:border>
+    <x:border>
+      <x:left style="none"/>
+      <x:bottom style="medium">
+        <x:color rgb="FF4CD6E5"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="none"/>
+      <x:bottom style="medium">
+        <x:color rgb="FF4CD6E5"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="none"/>
+      <x:top style="medium">
+        <x:color rgb="FF4CD6E5"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="none"/>
+      <x:top style="medium">
+        <x:color rgb="FF4CD6E5"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:top style="none"/>
+    </x:border>
+    <x:border>
+      <x:left style="none"/>
+      <x:right style="none"/>
+    </x:border>
+    <x:border>
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:bottom style="medium">
+        <x:color rgb="FF4CD6E5"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="none"/>
+      <x:right style="none"/>
+      <x:bottom style="none"/>
+    </x:border>
+    <x:border>
+      <x:left style="none"/>
+      <x:top style="none"/>
+      <x:bottom style="medium">
+        <x:color rgb="FF4CD6E5"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="none"/>
+      <x:bottom style="medium">
+        <x:color rgb="FF4CD6E5"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="none"/>
+      <x:top style="none"/>
+      <x:bottom style="medium">
+        <x:color rgb="FF4CD6E5"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="133">
+  <x:cellXfs count="244">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -552,6 +681,257 @@
     <x:xf numFmtId="202" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="10" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="24" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="23" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="23" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="24" fillId="12" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="24" fillId="12" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="12" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="12" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="19" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="19" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="19" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="19" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="19" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="19" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="23" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="23" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="23" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="23" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="201" fontId="23" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="202" fontId="23" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="23" fillId="12" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="23" fillId="12" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="12" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="12" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -883,7 +1263,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R084be8463b984317"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6d158b0de0b44fd3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -918,7 +1298,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf6098a4bd9184462"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R59b707c879644f5e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1164,7 +1544,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>MIMAR Product Suite — Investor Revenue Model</x:v>
+        <x:v>MIMAR Investor Snapshot</x:v>
       </x:c>
       <x:c r="B1" s="19" t="str">
         <x:v>MIMAR Portfolio — Investor Revenue Model</x:v>
@@ -1193,7 +1573,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>Paid Beta Nov 2026–Apr 2027 | Commercial forecast May 2027–Apr 2030 | Core + Engage: one platform, separate commercial models</x:v>
+        <x:v>Paid Beta, three-year outlook, and the assumptions behind the MIMAR product suite</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>Paid Beta Nov 2026–Apr 2027 | Commercial forecast May 2027–Apr 2030 | Explicit cohorts and segmented retention</x:v>
@@ -1258,170 +1638,170 @@
         <x:v>Total MIMAR</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="29" t="str">
+    <x:row r="5" ht="2" customHeight="1">
+      <x:c r="A5" s="137" t="str">
         <x:v>CORE — Beta cohort carry</x:v>
       </x:c>
-      <x:c r="B5" s="62" t="n">
+      <x:c r="B5" s="138" t="n">
         <x:f>SUM('Core Monthly'!F5:F16)+SUM('Core Monthly'!J5:J16)</x:f>
         <x:v>6384</x:v>
       </x:c>
-      <x:c r="C5" s="62" t="n">
+      <x:c r="C5" s="138" t="n">
         <x:f>SUM('Core Monthly'!F17:F28)+SUM('Core Monthly'!J17:J28)</x:f>
         <x:v>4240.800000000001</x:v>
       </x:c>
-      <x:c r="D5" s="62" t="n">
+      <x:c r="D5" s="138" t="n">
         <x:f>SUM('Core Monthly'!F29:F40)+SUM('Core Monthly'!J29:J40)</x:f>
         <x:v>2913.8399999999992</x:v>
       </x:c>
-      <x:c r="E5" s="29"/>
-      <x:c r="F5" s="29" t="str">
+      <x:c r="E5" s="139"/>
+      <x:c r="F5" s="139" t="str">
         <x:v>Y1</x:v>
       </x:c>
-      <x:c r="G5" s="62" t="n">
+      <x:c r="G5" s="138" t="n">
         <x:f>B11</x:f>
         <x:v>61484</x:v>
       </x:c>
-      <x:c r="H5" s="62" t="n">
+      <x:c r="H5" s="138" t="n">
         <x:f>B19</x:f>
         <x:v>58755</x:v>
       </x:c>
-      <x:c r="I5" s="62" t="n">
+      <x:c r="I5" s="140" t="n">
         <x:f>B21</x:f>
         <x:v>120239</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="29" t="str">
+    <x:row r="6" ht="2" customHeight="1">
+      <x:c r="A6" s="141" t="str">
         <x:v>CORE — Commercial individuals</x:v>
       </x:c>
-      <x:c r="B6" s="62" t="n">
+      <x:c r="B6" s="142" t="n">
         <x:f>SUM('Core Monthly'!H5:H16)</x:f>
         <x:v>10400</x:v>
       </x:c>
-      <x:c r="C6" s="62" t="n">
+      <x:c r="C6" s="142" t="n">
         <x:f>SUM('Core Monthly'!H17:H28)</x:f>
         <x:v>42210</x:v>
       </x:c>
-      <x:c r="D6" s="62" t="n">
+      <x:c r="D6" s="142" t="n">
         <x:f>SUM('Core Monthly'!H29:H40)</x:f>
         <x:v>109640</x:v>
       </x:c>
-      <x:c r="E6" s="29"/>
-      <x:c r="F6" s="29" t="str">
+      <x:c r="E6" s="143"/>
+      <x:c r="F6" s="143" t="str">
         <x:v>Y2</x:v>
       </x:c>
-      <x:c r="G6" s="62" t="n">
+      <x:c r="G6" s="142" t="n">
         <x:f>C11</x:f>
         <x:v>188747.13333333333</x:v>
       </x:c>
-      <x:c r="H6" s="62" t="n">
+      <x:c r="H6" s="142" t="n">
         <x:f>C19</x:f>
         <x:v>176016</x:v>
       </x:c>
-      <x:c r="I6" s="62" t="n">
+      <x:c r="I6" s="144" t="n">
         <x:f>C21</x:f>
         <x:v>364763.1333333333</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="29" t="str">
+    <x:row r="7" ht="2" customHeight="1">
+      <x:c r="A7" s="141" t="str">
         <x:v>CORE — Commercial team seats</x:v>
       </x:c>
-      <x:c r="B7" s="62" t="n">
+      <x:c r="B7" s="142" t="n">
         <x:f>SUM('Core Monthly'!L5:L16)</x:f>
         <x:v>20800</x:v>
       </x:c>
-      <x:c r="C7" s="62" t="n">
+      <x:c r="C7" s="142" t="n">
         <x:f>SUM('Core Monthly'!L17:L28)</x:f>
         <x:v>81378</x:v>
       </x:c>
-      <x:c r="D7" s="62" t="n">
+      <x:c r="D7" s="142" t="n">
         <x:f>SUM('Core Monthly'!L29:L40)</x:f>
         <x:v>218016</x:v>
       </x:c>
-      <x:c r="E7" s="29"/>
-      <x:c r="F7" s="29" t="str">
+      <x:c r="E7" s="143"/>
+      <x:c r="F7" s="143" t="str">
         <x:v>Y3</x:v>
       </x:c>
-      <x:c r="G7" s="62" t="n">
+      <x:c r="G7" s="142" t="n">
         <x:f>D11</x:f>
         <x:v>512425.83999999997</x:v>
       </x:c>
-      <x:c r="H7" s="62" t="n">
+      <x:c r="H7" s="142" t="n">
         <x:f>D19</x:f>
         <x:v>430706.642</x:v>
       </x:c>
-      <x:c r="I7" s="62" t="n">
+      <x:c r="I7" s="144" t="n">
         <x:f>D21</x:f>
         <x:v>943132.482</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
+    <x:row r="8" ht="2" customHeight="1">
+      <x:c r="A8" s="141" t="str">
         <x:v>CORE — Enterprise</x:v>
       </x:c>
-      <x:c r="B8" s="62" t="n">
+      <x:c r="B8" s="142" t="n">
         <x:f>SUM('Core Monthly'!N5:N16)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C8" s="62" t="n">
+      <x:c r="C8" s="142" t="n">
         <x:f>SUM('Core Monthly'!N17:N28)</x:f>
         <x:v>10833.333333333332</x:v>
       </x:c>
-      <x:c r="D8" s="62" t="n">
+      <x:c r="D8" s="142" t="n">
         <x:f>SUM('Core Monthly'!N29:N40)</x:f>
         <x:v>55550</x:v>
       </x:c>
-      <x:c r="E8" s="29"/>
-      <x:c r="F8" s="29"/>
-      <x:c r="G8" s="29"/>
-      <x:c r="H8" s="29"/>
-      <x:c r="I8" s="29"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
+      <x:c r="E8" s="143"/>
+      <x:c r="F8" s="143"/>
+      <x:c r="G8" s="143"/>
+      <x:c r="H8" s="143"/>
+      <x:c r="I8" s="145"/>
+    </x:row>
+    <x:row r="9" ht="2" customHeight="1">
+      <x:c r="A9" s="141" t="str">
         <x:v>CORE — Metered usage</x:v>
       </x:c>
-      <x:c r="B9" s="62" t="n">
+      <x:c r="B9" s="142" t="n">
         <x:f>SUM('Core Monthly'!P5:P16)</x:f>
         <x:v>3900</x:v>
       </x:c>
-      <x:c r="C9" s="62" t="n">
+      <x:c r="C9" s="142" t="n">
         <x:f>SUM('Core Monthly'!P17:P28)</x:f>
         <x:v>22185</x:v>
       </x:c>
-      <x:c r="D9" s="62" t="n">
+      <x:c r="D9" s="142" t="n">
         <x:f>SUM('Core Monthly'!P29:P40)</x:f>
         <x:v>79056</x:v>
       </x:c>
-      <x:c r="E9" s="29"/>
-      <x:c r="F9" s="29"/>
-      <x:c r="G9" s="29"/>
-      <x:c r="H9" s="29"/>
-      <x:c r="I9" s="29"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
+      <x:c r="E9" s="143"/>
+      <x:c r="F9" s="143"/>
+      <x:c r="G9" s="143"/>
+      <x:c r="H9" s="143"/>
+      <x:c r="I9" s="145"/>
+    </x:row>
+    <x:row r="10" ht="2" customHeight="1">
+      <x:c r="A10" s="146" t="str">
         <x:v>CORE — Onboarding</x:v>
       </x:c>
-      <x:c r="B10" s="62" t="n">
+      <x:c r="B10" s="147" t="n">
         <x:f>SUM('Core Monthly'!R5:R16)</x:f>
         <x:v>20000</x:v>
       </x:c>
-      <x:c r="C10" s="62" t="n">
+      <x:c r="C10" s="147" t="n">
         <x:f>SUM('Core Monthly'!R17:R28)</x:f>
         <x:v>27900</x:v>
       </x:c>
-      <x:c r="D10" s="62" t="n">
+      <x:c r="D10" s="147" t="n">
         <x:f>SUM('Core Monthly'!R29:R40)</x:f>
         <x:v>47250</x:v>
       </x:c>
-      <x:c r="E10" s="29"/>
-      <x:c r="F10" s="29"/>
-      <x:c r="G10" s="29"/>
-      <x:c r="H10" s="29"/>
-      <x:c r="I10" s="29"/>
+      <x:c r="E10" s="148"/>
+      <x:c r="F10" s="148"/>
+      <x:c r="G10" s="148"/>
+      <x:c r="H10" s="148"/>
+      <x:c r="I10" s="149"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="63" t="str">
@@ -1456,137 +1836,137 @@
       <x:c r="H12" s="29"/>
       <x:c r="I12" s="29"/>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
+    <x:row r="13" ht="2" customHeight="1">
+      <x:c r="A13" s="137" t="str">
         <x:v>ENGAGE — Starter</x:v>
       </x:c>
-      <x:c r="B13" s="62" t="n">
+      <x:c r="B13" s="138" t="n">
         <x:f>SUM('Engage Monthly'!E5:E16)</x:f>
         <x:v>9652.5</x:v>
       </x:c>
-      <x:c r="C13" s="62" t="n">
+      <x:c r="C13" s="138" t="n">
         <x:f>SUM('Engage Monthly'!E17:E28)</x:f>
         <x:v>28908</x:v>
       </x:c>
-      <x:c r="D13" s="62" t="n">
+      <x:c r="D13" s="138" t="n">
         <x:f>SUM('Engage Monthly'!E29:E40)</x:f>
         <x:v>55123.19999999999</x:v>
       </x:c>
-      <x:c r="E13" s="29"/>
-      <x:c r="F13" s="29"/>
-      <x:c r="G13" s="29"/>
-      <x:c r="H13" s="29"/>
-      <x:c r="I13" s="29"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
+      <x:c r="E13" s="139"/>
+      <x:c r="F13" s="139"/>
+      <x:c r="G13" s="139"/>
+      <x:c r="H13" s="139"/>
+      <x:c r="I13" s="150"/>
+    </x:row>
+    <x:row r="14" ht="2" customHeight="1">
+      <x:c r="A14" s="141" t="str">
         <x:v>ENGAGE — Growth</x:v>
       </x:c>
-      <x:c r="B14" s="62" t="n">
+      <x:c r="B14" s="142" t="n">
         <x:f>SUM('Engage Monthly'!G5:G16)</x:f>
         <x:v>19422</x:v>
       </x:c>
-      <x:c r="C14" s="62" t="n">
+      <x:c r="C14" s="142" t="n">
         <x:f>SUM('Engage Monthly'!G17:G28)</x:f>
         <x:v>72732.9</x:v>
       </x:c>
-      <x:c r="D14" s="62" t="n">
+      <x:c r="D14" s="142" t="n">
         <x:f>SUM('Engage Monthly'!G29:G40)</x:f>
         <x:v>193383.36</x:v>
       </x:c>
-      <x:c r="E14" s="29"/>
-      <x:c r="F14" s="29"/>
-      <x:c r="G14" s="29"/>
-      <x:c r="H14" s="29"/>
-      <x:c r="I14" s="29"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
+      <x:c r="E14" s="143"/>
+      <x:c r="F14" s="143"/>
+      <x:c r="G14" s="143"/>
+      <x:c r="H14" s="143"/>
+      <x:c r="I14" s="145"/>
+    </x:row>
+    <x:row r="15" ht="2" customHeight="1">
+      <x:c r="A15" s="141" t="str">
         <x:v>ENGAGE — Scale</x:v>
       </x:c>
-      <x:c r="B15" s="62" t="n">
+      <x:c r="B15" s="142" t="n">
         <x:f>SUM('Engage Monthly'!I5:I16)</x:f>
         <x:v>11680.5</x:v>
       </x:c>
-      <x:c r="C15" s="62" t="n">
+      <x:c r="C15" s="142" t="n">
         <x:f>SUM('Engage Monthly'!I17:I28)</x:f>
         <x:v>38875.100000000006</x:v>
       </x:c>
-      <x:c r="D15" s="62" t="n">
+      <x:c r="D15" s="142" t="n">
         <x:f>SUM('Engage Monthly'!I29:I40)</x:f>
         <x:v>96534.84</x:v>
       </x:c>
-      <x:c r="E15" s="29"/>
-      <x:c r="F15" s="29"/>
-      <x:c r="G15" s="29"/>
-      <x:c r="H15" s="29"/>
-      <x:c r="I15" s="29"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+      <x:c r="E15" s="143"/>
+      <x:c r="F15" s="143"/>
+      <x:c r="G15" s="143"/>
+      <x:c r="H15" s="143"/>
+      <x:c r="I15" s="145"/>
+    </x:row>
+    <x:row r="16" ht="2" customHeight="1">
+      <x:c r="A16" s="141" t="str">
         <x:v>ENGAGE — Enterprise</x:v>
       </x:c>
-      <x:c r="B16" s="62" t="n">
+      <x:c r="B16" s="142" t="n">
         <x:f>SUM('Engage Monthly'!K5:K16)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C16" s="62" t="n">
+      <x:c r="C16" s="142" t="n">
         <x:f>SUM('Engage Monthly'!K17:K28)</x:f>
         <x:v>6500</x:v>
       </x:c>
-      <x:c r="D16" s="62" t="n">
+      <x:c r="D16" s="142" t="n">
         <x:f>SUM('Engage Monthly'!K29:K40)</x:f>
         <x:v>23800</x:v>
       </x:c>
-      <x:c r="E16" s="29"/>
-      <x:c r="F16" s="29"/>
-      <x:c r="G16" s="29"/>
-      <x:c r="H16" s="29"/>
-      <x:c r="I16" s="29"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="E16" s="143"/>
+      <x:c r="F16" s="143"/>
+      <x:c r="G16" s="143"/>
+      <x:c r="H16" s="143"/>
+      <x:c r="I16" s="145"/>
+    </x:row>
+    <x:row r="17" ht="2" customHeight="1">
+      <x:c r="A17" s="141" t="str">
         <x:v>ENGAGE — Usage/add-ons</x:v>
       </x:c>
-      <x:c r="B17" s="62" t="n">
+      <x:c r="B17" s="142" t="n">
         <x:f>SUM('Engage Monthly'!M5:M16)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C17" s="62" t="n">
+      <x:c r="C17" s="142" t="n">
         <x:f>SUM('Engage Monthly'!M17:M28)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D17" s="62" t="n">
+      <x:c r="D17" s="142" t="n">
         <x:f>SUM('Engage Monthly'!M29:M40)</x:f>
         <x:v>11065.241999999998</x:v>
       </x:c>
-      <x:c r="E17" s="29"/>
-      <x:c r="F17" s="29"/>
-      <x:c r="G17" s="29"/>
-      <x:c r="H17" s="29"/>
-      <x:c r="I17" s="29"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+      <x:c r="E17" s="143"/>
+      <x:c r="F17" s="143"/>
+      <x:c r="G17" s="143"/>
+      <x:c r="H17" s="143"/>
+      <x:c r="I17" s="145"/>
+    </x:row>
+    <x:row r="18" ht="2" customHeight="1">
+      <x:c r="A18" s="146" t="str">
         <x:v>ENGAGE — Onboarding</x:v>
       </x:c>
-      <x:c r="B18" s="62" t="n">
+      <x:c r="B18" s="147" t="n">
         <x:f>SUM('Engage Monthly'!R5:R16)</x:f>
         <x:v>18000</x:v>
       </x:c>
-      <x:c r="C18" s="62" t="n">
+      <x:c r="C18" s="147" t="n">
         <x:f>SUM('Engage Monthly'!R17:R28)</x:f>
         <x:v>29000.00000000001</x:v>
       </x:c>
-      <x:c r="D18" s="62" t="n">
+      <x:c r="D18" s="147" t="n">
         <x:f>SUM('Engage Monthly'!R29:R40)</x:f>
         <x:v>50800.00000000001</x:v>
       </x:c>
-      <x:c r="E18" s="29"/>
-      <x:c r="F18" s="29"/>
-      <x:c r="G18" s="29"/>
-      <x:c r="H18" s="29"/>
-      <x:c r="I18" s="29"/>
+      <x:c r="E18" s="148"/>
+      <x:c r="F18" s="148"/>
+      <x:c r="G18" s="148"/>
+      <x:c r="H18" s="148"/>
+      <x:c r="I18" s="149"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="63" t="str">
@@ -1749,7 +2129,7 @@
       </x:c>
       <x:c r="E26" s="29"/>
       <x:c r="F26" s="68" t="str">
-        <x:v>Underwriting note: Paid Beta bookings are shown separately from recognized revenue. Commercial Y1 begins at GA. Beta customers roll into Y1 as opening cohorts and are never counted twice. B2B retention remains a disclosed 90% management target pending renewal evidence.</x:v>
+        <x:v>Beta cash bookings are separate from recognized revenue. Commercial Y1 begins at GA, Beta cohorts roll forward once, and the 90% B2B retention rate remains a target until renewal evidence exists.</x:v>
       </x:c>
       <x:c r="G26" s="68" t="str">
         <x:v>Underwriting note: Paid Beta bookings are shown separately from recognized revenue. Commercial Y1 begins at GA. Beta customers roll into Y1 as opening cohorts and are never counted twice. B2B retention remains a disclosed 90% management target pending renewal evidence.</x:v>
@@ -1862,28 +2242,28 @@
       <x:c r="H30" s="29"/>
       <x:c r="I30" s="29"/>
     </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="29" t="str">
+    <x:row r="31" ht="2" customHeight="1">
+      <x:c r="A31" s="151" t="str">
         <x:f>'Scenarios'!A5</x:f>
         <x:v>Conservative</x:v>
       </x:c>
-      <x:c r="B31" s="62" t="n">
+      <x:c r="B31" s="152" t="n">
         <x:f>'Scenarios'!B5</x:f>
         <x:v>83997.2</x:v>
       </x:c>
-      <x:c r="C31" s="62" t="n">
+      <x:c r="C31" s="152" t="n">
         <x:f>'Scenarios'!C5</x:f>
         <x:v>266877.7766666666</x:v>
       </x:c>
-      <x:c r="D31" s="62" t="n">
+      <x:c r="D31" s="152" t="n">
         <x:f>'Scenarios'!D5</x:f>
         <x:v>719471.6521</x:v>
       </x:c>
-      <x:c r="E31" s="29"/>
-      <x:c r="F31" s="29"/>
-      <x:c r="G31" s="29"/>
-      <x:c r="H31" s="29"/>
-      <x:c r="I31" s="29"/>
+      <x:c r="E31" s="153"/>
+      <x:c r="F31" s="153"/>
+      <x:c r="G31" s="153"/>
+      <x:c r="H31" s="153"/>
+      <x:c r="I31" s="154"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="29" t="str">
@@ -1931,23 +2311,28 @@
       <x:c r="H33" s="29"/>
       <x:c r="I33" s="29"/>
     </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="98" t="str">
+    <x:row r="34" ht="2" customHeight="1">
+      <x:c r="A34" s="161" t="str">
         <x:f>'Scenarios'!A8</x:f>
         <x:v>Upside</x:v>
       </x:c>
-      <x:c r="B34" s="99" t="n">
+      <x:c r="B34" s="162" t="n">
         <x:f>'Scenarios'!B8</x:f>
         <x:v>155574.59</x:v>
       </x:c>
-      <x:c r="C34" s="99" t="n">
+      <x:c r="C34" s="162" t="n">
         <x:f>'Scenarios'!C8</x:f>
         <x:v>494816.3022</x:v>
       </x:c>
-      <x:c r="D34" s="99" t="n">
+      <x:c r="D34" s="162" t="n">
         <x:f>'Scenarios'!D8</x:f>
         <x:v>1333338.16806</x:v>
       </x:c>
+      <x:c r="E34" s="163"/>
+      <x:c r="F34" s="163"/>
+      <x:c r="G34" s="163"/>
+      <x:c r="H34" s="163"/>
+      <x:c r="I34" s="164"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1956,7 +2341,7 @@
     <x:mergeCell ref="F26:I28"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c4b02dc3896495e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0e71685d1f049b6"/>
 </x:worksheet>
 </file>
 
@@ -1980,7 +2365,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="126" t="str">
-        <x:v>Marketing-Backed Operating Plan</x:v>
+        <x:v>Go-to-Market Plan</x:v>
       </x:c>
       <x:c r="B1" s="126"/>
       <x:c r="C1" s="126"/>
@@ -1996,7 +2381,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="127" t="str">
-        <x:v>The Underwritten Base remains the investor commitment. This case keeps price and retention unchanged and increases gross-new acquisition only.</x:v>
+        <x:v>Acquisition targets, scale gates, budgets, and the revenue uplift they support</x:v>
       </x:c>
       <x:c r="B2" s="127"/>
       <x:c r="C2" s="127"/>
@@ -2493,120 +2878,145 @@
         <x:v>Product-suite efficiency</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="28" customHeight="1">
-      <x:c r="A30" s="107" t="str">
+    <x:row r="30" ht="2" customHeight="1">
+      <x:c r="A30" s="232" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="B30" s="107" t="str">
+      <x:c r="B30" s="233" t="str">
         <x:v>Timing</x:v>
       </x:c>
-      <x:c r="C30" s="107" t="str">
+      <x:c r="C30" s="233" t="str">
         <x:v>Goal</x:v>
       </x:c>
-      <x:c r="D30" s="107" t="str">
+      <x:c r="D30" s="233" t="str">
         <x:v>Individuals</x:v>
       </x:c>
-      <x:c r="E30" s="107" t="str">
+      <x:c r="E30" s="233" t="str">
         <x:v>Teams</x:v>
       </x:c>
-      <x:c r="F30" s="107" t="str">
+      <x:c r="F30" s="233" t="str">
         <x:v>Engage</x:v>
       </x:c>
-      <x:c r="G30" s="107" t="str">
+      <x:c r="G30" s="233" t="str">
         <x:v>Evidence produced</x:v>
       </x:c>
-    </x:row>
-    <x:row r="31" ht="48" customHeight="1">
-      <x:c r="A31" s="130" t="str">
+      <x:c r="H30" s="234"/>
+      <x:c r="I30" s="234"/>
+      <x:c r="J30" s="234"/>
+      <x:c r="K30" s="234"/>
+      <x:c r="L30" s="235"/>
+    </x:row>
+    <x:row r="31" ht="2" customHeight="1">
+      <x:c r="A31" s="236" t="str">
         <x:v>Close Beta</x:v>
       </x:c>
-      <x:c r="B31" s="130" t="str">
+      <x:c r="B31" s="237" t="str">
         <x:v>Now → access release</x:v>
       </x:c>
-      <x:c r="C31" s="130" t="str">
+      <x:c r="C31" s="237" t="str">
         <x:v>Sign the starting cohort</x:v>
       </x:c>
-      <x:c r="D31" s="130" t="str">
+      <x:c r="D31" s="237" t="str">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="E31" s="130" t="str">
+      <x:c r="E31" s="237" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F31" s="130" t="str">
+      <x:c r="F31" s="237" t="str">
         <x:v>Design partners</x:v>
       </x:c>
-      <x:c r="G31" s="130" t="str">
+      <x:c r="G31" s="237" t="str">
         <x:v>Signed commitments + ICP notes</x:v>
       </x:c>
-    </x:row>
-    <x:row r="32" ht="48" customHeight="1">
-      <x:c r="A32" s="130" t="str">
+      <x:c r="H31" s="238"/>
+      <x:c r="I31" s="238"/>
+      <x:c r="J31" s="238"/>
+      <x:c r="K31" s="238"/>
+      <x:c r="L31" s="239"/>
+    </x:row>
+    <x:row r="32" ht="2" customHeight="1">
+      <x:c r="A32" s="236" t="str">
         <x:v>Build + validate</x:v>
       </x:c>
-      <x:c r="B32" s="130" t="str">
+      <x:c r="B32" s="237" t="str">
         <x:v>Beta months 1–4</x:v>
       </x:c>
-      <x:c r="C32" s="130" t="str">
+      <x:c r="C32" s="237" t="str">
         <x:v>Prove recurring workflow value</x:v>
       </x:c>
-      <x:c r="D32" s="130" t="str">
+      <x:c r="D32" s="237" t="str">
         <x:v>12 active</x:v>
       </x:c>
-      <x:c r="E32" s="130" t="str">
+      <x:c r="E32" s="237" t="str">
         <x:v>2 active</x:v>
       </x:c>
-      <x:c r="F32" s="130" t="str">
+      <x:c r="F32" s="237" t="str">
         <x:v>Workflow interviews</x:v>
       </x:c>
-      <x:c r="G32" s="130" t="str">
+      <x:c r="G32" s="237" t="str">
         <x:v>Activation, usage, pilot feedback</x:v>
       </x:c>
-    </x:row>
-    <x:row r="33" ht="48" customHeight="1">
-      <x:c r="A33" s="130" t="str">
+      <x:c r="H32" s="238"/>
+      <x:c r="I32" s="238"/>
+      <x:c r="J32" s="238"/>
+      <x:c r="K32" s="238"/>
+      <x:c r="L32" s="239"/>
+    </x:row>
+    <x:row r="33" ht="2" customHeight="1">
+      <x:c r="A33" s="236" t="str">
         <x:v>Expand Beta</x:v>
       </x:c>
-      <x:c r="B33" s="130" t="str">
+      <x:c r="B33" s="237" t="str">
         <x:v>Beta months 5–6</x:v>
       </x:c>
-      <x:c r="C33" s="130" t="str">
+      <x:c r="C33" s="237" t="str">
         <x:v>Test referrals and repeatability</x:v>
       </x:c>
-      <x:c r="D33" s="130" t="str">
+      <x:c r="D33" s="237" t="str">
         <x:v>30 active</x:v>
       </x:c>
-      <x:c r="E33" s="130" t="str">
+      <x:c r="E33" s="237" t="str">
         <x:v>2 active</x:v>
       </x:c>
-      <x:c r="F33" s="130" t="str">
+      <x:c r="F33" s="237" t="str">
         <x:v>First vertical shortlist</x:v>
       </x:c>
-      <x:c r="G33" s="130" t="str">
+      <x:c r="G33" s="237" t="str">
         <x:v>Individual expansion, Team Pro workflow adoption, pilot feedback</x:v>
       </x:c>
-    </x:row>
-    <x:row r="34" ht="48" customHeight="1">
-      <x:c r="A34" s="130" t="str">
+      <x:c r="H33" s="238"/>
+      <x:c r="I33" s="238"/>
+      <x:c r="J33" s="238"/>
+      <x:c r="K33" s="238"/>
+      <x:c r="L33" s="239"/>
+    </x:row>
+    <x:row r="34" ht="2" customHeight="1">
+      <x:c r="A34" s="240" t="str">
         <x:v>Commercial scale</x:v>
       </x:c>
-      <x:c r="B34" s="130" t="str">
+      <x:c r="B34" s="241" t="str">
         <x:v>From May 2027</x:v>
       </x:c>
-      <x:c r="C34" s="130" t="str">
+      <x:c r="C34" s="241" t="str">
         <x:v>Acquire only behind gates</x:v>
       </x:c>
-      <x:c r="D34" s="130" t="str">
+      <x:c r="D34" s="241" t="str">
         <x:v>120 Y1 new</x:v>
       </x:c>
-      <x:c r="E34" s="130" t="str">
+      <x:c r="E34" s="241" t="str">
         <x:v>24 Y1 new</x:v>
       </x:c>
-      <x:c r="F34" s="130" t="str">
+      <x:c r="F34" s="241" t="str">
         <x:v>36 Y1 new</x:v>
       </x:c>
-      <x:c r="G34" s="130" t="str">
+      <x:c r="G34" s="241" t="str">
         <x:v>Conversion, retention, CAC payback</x:v>
       </x:c>
+      <x:c r="H34" s="242"/>
+      <x:c r="I34" s="242"/>
+      <x:c r="J34" s="242"/>
+      <x:c r="K34" s="242"/>
+      <x:c r="L34" s="243"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2614,7 +3024,7 @@
     <x:mergeCell ref="A2:L2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raff36639ceb24aee"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe8729dc5b6644f6"/>
 </x:worksheet>
 </file>
 
@@ -2626,13 +3036,13 @@
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="1" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="1" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="1" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="1" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
@@ -2640,7 +3050,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>Paid Private Beta — Six-Month Underwriting</x:v>
+        <x:v>Paid Beta Plan</x:v>
       </x:c>
       <x:c r="B1" s="19" t="str">
         <x:v>Paid Private Beta — Six-Month Underwriting</x:v>
@@ -2651,10 +3061,10 @@
       <x:c r="D1" s="19" t="str">
         <x:v>Paid Private Beta — Six-Month Underwriting</x:v>
       </x:c>
-      <x:c r="E1" s="19" t="str">
+      <x:c r="E1" s="177" t="str">
         <x:v>Paid Private Beta — Six-Month Underwriting</x:v>
       </x:c>
-      <x:c r="F1" s="19" t="str">
+      <x:c r="F1" s="178" t="str">
         <x:v>Paid Private Beta — Six-Month Underwriting</x:v>
       </x:c>
       <x:c r="G1" s="19" t="str">
@@ -2666,10 +3076,10 @@
       <x:c r="I1" s="19" t="str">
         <x:v>Paid Private Beta — Six-Month Underwriting</x:v>
       </x:c>
-      <x:c r="J1" s="19" t="str">
+      <x:c r="J1" s="177" t="str">
         <x:v>Paid Private Beta — Six-Month Underwriting</x:v>
       </x:c>
-      <x:c r="K1" s="19" t="str">
+      <x:c r="K1" s="178" t="str">
         <x:v>Paid Private Beta — Six-Month Underwriting</x:v>
       </x:c>
       <x:c r="L1" s="19" t="str">
@@ -2684,7 +3094,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>Recruit now, release access mid-Oct 2026, model six full months Nov 2026–Apr 2027, then commercial GA. Beta target: 30 Individual Pro passes and two founding Team Pro workspaces.</x:v>
+        <x:v>Six-month cohort plan, bookings, recognized revenue, and exit ARR</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>Recruit now, release access mid-Oct 2026, model six full months Nov 2026–Apr 2027, then commercial GA in May 2027.</x:v>
@@ -2695,10 +3105,10 @@
       <x:c r="D2" s="20" t="str">
         <x:v>Recruit now, release access mid-Oct 2026, model six full months Nov 2026–Apr 2027, then commercial GA in May 2027.</x:v>
       </x:c>
-      <x:c r="E2" s="20" t="str">
+      <x:c r="E2" s="179" t="str">
         <x:v>Recruit now, release access mid-Oct 2026, model six full months Nov 2026–Apr 2027, then commercial GA in May 2027.</x:v>
       </x:c>
-      <x:c r="F2" s="20" t="str">
+      <x:c r="F2" s="180" t="str">
         <x:v>Recruit now, release access mid-Oct 2026, model six full months Nov 2026–Apr 2027, then commercial GA in May 2027.</x:v>
       </x:c>
       <x:c r="G2" s="20" t="str">
@@ -2710,10 +3120,10 @@
       <x:c r="I2" s="20" t="str">
         <x:v>Recruit now, release access mid-Oct 2026, model six full months Nov 2026–Apr 2027, then commercial GA in May 2027.</x:v>
       </x:c>
-      <x:c r="J2" s="20" t="str">
+      <x:c r="J2" s="179" t="str">
         <x:v>Recruit now, release access mid-Oct 2026, model six full months Nov 2026–Apr 2027, then commercial GA in May 2027.</x:v>
       </x:c>
-      <x:c r="K2" s="20" t="str">
+      <x:c r="K2" s="180" t="str">
         <x:v>Recruit now, release access mid-Oct 2026, model six full months Nov 2026–Apr 2027, then commercial GA in May 2027.</x:v>
       </x:c>
       <x:c r="L2" s="20" t="str">
@@ -2731,13 +3141,13 @@
       <x:c r="B3" s="29"/>
       <x:c r="C3" s="29"/>
       <x:c r="D3" s="29"/>
-      <x:c r="E3" s="29"/>
-      <x:c r="F3" s="29"/>
+      <x:c r="E3" s="141"/>
+      <x:c r="F3" s="145"/>
       <x:c r="G3" s="29"/>
       <x:c r="H3" s="29"/>
       <x:c r="I3" s="29"/>
-      <x:c r="J3" s="29"/>
-      <x:c r="K3" s="29"/>
+      <x:c r="J3" s="141"/>
+      <x:c r="K3" s="145"/>
       <x:c r="L3" s="29"/>
       <x:c r="M3" s="29"/>
       <x:c r="N3" s="29"/>
@@ -2755,10 +3165,10 @@
       <x:c r="D4" s="22" t="str">
         <x:v>Active individuals</x:v>
       </x:c>
-      <x:c r="E4" s="22" t="str">
+      <x:c r="E4" s="181" t="str">
         <x:v>Individual bookings</x:v>
       </x:c>
-      <x:c r="F4" s="22" t="str">
+      <x:c r="F4" s="182" t="str">
         <x:v>Individual revenue</x:v>
       </x:c>
       <x:c r="G4" s="22" t="str">
@@ -2770,10 +3180,10 @@
       <x:c r="I4" s="22" t="str">
         <x:v>Seats / team</x:v>
       </x:c>
-      <x:c r="J4" s="22" t="str">
+      <x:c r="J4" s="181" t="str">
         <x:v>Team bookings</x:v>
       </x:c>
-      <x:c r="K4" s="22" t="str">
+      <x:c r="K4" s="182" t="str">
         <x:v>Team revenue</x:v>
       </x:c>
       <x:c r="L4" s="22" t="str">
@@ -2801,11 +3211,11 @@
         <x:f>C5</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="E5" s="76" t="n">
+      <x:c r="E5" s="183" t="n">
         <x:f>C5*'Assumptions'!$B$10</x:f>
         <x:v>2280</x:v>
       </x:c>
-      <x:c r="F5" s="76" t="n">
+      <x:c r="F5" s="184" t="n">
         <x:f>D5*'Assumptions'!$B$10/12</x:f>
         <x:v>190</x:v>
       </x:c>
@@ -2821,11 +3231,11 @@
         <x:f>'Assumptions'!$B$13</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="J5" s="76" t="n">
+      <x:c r="J5" s="183" t="n">
         <x:f>G5*I5*'Assumptions'!$B$14</x:f>
         <x:v>1440</x:v>
       </x:c>
-      <x:c r="K5" s="76" t="n">
+      <x:c r="K5" s="184" t="n">
         <x:f>H5*I5*'Assumptions'!$B$14/12</x:f>
         <x:v>120</x:v>
       </x:c>
@@ -2857,11 +3267,11 @@
         <x:f>D5+C6</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="E6" s="76" t="n">
+      <x:c r="E6" s="183" t="n">
         <x:f>C6*'Assumptions'!$B$10</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F6" s="76" t="n">
+      <x:c r="F6" s="184" t="n">
         <x:f>D6*'Assumptions'!$B$10/12</x:f>
         <x:v>190</x:v>
       </x:c>
@@ -2877,11 +3287,11 @@
         <x:f>'Assumptions'!$B$13</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="J6" s="76" t="n">
+      <x:c r="J6" s="183" t="n">
         <x:f>G6*I6*'Assumptions'!$B$14</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K6" s="76" t="n">
+      <x:c r="K6" s="184" t="n">
         <x:f>H6*I6*'Assumptions'!$B$14/12</x:f>
         <x:v>120</x:v>
       </x:c>
@@ -2913,11 +3323,11 @@
         <x:f>D6+C7</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="E7" s="76" t="n">
+      <x:c r="E7" s="183" t="n">
         <x:f>C7*'Assumptions'!$B$10</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F7" s="76" t="n">
+      <x:c r="F7" s="184" t="n">
         <x:f>D7*'Assumptions'!$B$10/12</x:f>
         <x:v>190</x:v>
       </x:c>
@@ -2933,11 +3343,11 @@
         <x:f>'Assumptions'!$B$13</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="J7" s="76" t="n">
+      <x:c r="J7" s="183" t="n">
         <x:f>G7*I7*'Assumptions'!$B$14</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K7" s="76" t="n">
+      <x:c r="K7" s="184" t="n">
         <x:f>H7*I7*'Assumptions'!$B$14/12</x:f>
         <x:v>120</x:v>
       </x:c>
@@ -2969,11 +3379,11 @@
         <x:f>D7+C8</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="E8" s="76" t="n">
+      <x:c r="E8" s="183" t="n">
         <x:f>C8*'Assumptions'!$B$10</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F8" s="76" t="n">
+      <x:c r="F8" s="184" t="n">
         <x:f>D8*'Assumptions'!$B$10/12</x:f>
         <x:v>190</x:v>
       </x:c>
@@ -2989,11 +3399,11 @@
         <x:f>'Assumptions'!$B$13</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="J8" s="76" t="n">
+      <x:c r="J8" s="183" t="n">
         <x:f>G8*I8*'Assumptions'!$B$14</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K8" s="76" t="n">
+      <x:c r="K8" s="184" t="n">
         <x:f>H8*I8*'Assumptions'!$B$14/12</x:f>
         <x:v>120</x:v>
       </x:c>
@@ -3025,11 +3435,11 @@
         <x:f>D8+C9</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="E9" s="76" t="n">
+      <x:c r="E9" s="183" t="n">
         <x:f>C9*'Assumptions'!$B$10</x:f>
         <x:v>3420</x:v>
       </x:c>
-      <x:c r="F9" s="76" t="n">
+      <x:c r="F9" s="184" t="n">
         <x:f>D9*'Assumptions'!$B$10/12</x:f>
         <x:v>475</x:v>
       </x:c>
@@ -3045,11 +3455,11 @@
         <x:f>'Assumptions'!$B$13</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="J9" s="76" t="n">
+      <x:c r="J9" s="183" t="n">
         <x:f>G9*I9*'Assumptions'!$B$14</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K9" s="76" t="n">
+      <x:c r="K9" s="184" t="n">
         <x:f>H9*I9*'Assumptions'!$B$14/12</x:f>
         <x:v>120</x:v>
       </x:c>
@@ -3081,11 +3491,11 @@
         <x:f>D9+C10</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="E10" s="76" t="n">
+      <x:c r="E10" s="183" t="n">
         <x:f>C10*'Assumptions'!$B$10</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F10" s="76" t="n">
+      <x:c r="F10" s="184" t="n">
         <x:f>D10*'Assumptions'!$B$10/12</x:f>
         <x:v>475</x:v>
       </x:c>
@@ -3101,11 +3511,11 @@
         <x:f>'Assumptions'!$B$13</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="J10" s="76" t="n">
+      <x:c r="J10" s="183" t="n">
         <x:f>G10*I10*'Assumptions'!$B$14</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K10" s="76" t="n">
+      <x:c r="K10" s="184" t="n">
         <x:f>H10*I10*'Assumptions'!$B$14/12</x:f>
         <x:v>120</x:v>
       </x:c>
@@ -3127,13 +3537,13 @@
       <x:c r="B11" s="29"/>
       <x:c r="C11" s="75"/>
       <x:c r="D11" s="75"/>
-      <x:c r="E11" s="76"/>
-      <x:c r="F11" s="76"/>
+      <x:c r="E11" s="183"/>
+      <x:c r="F11" s="184"/>
       <x:c r="G11" s="75"/>
       <x:c r="H11" s="75"/>
       <x:c r="I11" s="75"/>
-      <x:c r="J11" s="76"/>
-      <x:c r="K11" s="76"/>
+      <x:c r="J11" s="183"/>
+      <x:c r="K11" s="184"/>
       <x:c r="L11" s="76"/>
       <x:c r="M11" s="76"/>
       <x:c r="N11" s="76"/>
@@ -3145,22 +3555,22 @@
       <x:c r="B12" s="65"/>
       <x:c r="C12" s="77"/>
       <x:c r="D12" s="77"/>
-      <x:c r="E12" s="78" t="n">
+      <x:c r="E12" s="185" t="n">
         <x:f>SUM(E5:E10)</x:f>
         <x:v>5700</x:v>
       </x:c>
-      <x:c r="F12" s="78" t="n">
+      <x:c r="F12" s="186" t="n">
         <x:f>SUM(F5:F10)</x:f>
         <x:v>1710</x:v>
       </x:c>
       <x:c r="G12" s="77"/>
       <x:c r="H12" s="77"/>
       <x:c r="I12" s="77"/>
-      <x:c r="J12" s="78" t="n">
+      <x:c r="J12" s="185" t="n">
         <x:f>SUM(J5:J10)</x:f>
         <x:v>1440</x:v>
       </x:c>
-      <x:c r="K12" s="78" t="n">
+      <x:c r="K12" s="186" t="n">
         <x:f>SUM(K5:K10)</x:f>
         <x:v>720</x:v>
       </x:c>
@@ -3182,20 +3592,20 @@
       <x:c r="B13" s="29"/>
       <x:c r="C13" s="29"/>
       <x:c r="D13" s="29"/>
-      <x:c r="E13" s="29"/>
-      <x:c r="F13" s="29"/>
+      <x:c r="E13" s="141"/>
+      <x:c r="F13" s="145"/>
       <x:c r="G13" s="29"/>
       <x:c r="H13" s="29"/>
       <x:c r="I13" s="29"/>
-      <x:c r="J13" s="29"/>
-      <x:c r="K13" s="29"/>
+      <x:c r="J13" s="141"/>
+      <x:c r="K13" s="145"/>
       <x:c r="L13" s="29"/>
       <x:c r="M13" s="29"/>
       <x:c r="N13" s="29"/>
     </x:row>
     <x:row r="14" ht="40" customHeight="1">
       <x:c r="A14" s="68" t="str">
-        <x:v>Accounting note: annual subscriptions are bookings/cash when collected, but revenue is recognized ratably. Beta customers enter Commercial Year 1 as opening cohorts and are not counted again as new acquisition.</x:v>
+        <x:v>Annual plans are collected upfront and recognized monthly. Beta customers enter Commercial Y1 as opening cohorts, not new acquisition.</x:v>
       </x:c>
       <x:c r="B14" s="68" t="str">
         <x:v>Accounting note: annual subscriptions are bookings/cash when collected, but revenue is recognized ratably. Beta customers enter Commercial Year 1 as opening cohorts and are not counted again as new acquisition.</x:v>
@@ -3206,10 +3616,10 @@
       <x:c r="D14" s="68" t="str">
         <x:v>Accounting note: annual subscriptions are bookings/cash when collected, but revenue is recognized ratably. Beta customers enter Commercial Year 1 as opening cohorts and are not counted again as new acquisition.</x:v>
       </x:c>
-      <x:c r="E14" s="68" t="str">
+      <x:c r="E14" s="187" t="str">
         <x:v>Accounting note: annual subscriptions are bookings/cash when collected, but revenue is recognized ratably. Beta customers enter Commercial Year 1 as opening cohorts and are not counted again as new acquisition.</x:v>
       </x:c>
-      <x:c r="F14" s="68" t="str">
+      <x:c r="F14" s="188" t="str">
         <x:v>Accounting note: annual subscriptions are bookings/cash when collected, but revenue is recognized ratably. Beta customers enter Commercial Year 1 as opening cohorts and are not counted again as new acquisition.</x:v>
       </x:c>
       <x:c r="G14" s="68" t="str">
@@ -3221,10 +3631,10 @@
       <x:c r="I14" s="68" t="str">
         <x:v>Accounting note: annual subscriptions are bookings/cash when collected, but revenue is recognized ratably. Beta customers enter Commercial Year 1 as opening cohorts and are not counted again as new acquisition.</x:v>
       </x:c>
-      <x:c r="J14" s="68" t="str">
+      <x:c r="J14" s="187" t="str">
         <x:v>Accounting note: annual subscriptions are bookings/cash when collected, but revenue is recognized ratably. Beta customers enter Commercial Year 1 as opening cohorts and are not counted again as new acquisition.</x:v>
       </x:c>
-      <x:c r="K14" s="68" t="str">
+      <x:c r="K14" s="188" t="str">
         <x:v>Accounting note: annual subscriptions are bookings/cash when collected, but revenue is recognized ratably. Beta customers enter Commercial Year 1 as opening cohorts and are not counted again as new acquisition.</x:v>
       </x:c>
       <x:c r="L14" s="68" t="str">
@@ -3256,14 +3666,14 @@
     <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="1" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="21" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="1" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>MIMAR Revenue Model — Defensible Assumptions</x:v>
+        <x:v>Key Model Assumptions</x:v>
       </x:c>
       <x:c r="B1" s="19" t="str">
         <x:v>MIMAR Revenue Model — Defensible Assumptions</x:v>
@@ -3277,19 +3687,19 @@
       <x:c r="E1" s="19" t="str">
         <x:v>MIMAR Revenue Model — Defensible Assumptions</x:v>
       </x:c>
-      <x:c r="F1" s="19" t="str">
+      <x:c r="F1" s="189" t="str">
         <x:v>MIMAR Revenue Model — Defensible Assumptions</x:v>
       </x:c>
       <x:c r="G1" s="19" t="str">
         <x:v>MIMAR Revenue Model — Defensible Assumptions</x:v>
       </x:c>
-      <x:c r="H1" s="19" t="str">
+      <x:c r="H1" s="189" t="str">
         <x:v>MIMAR Revenue Model — Defensible Assumptions</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>Paid Beta precedes a 36-month commercial forecast. Blue cells are editable; formulas roll from these drivers.</x:v>
+        <x:v>Commercial inputs and current validation status. Evidence and rationale remain in the supporting columns.</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>Paid Beta precedes a 36-month commercial forecast. Blue cells are editable; formulas roll from these drivers.</x:v>
@@ -3303,13 +3713,13 @@
       <x:c r="E2" s="20" t="str">
         <x:v>Paid Beta precedes a 36-month commercial forecast. Blue cells are editable; formulas roll from these drivers.</x:v>
       </x:c>
-      <x:c r="F2" s="20" t="str">
+      <x:c r="F2" s="190" t="str">
         <x:v>Paid Beta precedes a 36-month commercial forecast. Blue cells are editable; formulas roll from these drivers.</x:v>
       </x:c>
       <x:c r="G2" s="20" t="str">
         <x:v>Paid Beta precedes a 36-month commercial forecast. Blue cells are editable; formulas roll from these drivers.</x:v>
       </x:c>
-      <x:c r="H2" s="20" t="str">
+      <x:c r="H2" s="190" t="str">
         <x:v>Paid Beta precedes a 36-month commercial forecast. Blue cells are editable; formulas roll from these drivers.</x:v>
       </x:c>
     </x:row>
@@ -3319,9 +3729,9 @@
       <x:c r="C3" s="29"/>
       <x:c r="D3" s="29"/>
       <x:c r="E3" s="29"/>
-      <x:c r="F3" s="29"/>
+      <x:c r="F3" s="191"/>
       <x:c r="G3" s="29"/>
-      <x:c r="H3" s="29"/>
+      <x:c r="H3" s="191"/>
     </x:row>
     <x:row r="4" ht="27" customHeight="1">
       <x:c r="A4" s="22" t="str">
@@ -3339,13 +3749,13 @@
       <x:c r="E4" s="22" t="str">
         <x:v>Unit</x:v>
       </x:c>
-      <x:c r="F4" s="22" t="str">
+      <x:c r="F4" s="192" t="str">
         <x:v>Evidence type</x:v>
       </x:c>
       <x:c r="G4" s="22" t="str">
         <x:v>Validation status</x:v>
       </x:c>
-      <x:c r="H4" s="22" t="str">
+      <x:c r="H4" s="192" t="str">
         <x:v>Source / rationale</x:v>
       </x:c>
     </x:row>
@@ -3361,13 +3771,13 @@
       <x:c r="E5" s="29" t="str">
         <x:v>date</x:v>
       </x:c>
-      <x:c r="F5" s="29" t="str">
+      <x:c r="F5" s="191" t="str">
         <x:v>Management plan</x:v>
       </x:c>
       <x:c r="G5" s="29" t="str">
         <x:v>Scheduling</x:v>
       </x:c>
-      <x:c r="H5" s="36" t="str">
+      <x:c r="H5" s="196" t="str">
         <x:v>Mid-Oct operational target; monthly model begins Nov 2026</x:v>
       </x:c>
     </x:row>
@@ -3383,13 +3793,13 @@
       <x:c r="E6" s="29" t="str">
         <x:v>date</x:v>
       </x:c>
-      <x:c r="F6" s="29" t="str">
+      <x:c r="F6" s="191" t="str">
         <x:v>Management plan</x:v>
       </x:c>
       <x:c r="G6" s="29" t="str">
         <x:v>Scheduling</x:v>
       </x:c>
-      <x:c r="H6" s="36" t="str">
+      <x:c r="H6" s="196" t="str">
         <x:v>Six full modeled Beta months, then commercial launch</x:v>
       </x:c>
     </x:row>
@@ -3405,13 +3815,13 @@
       <x:c r="E7" s="29" t="str">
         <x:v>months</x:v>
       </x:c>
-      <x:c r="F7" s="29" t="str">
+      <x:c r="F7" s="191" t="str">
         <x:v>Management plan</x:v>
       </x:c>
       <x:c r="G7" s="29" t="str">
         <x:v>Defined</x:v>
       </x:c>
-      <x:c r="H7" s="36" t="str">
+      <x:c r="H7" s="196" t="str">
         <x:v>Private Beta development and validation window</x:v>
       </x:c>
     </x:row>
@@ -3427,13 +3837,13 @@
       <x:c r="E8" s="29" t="str">
         <x:v>users</x:v>
       </x:c>
-      <x:c r="F8" s="29" t="str">
+      <x:c r="F8" s="191" t="str">
         <x:v>Management target</x:v>
       </x:c>
       <x:c r="G8" s="29" t="str">
         <x:v>Closing now</x:v>
       </x:c>
-      <x:c r="H8" s="36" t="str">
+      <x:c r="H8" s="196" t="str">
         <x:v>Active during Beta months 1–4 and thereafter</x:v>
       </x:c>
     </x:row>
@@ -3449,13 +3859,13 @@
       <x:c r="E9" s="29" t="str">
         <x:v>users</x:v>
       </x:c>
-      <x:c r="F9" s="29" t="str">
+      <x:c r="F9" s="191" t="str">
         <x:v>Management target</x:v>
       </x:c>
       <x:c r="G9" s="29" t="str">
         <x:v>Recruit in Beta</x:v>
       </x:c>
-      <x:c r="H9" s="36" t="str">
+      <x:c r="H9" s="196" t="str">
         <x:v>Added in Beta month 5; 30 total at Beta exit</x:v>
       </x:c>
     </x:row>
@@ -3471,13 +3881,13 @@
       <x:c r="E10" s="29" t="str">
         <x:v>$/user/year</x:v>
       </x:c>
-      <x:c r="F10" s="29" t="str">
+      <x:c r="F10" s="191" t="str">
         <x:v>Founder price</x:v>
       </x:c>
       <x:c r="G10" s="29" t="str">
         <x:v>Management decision</x:v>
       </x:c>
-      <x:c r="H10" s="36" t="str">
+      <x:c r="H10" s="196" t="str">
         <x:v>Annual Pro price supplied by management</x:v>
       </x:c>
     </x:row>
@@ -3493,13 +3903,13 @@
       <x:c r="E11" s="29" t="str">
         <x:v>workspaces</x:v>
       </x:c>
-      <x:c r="F11" s="29" t="str">
+      <x:c r="F11" s="191" t="str">
         <x:v>Management target</x:v>
       </x:c>
       <x:c r="G11" s="29" t="str">
         <x:v>Closing now</x:v>
       </x:c>
-      <x:c r="H11" s="36" t="str">
+      <x:c r="H11" s="196" t="str">
         <x:v>First two team workspaces</x:v>
       </x:c>
     </x:row>
@@ -3515,13 +3925,13 @@
       <x:c r="E12" s="29" t="str">
         <x:v>workspaces</x:v>
       </x:c>
-      <x:c r="F12" s="29" t="str">
+      <x:c r="F12" s="191" t="str">
         <x:v>Management target</x:v>
       </x:c>
       <x:c r="G12" s="29" t="str">
         <x:v>Not targeted</x:v>
       </x:c>
-      <x:c r="H12" s="36" t="str">
+      <x:c r="H12" s="196" t="str">
         <x:v>Team Beta target is two founding Team Pro workspaces.</x:v>
       </x:c>
     </x:row>
@@ -3537,13 +3947,13 @@
       <x:c r="E13" s="29" t="str">
         <x:v>seats/workspace</x:v>
       </x:c>
-      <x:c r="F13" s="29" t="str">
+      <x:c r="F13" s="191" t="str">
         <x:v>Pricing assumption</x:v>
       </x:c>
       <x:c r="G13" s="29" t="str">
         <x:v>Validate in contracts</x:v>
       </x:c>
-      <x:c r="H13" s="36" t="str">
+      <x:c r="H13" s="196" t="str">
         <x:v>Minimum paid seats; team is not one user</x:v>
       </x:c>
     </x:row>
@@ -3559,13 +3969,13 @@
       <x:c r="E14" s="29" t="str">
         <x:v>$/seat/year</x:v>
       </x:c>
-      <x:c r="F14" s="29" t="str">
+      <x:c r="F14" s="191" t="str">
         <x:v>Founder price</x:v>
       </x:c>
       <x:c r="G14" s="29" t="str">
         <x:v>Management decision</x:v>
       </x:c>
-      <x:c r="H14" s="36" t="str">
+      <x:c r="H14" s="196" t="str">
         <x:v>$240 / seat / year Team Pro Beta offer; three-seat minimum per team.</x:v>
       </x:c>
     </x:row>
@@ -3581,13 +3991,13 @@
       <x:c r="E15" s="29" t="str">
         <x:v>% retained</x:v>
       </x:c>
-      <x:c r="F15" s="29" t="str">
+      <x:c r="F15" s="191" t="str">
         <x:v>Market anchored</x:v>
       </x:c>
       <x:c r="G15" s="29" t="str">
         <x:v>Validate at renewal</x:v>
       </x:c>
-      <x:c r="H15" s="36" t="str">
+      <x:c r="H15" s="196" t="str">
         <x:v>Applied at each annual renewal</x:v>
       </x:c>
     </x:row>
@@ -3603,13 +4013,13 @@
       <x:c r="E16" s="29" t="str">
         <x:v>% retained</x:v>
       </x:c>
-      <x:c r="F16" s="29" t="str">
+      <x:c r="F16" s="191" t="str">
         <x:v>Management target</x:v>
       </x:c>
       <x:c r="G16" s="29" t="str">
         <x:v>Validate at renewal</x:v>
       </x:c>
-      <x:c r="H16" s="36" t="str">
+      <x:c r="H16" s="196" t="str">
         <x:v>Applied at each annual renewal</x:v>
       </x:c>
     </x:row>
@@ -3625,13 +4035,13 @@
       <x:c r="E17" s="29" t="str">
         <x:v>months</x:v>
       </x:c>
-      <x:c r="F17" s="29" t="str">
+      <x:c r="F17" s="191" t="str">
         <x:v>Timing formula</x:v>
       </x:c>
       <x:c r="G17" s="29" t="str">
         <x:v>Defined</x:v>
       </x:c>
-      <x:c r="H17" s="36" t="str">
+      <x:c r="H17" s="196" t="str">
         <x:v>Nov 2026 start; renewal after six commercial months</x:v>
       </x:c>
     </x:row>
@@ -3647,13 +4057,13 @@
       <x:c r="E18" s="29" t="str">
         <x:v>months</x:v>
       </x:c>
-      <x:c r="F18" s="29" t="str">
+      <x:c r="F18" s="191" t="str">
         <x:v>Timing formula</x:v>
       </x:c>
       <x:c r="G18" s="29" t="str">
         <x:v>Defined</x:v>
       </x:c>
-      <x:c r="H18" s="36" t="str">
+      <x:c r="H18" s="196" t="str">
         <x:v>Mar 2027 start; renewal after ten commercial months</x:v>
       </x:c>
     </x:row>
@@ -3663,9 +4073,9 @@
       <x:c r="C19" s="32"/>
       <x:c r="D19" s="32"/>
       <x:c r="E19" s="29"/>
-      <x:c r="F19" s="29"/>
+      <x:c r="F19" s="191"/>
       <x:c r="G19" s="29"/>
-      <x:c r="H19" s="36"/>
+      <x:c r="H19" s="196"/>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="35" t="str">
@@ -3683,13 +4093,13 @@
       <x:c r="E20" s="29" t="str">
         <x:v>new users</x:v>
       </x:c>
-      <x:c r="F20" s="29" t="str">
+      <x:c r="F20" s="191" t="str">
         <x:v>Management case</x:v>
       </x:c>
       <x:c r="G20" s="29" t="str">
         <x:v>Validate with cohorts</x:v>
       </x:c>
-      <x:c r="H20" s="36" t="str">
+      <x:c r="H20" s="196" t="str">
         <x:v>Commercial acquisition excludes Beta customers</x:v>
       </x:c>
     </x:row>
@@ -3709,13 +4119,13 @@
       <x:c r="E21" s="29" t="str">
         <x:v>% retained</x:v>
       </x:c>
-      <x:c r="F21" s="29" t="str">
+      <x:c r="F21" s="191" t="str">
         <x:v>Market anchored</x:v>
       </x:c>
       <x:c r="G21" s="29" t="str">
         <x:v>Benchmark anchored</x:v>
       </x:c>
-      <x:c r="H21" s="36" t="str">
+      <x:c r="H21" s="196" t="str">
         <x:v>ChartMogul low-ARPA annual retention is ~62% on annual billing</x:v>
       </x:c>
     </x:row>
@@ -3735,13 +4145,13 @@
       <x:c r="E22" s="29" t="str">
         <x:v>$/month</x:v>
       </x:c>
-      <x:c r="F22" s="29" t="str">
+      <x:c r="F22" s="191" t="str">
         <x:v>Published price + mix</x:v>
       </x:c>
       <x:c r="G22" s="29" t="str">
         <x:v>Market anchored</x:v>
       </x:c>
-      <x:c r="H22" s="36" t="str">
+      <x:c r="H22" s="196" t="str">
         <x:v>Commercial mix; Beta Pro price is modeled separately</x:v>
       </x:c>
     </x:row>
@@ -3761,13 +4171,13 @@
       <x:c r="E23" s="29" t="str">
         <x:v>new workspaces</x:v>
       </x:c>
-      <x:c r="F23" s="29" t="str">
+      <x:c r="F23" s="191" t="str">
         <x:v>Management case</x:v>
       </x:c>
       <x:c r="G23" s="29" t="str">
         <x:v>Validate with pipeline</x:v>
       </x:c>
-      <x:c r="H23" s="36" t="str">
+      <x:c r="H23" s="196" t="str">
         <x:v>Commercial gross new workspaces; excludes two Beta teams</x:v>
       </x:c>
     </x:row>
@@ -3787,13 +4197,13 @@
       <x:c r="E24" s="29" t="str">
         <x:v>% retained</x:v>
       </x:c>
-      <x:c r="F24" s="29" t="str">
+      <x:c r="F24" s="191" t="str">
         <x:v>Management target</x:v>
       </x:c>
       <x:c r="G24" s="29" t="str">
         <x:v>Conditional target</x:v>
       </x:c>
-      <x:c r="H24" s="36" t="str">
+      <x:c r="H24" s="196" t="str">
         <x:v>Requires annual billing, workflow embedding and assisted onboarding</x:v>
       </x:c>
     </x:row>
@@ -3813,13 +4223,13 @@
       <x:c r="E25" s="29" t="str">
         <x:v>seats/workspace</x:v>
       </x:c>
-      <x:c r="F25" s="29" t="str">
+      <x:c r="F25" s="191" t="str">
         <x:v>Management assumption</x:v>
       </x:c>
       <x:c r="G25" s="29" t="str">
         <x:v>Validate with cohorts</x:v>
       </x:c>
-      <x:c r="H25" s="36" t="str">
+      <x:c r="H25" s="196" t="str">
         <x:v>Commercial seat expansion is explicit</x:v>
       </x:c>
     </x:row>
@@ -3839,13 +4249,13 @@
       <x:c r="E26" s="29" t="str">
         <x:v>$/seat/month</x:v>
       </x:c>
-      <x:c r="F26" s="29" t="str">
+      <x:c r="F26" s="191" t="str">
         <x:v>Published price + mix</x:v>
       </x:c>
       <x:c r="G26" s="29" t="str">
         <x:v>Market anchored</x:v>
       </x:c>
-      <x:c r="H26" s="36" t="str">
+      <x:c r="H26" s="196" t="str">
         <x:v>$12 Team Plus / $30 Team Pro</x:v>
       </x:c>
     </x:row>
@@ -3865,13 +4275,13 @@
       <x:c r="E27" s="29" t="str">
         <x:v>new contracts</x:v>
       </x:c>
-      <x:c r="F27" s="29" t="str">
+      <x:c r="F27" s="191" t="str">
         <x:v>Management case</x:v>
       </x:c>
       <x:c r="G27" s="29" t="str">
         <x:v>Pipeline gated</x:v>
       </x:c>
-      <x:c r="H27" s="36" t="str">
+      <x:c r="H27" s="196" t="str">
         <x:v>No enterprise revenue in commercial Y1 without contract</x:v>
       </x:c>
     </x:row>
@@ -3891,13 +4301,13 @@
       <x:c r="E28" s="29" t="str">
         <x:v>$/year</x:v>
       </x:c>
-      <x:c r="F28" s="29" t="str">
+      <x:c r="F28" s="191" t="str">
         <x:v>Market assumption</x:v>
       </x:c>
       <x:c r="G28" s="29" t="str">
         <x:v>Pipeline gated</x:v>
       </x:c>
-      <x:c r="H28" s="36" t="str">
+      <x:c r="H28" s="196" t="str">
         <x:v>Security, SSO, SLA and procurement required</x:v>
       </x:c>
     </x:row>
@@ -3917,13 +4327,13 @@
       <x:c r="E29" s="29" t="str">
         <x:v>new wallets</x:v>
       </x:c>
-      <x:c r="F29" s="29" t="str">
+      <x:c r="F29" s="191" t="str">
         <x:v>Management case</x:v>
       </x:c>
       <x:c r="G29" s="29" t="str">
         <x:v>Reliability gated</x:v>
       </x:c>
-      <x:c r="H29" s="36" t="str">
+      <x:c r="H29" s="196" t="str">
         <x:v>Usage retention modeled separately</x:v>
       </x:c>
     </x:row>
@@ -3943,13 +4353,13 @@
       <x:c r="E30" s="29" t="str">
         <x:v>% retained</x:v>
       </x:c>
-      <x:c r="F30" s="29" t="str">
+      <x:c r="F30" s="191" t="str">
         <x:v>Planning assumption</x:v>
       </x:c>
       <x:c r="G30" s="29" t="str">
         <x:v>Validate with wallets</x:v>
       </x:c>
-      <x:c r="H30" s="36" t="str">
+      <x:c r="H30" s="196" t="str">
         <x:v>Wallet usage is more volatile than B2B subscriptions</x:v>
       </x:c>
     </x:row>
@@ -3969,13 +4379,13 @@
       <x:c r="E31" s="29" t="str">
         <x:v>$/wallet/month</x:v>
       </x:c>
-      <x:c r="F31" s="29" t="str">
+      <x:c r="F31" s="191" t="str">
         <x:v>Usage assumption</x:v>
       </x:c>
       <x:c r="G31" s="29" t="str">
         <x:v>Validate with wallets</x:v>
       </x:c>
-      <x:c r="H31" s="36" t="str">
+      <x:c r="H31" s="196" t="str">
         <x:v>Only consumed prepaid balance is revenue</x:v>
       </x:c>
     </x:row>
@@ -3995,13 +4405,13 @@
       <x:c r="E32" s="29" t="str">
         <x:v>$/new account</x:v>
       </x:c>
-      <x:c r="F32" s="29" t="str">
+      <x:c r="F32" s="191" t="str">
         <x:v>Management decision</x:v>
       </x:c>
       <x:c r="G32" s="29" t="str">
         <x:v>Market anchored</x:v>
       </x:c>
-      <x:c r="H32" s="36" t="str">
+      <x:c r="H32" s="196" t="str">
         <x:v>Commercial gross new team and enterprise cohorts only</x:v>
       </x:c>
     </x:row>
@@ -4021,13 +4431,13 @@
       <x:c r="E33" s="29" t="str">
         <x:v>% revenue</x:v>
       </x:c>
-      <x:c r="F33" s="29" t="str">
+      <x:c r="F33" s="191" t="str">
         <x:v>Conservative benchmark</x:v>
       </x:c>
       <x:c r="G33" s="29" t="str">
         <x:v>Model assumption</x:v>
       </x:c>
-      <x:c r="H33" s="36" t="str">
+      <x:c r="H33" s="196" t="str">
         <x:v>Inference, hosting, storage and direct support</x:v>
       </x:c>
     </x:row>
@@ -4047,13 +4457,13 @@
       <x:c r="E34" s="29" t="str">
         <x:v>% revenue</x:v>
       </x:c>
-      <x:c r="F34" s="29" t="str">
+      <x:c r="F34" s="191" t="str">
         <x:v>Conservative benchmark</x:v>
       </x:c>
       <x:c r="G34" s="29" t="str">
         <x:v>Model assumption</x:v>
       </x:c>
-      <x:c r="H34" s="36" t="str">
+      <x:c r="H34" s="196" t="str">
         <x:v>Usage margin starts below mature software margin</x:v>
       </x:c>
     </x:row>
@@ -4073,13 +4483,13 @@
       <x:c r="E35" s="29" t="str">
         <x:v>% revenue</x:v>
       </x:c>
-      <x:c r="F35" s="29" t="str">
+      <x:c r="F35" s="191" t="str">
         <x:v>Industry benchmark</x:v>
       </x:c>
       <x:c r="G35" s="29" t="str">
         <x:v>Benchmark anchored</x:v>
       </x:c>
-      <x:c r="H35" s="36" t="str">
+      <x:c r="H35" s="196" t="str">
         <x:v>Professional services at 30% gross margin</x:v>
       </x:c>
     </x:row>
@@ -4089,9 +4499,9 @@
       <x:c r="C36" s="32"/>
       <x:c r="D36" s="32"/>
       <x:c r="E36" s="29"/>
-      <x:c r="F36" s="29"/>
+      <x:c r="F36" s="191"/>
       <x:c r="G36" s="29"/>
-      <x:c r="H36" s="36"/>
+      <x:c r="H36" s="196"/>
     </x:row>
     <x:row r="37" ht="22" customHeight="1">
       <x:c r="A37" s="35" t="str">
@@ -4109,13 +4519,13 @@
       <x:c r="E37" s="29" t="str">
         <x:v>new workspaces</x:v>
       </x:c>
-      <x:c r="F37" s="29" t="str">
+      <x:c r="F37" s="191" t="str">
         <x:v>Management case</x:v>
       </x:c>
       <x:c r="G37" s="29" t="str">
         <x:v>Validate with cohorts</x:v>
       </x:c>
-      <x:c r="H37" s="36" t="str">
+      <x:c r="H37" s="196" t="str">
         <x:v>Starts at commercial GA</x:v>
       </x:c>
     </x:row>
@@ -4135,13 +4545,13 @@
       <x:c r="E38" s="29" t="str">
         <x:v>$/month</x:v>
       </x:c>
-      <x:c r="F38" s="29" t="str">
+      <x:c r="F38" s="191" t="str">
         <x:v>Published price</x:v>
       </x:c>
       <x:c r="G38" s="29" t="str">
         <x:v>Market anchored</x:v>
       </x:c>
-      <x:c r="H38" s="36" t="str">
+      <x:c r="H38" s="196" t="str">
         <x:v>Current product price</x:v>
       </x:c>
     </x:row>
@@ -4161,13 +4571,13 @@
       <x:c r="E39" s="29" t="str">
         <x:v>new workspaces</x:v>
       </x:c>
-      <x:c r="F39" s="29" t="str">
+      <x:c r="F39" s="191" t="str">
         <x:v>Management case</x:v>
       </x:c>
       <x:c r="G39" s="29" t="str">
         <x:v>Validate with cohorts</x:v>
       </x:c>
-      <x:c r="H39" s="36" t="str">
+      <x:c r="H39" s="196" t="str">
         <x:v>Primary paid plan</x:v>
       </x:c>
     </x:row>
@@ -4187,13 +4597,13 @@
       <x:c r="E40" s="29" t="str">
         <x:v>$/month</x:v>
       </x:c>
-      <x:c r="F40" s="29" t="str">
+      <x:c r="F40" s="191" t="str">
         <x:v>Published price</x:v>
       </x:c>
       <x:c r="G40" s="29" t="str">
         <x:v>Market anchored</x:v>
       </x:c>
-      <x:c r="H40" s="36" t="str">
+      <x:c r="H40" s="196" t="str">
         <x:v>Current product price</x:v>
       </x:c>
     </x:row>
@@ -4213,13 +4623,13 @@
       <x:c r="E41" s="29" t="str">
         <x:v>new workspaces</x:v>
       </x:c>
-      <x:c r="F41" s="29" t="str">
+      <x:c r="F41" s="191" t="str">
         <x:v>Management case</x:v>
       </x:c>
       <x:c r="G41" s="29" t="str">
         <x:v>Validate with cohorts</x:v>
       </x:c>
-      <x:c r="H41" s="36" t="str">
+      <x:c r="H41" s="196" t="str">
         <x:v>Higher-support segment</x:v>
       </x:c>
     </x:row>
@@ -4239,13 +4649,13 @@
       <x:c r="E42" s="29" t="str">
         <x:v>$/month</x:v>
       </x:c>
-      <x:c r="F42" s="29" t="str">
+      <x:c r="F42" s="191" t="str">
         <x:v>Published price</x:v>
       </x:c>
       <x:c r="G42" s="29" t="str">
         <x:v>Market anchored</x:v>
       </x:c>
-      <x:c r="H42" s="36" t="str">
+      <x:c r="H42" s="196" t="str">
         <x:v>Current product price</x:v>
       </x:c>
     </x:row>
@@ -4265,13 +4675,13 @@
       <x:c r="E43" s="29" t="str">
         <x:v>new contracts</x:v>
       </x:c>
-      <x:c r="F43" s="29" t="str">
+      <x:c r="F43" s="191" t="str">
         <x:v>Management case</x:v>
       </x:c>
       <x:c r="G43" s="29" t="str">
         <x:v>Pipeline gated</x:v>
       </x:c>
-      <x:c r="H43" s="36" t="str">
+      <x:c r="H43" s="196" t="str">
         <x:v>No enterprise in commercial Y1 base</x:v>
       </x:c>
     </x:row>
@@ -4291,13 +4701,13 @@
       <x:c r="E44" s="29" t="str">
         <x:v>$/month</x:v>
       </x:c>
-      <x:c r="F44" s="29" t="str">
+      <x:c r="F44" s="191" t="str">
         <x:v>Published floor</x:v>
       </x:c>
       <x:c r="G44" s="29" t="str">
         <x:v>Market anchored</x:v>
       </x:c>
-      <x:c r="H44" s="36" t="str">
+      <x:c r="H44" s="196" t="str">
         <x:v>$12k minimum ACV</x:v>
       </x:c>
     </x:row>
@@ -4317,13 +4727,13 @@
       <x:c r="E45" s="29" t="str">
         <x:v>% retained</x:v>
       </x:c>
-      <x:c r="F45" s="29" t="str">
+      <x:c r="F45" s="191" t="str">
         <x:v>Management target</x:v>
       </x:c>
       <x:c r="G45" s="29" t="str">
         <x:v>Conditional target</x:v>
       </x:c>
-      <x:c r="H45" s="36" t="str">
+      <x:c r="H45" s="196" t="str">
         <x:v>Applied cohort by cohort</x:v>
       </x:c>
     </x:row>
@@ -4343,13 +4753,13 @@
       <x:c r="E46" s="29" t="str">
         <x:v>% subscription</x:v>
       </x:c>
-      <x:c r="F46" s="29" t="str">
+      <x:c r="F46" s="191" t="str">
         <x:v>Conservative assumption</x:v>
       </x:c>
       <x:c r="G46" s="29" t="str">
         <x:v>Evidence gated</x:v>
       </x:c>
-      <x:c r="H46" s="36" t="str">
+      <x:c r="H46" s="196" t="str">
         <x:v>No uplift before observed overages</x:v>
       </x:c>
     </x:row>
@@ -4369,13 +4779,13 @@
       <x:c r="E47" s="29" t="str">
         <x:v>$/new workspace</x:v>
       </x:c>
-      <x:c r="F47" s="29" t="str">
+      <x:c r="F47" s="191" t="str">
         <x:v>Management decision</x:v>
       </x:c>
       <x:c r="G47" s="29" t="str">
         <x:v>Market anchored</x:v>
       </x:c>
-      <x:c r="H47" s="36" t="str">
+      <x:c r="H47" s="196" t="str">
         <x:v>Gross new workspaces only</x:v>
       </x:c>
     </x:row>
@@ -4395,13 +4805,13 @@
       <x:c r="E48" s="29" t="str">
         <x:v>$/new contract</x:v>
       </x:c>
-      <x:c r="F48" s="29" t="str">
+      <x:c r="F48" s="191" t="str">
         <x:v>Management decision</x:v>
       </x:c>
       <x:c r="G48" s="29" t="str">
         <x:v>Pipeline gated</x:v>
       </x:c>
-      <x:c r="H48" s="36" t="str">
+      <x:c r="H48" s="196" t="str">
         <x:v>Integration and security scope</x:v>
       </x:c>
     </x:row>
@@ -4421,13 +4831,13 @@
       <x:c r="E49" s="29" t="str">
         <x:v>% revenue</x:v>
       </x:c>
-      <x:c r="F49" s="29" t="str">
+      <x:c r="F49" s="191" t="str">
         <x:v>Conservative benchmark</x:v>
       </x:c>
       <x:c r="G49" s="29" t="str">
         <x:v>Model assumption</x:v>
       </x:c>
-      <x:c r="H49" s="36" t="str">
+      <x:c r="H49" s="196" t="str">
         <x:v>AI, hosting and direct support</x:v>
       </x:c>
     </x:row>
@@ -4447,13 +4857,13 @@
       <x:c r="E50" s="29" t="str">
         <x:v>% revenue</x:v>
       </x:c>
-      <x:c r="F50" s="29" t="str">
+      <x:c r="F50" s="191" t="str">
         <x:v>Planning assumption</x:v>
       </x:c>
       <x:c r="G50" s="29" t="str">
         <x:v>Model assumption</x:v>
       </x:c>
-      <x:c r="H50" s="36" t="str">
+      <x:c r="H50" s="196" t="str">
         <x:v>Usage-layer margin</x:v>
       </x:c>
     </x:row>
@@ -4473,13 +4883,13 @@
       <x:c r="E51" s="29" t="str">
         <x:v>% revenue</x:v>
       </x:c>
-      <x:c r="F51" s="29" t="str">
+      <x:c r="F51" s="191" t="str">
         <x:v>Industry benchmark</x:v>
       </x:c>
       <x:c r="G51" s="29" t="str">
         <x:v>Benchmark anchored</x:v>
       </x:c>
-      <x:c r="H51" s="36" t="str">
+      <x:c r="H51" s="196" t="str">
         <x:v>Professional services at 30% gross margin</x:v>
       </x:c>
     </x:row>
@@ -4489,9 +4899,9 @@
       <x:c r="C52" s="32"/>
       <x:c r="D52" s="32"/>
       <x:c r="E52" s="29"/>
-      <x:c r="F52" s="29"/>
+      <x:c r="F52" s="193"/>
       <x:c r="G52" s="29"/>
-      <x:c r="H52" s="36"/>
+      <x:c r="H52" s="197"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4499,7 +4909,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabf7071656294ef5"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fce820a502f49a5"/>
 </x:worksheet>
 </file>
 
@@ -4520,7 +4930,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>Customer Cohort Bridge</x:v>
+        <x:v>Calculation Schedule · Cohort Bridge</x:v>
       </x:c>
       <x:c r="B1" s="19" t="str">
         <x:v>Customer Cohort Bridge</x:v>
@@ -4549,7 +4959,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>Beta exit cohorts roll into Commercial Year 1; ending customers equal retained prior cohorts plus new cohorts.</x:v>
+        <x:v>Supporting schedule for Beta carry-forward and retained opening cohorts</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>Beta exit cohorts roll into Commercial Year 1; ending customers equal retained prior cohorts plus new cohorts.</x:v>
@@ -4991,7 +5401,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>MIMAR Core — Monthly Commercial Cohort Build</x:v>
+        <x:v>Calculation Schedule · MIMAR Core</x:v>
       </x:c>
       <x:c r="B1" s="19" t="str">
         <x:v>MIMAR Core — Monthly Commercial Cohort Build</x:v>
@@ -5056,7 +5466,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>May 2027–Apr 2030. Beta carry is tracked separately from commercial acquisition and renews on its original contract dates.</x:v>
+        <x:v>Monthly cohort engine supporting the annual Core forecast</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>May 2027–Apr 2030. Beta carry is tracked separately from commercial acquisition and renews on its original contract dates.</x:v>
@@ -8197,7 +8607,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>MIMAR Engage — Monthly Commercial Cohort Build</x:v>
+        <x:v>Calculation Schedule · MIMAR Engage</x:v>
       </x:c>
       <x:c r="B1" s="19" t="str">
         <x:v>MIMAR Engage — Monthly Commercial Cohort Build</x:v>
@@ -8262,7 +8672,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>MIMAR Engage begins at commercial GA; retained workspaces and gross new cohorts are shown separately from onboarding.</x:v>
+        <x:v>Monthly cohort engine supporting the annual Engage forecast</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>MIMAR Engage begins at commercial GA; retained workspaces and gross new cohorts are shown separately from onboarding.</x:v>
@@ -11436,7 +11846,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>Scenario View — Beta + Commercial Cohort Underwriting</x:v>
+        <x:v>Scenario Summary</x:v>
       </x:c>
       <x:c r="B1" s="19" t="str">
         <x:v>Scenario View — Beta + Commercial Cohort Underwriting</x:v>
@@ -11492,7 +11902,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>Each scenario changes Beta attainment, commercial acquisition and retention, then recomputes every revenue stream.</x:v>
+        <x:v>Four revenue cases and the acquisition and retention assumptions that drive them</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>Each scenario changes Beta attainment, commercial acquisition and retention, then recomputes every revenue stream.</x:v>
@@ -11920,946 +12330,946 @@
       <x:c r="Q14" s="29"/>
       <x:c r="R14" s="29"/>
     </x:row>
-    <x:row r="15" ht="27" customHeight="1">
-      <x:c r="A15" s="22" t="str">
+    <x:row r="15" ht="2" customHeight="1">
+      <x:c r="A15" s="215" t="str">
         <x:v>Scenario</x:v>
       </x:c>
-      <x:c r="B15" s="22" t="str">
+      <x:c r="B15" s="216" t="str">
         <x:v>Year</x:v>
       </x:c>
-      <x:c r="C15" s="22" t="str">
+      <x:c r="C15" s="216" t="str">
         <x:v>Beta attainment</x:v>
       </x:c>
-      <x:c r="D15" s="22" t="str">
+      <x:c r="D15" s="216" t="str">
         <x:v>Acq. multiplier</x:v>
       </x:c>
-      <x:c r="E15" s="22" t="str">
+      <x:c r="E15" s="216" t="str">
         <x:v>Ind. retention</x:v>
       </x:c>
-      <x:c r="F15" s="22" t="str">
+      <x:c r="F15" s="216" t="str">
         <x:v>B2B retention</x:v>
       </x:c>
-      <x:c r="G15" s="22" t="str">
+      <x:c r="G15" s="216" t="str">
         <x:v>API retention</x:v>
       </x:c>
-      <x:c r="H15" s="22" t="str">
+      <x:c r="H15" s="216" t="str">
         <x:v>Beta carry</x:v>
       </x:c>
-      <x:c r="I15" s="22" t="str">
+      <x:c r="I15" s="216" t="str">
         <x:v>Individuals</x:v>
       </x:c>
-      <x:c r="J15" s="22" t="str">
+      <x:c r="J15" s="216" t="str">
         <x:v>Team seats</x:v>
       </x:c>
-      <x:c r="K15" s="22" t="str">
+      <x:c r="K15" s="216" t="str">
         <x:v>Enterprise</x:v>
       </x:c>
-      <x:c r="L15" s="22" t="str">
+      <x:c r="L15" s="216" t="str">
         <x:v>API</x:v>
       </x:c>
-      <x:c r="M15" s="22" t="str">
+      <x:c r="M15" s="216" t="str">
         <x:v>Core onboarding</x:v>
       </x:c>
-      <x:c r="N15" s="22" t="str">
+      <x:c r="N15" s="216" t="str">
         <x:v>CORE TOTAL</x:v>
       </x:c>
-      <x:c r="O15" s="22" t="str">
+      <x:c r="O15" s="216" t="str">
         <x:v>Engage subs</x:v>
       </x:c>
-      <x:c r="P15" s="22" t="str">
+      <x:c r="P15" s="216" t="str">
         <x:v>Usage</x:v>
       </x:c>
-      <x:c r="Q15" s="22" t="str">
+      <x:c r="Q15" s="216" t="str">
         <x:v>Engage onboarding</x:v>
       </x:c>
-      <x:c r="R15" s="22" t="str">
+      <x:c r="R15" s="217" t="str">
         <x:v>TOTAL MIMAR</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+    <x:row r="16" ht="2" customHeight="1">
+      <x:c r="A16" s="141" t="str">
         <x:f>$A$11</x:f>
         <x:v>Conservative</x:v>
       </x:c>
-      <x:c r="B16" s="29" t="n">
+      <x:c r="B16" s="143" t="n">
         <x:f>1</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C16" s="67" t="n">
+      <x:c r="C16" s="218" t="n">
         <x:f>$B$11</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="D16" s="67" t="n">
+      <x:c r="D16" s="218" t="n">
         <x:f>$C$11</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="E16" s="67" t="n">
+      <x:c r="E16" s="218" t="n">
         <x:f>$F$11</x:f>
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="F16" s="67" t="n">
+      <x:c r="F16" s="218" t="n">
         <x:f>$G$11</x:f>
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="G16" s="67" t="n">
+      <x:c r="G16" s="218" t="n">
         <x:f>$H$11</x:f>
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="H16" s="62" t="n">
+      <x:c r="H16" s="142" t="n">
         <x:f>$C16*(('Assumptions'!$B$8*(6*$E16^0+6*$E16^1)+'Assumptions'!$B$9*(10*$E16^0+2*$E16^1))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F16^0+6*$F16^1)+'Assumptions'!$B$12*(10*$F16^0+2*$F16^1))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>4298.7</x:v>
       </x:c>
-      <x:c r="I16" s="62" t="n">
+      <x:c r="I16" s="142" t="n">
         <x:f>('Assumptions'!$B$20*$D16*6.5)*'Assumptions'!$B$22</x:f>
         <x:v>7280</x:v>
       </x:c>
-      <x:c r="J16" s="62" t="n">
+      <x:c r="J16" s="142" t="n">
         <x:f>'Assumptions'!$B$23*$D16*6.5*'Assumptions'!$B$25*'Assumptions'!$B$26</x:f>
         <x:v>14560</x:v>
       </x:c>
-      <x:c r="K16" s="62" t="n">
+      <x:c r="K16" s="142" t="n">
         <x:f>'Assumptions'!$B$27*$D16*6.5/12*'Assumptions'!$B$28</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L16" s="62" t="n">
+      <x:c r="L16" s="142" t="n">
         <x:f>'Assumptions'!$B$29*$D16*6.5*'Assumptions'!$B$31</x:f>
         <x:v>2730</x:v>
       </x:c>
-      <x:c r="M16" s="62" t="n">
+      <x:c r="M16" s="142" t="n">
         <x:f>('Assumptions'!$B$23+'Assumptions'!$B$27)*$D16*'Assumptions'!$B$32</x:f>
         <x:v>14000</x:v>
       </x:c>
-      <x:c r="N16" s="62" t="n">
+      <x:c r="N16" s="142" t="n">
         <x:f>SUM(H16:M16)</x:f>
         <x:v>42868.7</x:v>
       </x:c>
-      <x:c r="O16" s="62" t="n">
+      <x:c r="O16" s="142" t="n">
         <x:f>'Assumptions'!$B$37*$D16*6.5*'Assumptions'!$B$38+'Assumptions'!$B$39*$D16*6.5*'Assumptions'!$B$40+'Assumptions'!$B$41*$D16*6.5*'Assumptions'!$B$42+'Assumptions'!$B$43*$D16*6.5*'Assumptions'!$B$44</x:f>
         <x:v>28528.499999999996</x:v>
       </x:c>
-      <x:c r="P16" s="62" t="n">
+      <x:c r="P16" s="142" t="n">
         <x:f>O16*'Assumptions'!$B$46</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q16" s="62" t="n">
+      <x:c r="Q16" s="142" t="n">
         <x:f>(('Assumptions'!$B$37+'Assumptions'!$B$39+'Assumptions'!$B$41)*'Assumptions'!$B$47+'Assumptions'!$B$43*'Assumptions'!$B$48)*$D16</x:f>
         <x:v>12600</x:v>
       </x:c>
-      <x:c r="R16" s="62" t="n">
+      <x:c r="R16" s="144" t="n">
         <x:f>N16+O16+P16+Q16</x:f>
         <x:v>83997.2</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+    <x:row r="17" ht="2" customHeight="1">
+      <x:c r="A17" s="141" t="str">
         <x:f>$A$11</x:f>
         <x:v>Conservative</x:v>
       </x:c>
-      <x:c r="B17" s="29" t="n">
+      <x:c r="B17" s="143" t="n">
         <x:f>2</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C17" s="67" t="n">
+      <x:c r="C17" s="218" t="n">
         <x:f>$B$11</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="D17" s="67" t="n">
+      <x:c r="D17" s="218" t="n">
         <x:f>$D$11</x:f>
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="E17" s="67" t="n">
+      <x:c r="E17" s="218" t="n">
         <x:f>$F$11</x:f>
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="F17" s="67" t="n">
+      <x:c r="F17" s="218" t="n">
         <x:f>$G$11</x:f>
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="G17" s="67" t="n">
+      <x:c r="G17" s="218" t="n">
         <x:f>$H$11</x:f>
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="H17" s="62" t="n">
+      <x:c r="H17" s="142" t="n">
         <x:f>$C17*(('Assumptions'!$B$8*(6*$E17^1+6*$E17^2)+'Assumptions'!$B$9*(10*$E17^1+2*$E17^2))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F17^1+6*$F17^2)+'Assumptions'!$B$12*(10*$F17^1+2*$F17^2))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>2421.5099999999998</x:v>
       </x:c>
-      <x:c r="I17" s="62" t="n">
+      <x:c r="I17" s="142" t="n">
         <x:f>('Assumptions'!$B$20*$D16*$E17*12+'Assumptions'!$C$20*$D17*6.5)*'Assumptions'!$C$22</x:f>
         <x:v>30960</x:v>
       </x:c>
-      <x:c r="J17" s="62" t="n">
+      <x:c r="J17" s="142" t="n">
         <x:f>('Assumptions'!$B$23*$D16*$F17*12+'Assumptions'!$C$23*$D17*6.5)*'Assumptions'!$C$25*'Assumptions'!$C$26</x:f>
         <x:v>57499.2</x:v>
       </x:c>
-      <x:c r="K17" s="62" t="n">
+      <x:c r="K17" s="142" t="n">
         <x:f>('Assumptions'!$B$27*$D16*$F17*12+'Assumptions'!$C$27*$D17*6.5)/12*'Assumptions'!$C$28</x:f>
         <x:v>8666.666666666666</x:v>
       </x:c>
-      <x:c r="L17" s="62" t="n">
+      <x:c r="L17" s="142" t="n">
         <x:f>('Assumptions'!$B$29*$D16*$G17*12+'Assumptions'!$C$29*$D17*6.5)*'Assumptions'!$C$31</x:f>
         <x:v>16236</x:v>
       </x:c>
-      <x:c r="M17" s="62" t="n">
+      <x:c r="M17" s="142" t="n">
         <x:f>('Assumptions'!$C$23+'Assumptions'!$C$27)*$D17*'Assumptions'!$C$32</x:f>
         <x:v>22320</x:v>
       </x:c>
-      <x:c r="N17" s="62" t="n">
+      <x:c r="N17" s="142" t="n">
         <x:f>SUM(H17:M17)</x:f>
         <x:v>138103.37666666665</x:v>
       </x:c>
-      <x:c r="O17" s="62" t="n">
+      <x:c r="O17" s="142" t="n">
         <x:f>('Assumptions'!$B$37*$D16*$F17*12+'Assumptions'!$C$37*$D17*6.5)*'Assumptions'!$C$38+('Assumptions'!$B$39*$D16*$F17*12+'Assumptions'!$C$39*$D17*6.5)*'Assumptions'!$C$40+('Assumptions'!$B$41*$D16*$F17*12+'Assumptions'!$C$41*$D17*6.5)*'Assumptions'!$C$42+('Assumptions'!$B$43*$D16*$F17*12+'Assumptions'!$C$43*$D17*6.5)*'Assumptions'!$C$44</x:f>
         <x:v>105574.4</x:v>
       </x:c>
-      <x:c r="P17" s="62" t="n">
+      <x:c r="P17" s="142" t="n">
         <x:f>O17*'Assumptions'!$C$46</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q17" s="62" t="n">
+      <x:c r="Q17" s="142" t="n">
         <x:f>(('Assumptions'!$C$37+'Assumptions'!$C$39+'Assumptions'!$C$41)*'Assumptions'!$C$47+'Assumptions'!$C$43*'Assumptions'!$C$48)*$D17</x:f>
         <x:v>23200</x:v>
       </x:c>
-      <x:c r="R17" s="62" t="n">
+      <x:c r="R17" s="144" t="n">
         <x:f>N17+O17+P17+Q17</x:f>
         <x:v>266877.7766666666</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+    <x:row r="18" ht="2" customHeight="1">
+      <x:c r="A18" s="141" t="str">
         <x:f>$A$11</x:f>
         <x:v>Conservative</x:v>
       </x:c>
-      <x:c r="B18" s="29" t="n">
+      <x:c r="B18" s="143" t="n">
         <x:f>3</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C18" s="67" t="n">
+      <x:c r="C18" s="218" t="n">
         <x:f>$B$11</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="D18" s="67" t="n">
+      <x:c r="D18" s="218" t="n">
         <x:f>$E$11</x:f>
         <x:v>0.85</x:v>
       </x:c>
-      <x:c r="E18" s="67" t="n">
+      <x:c r="E18" s="218" t="n">
         <x:f>$F$11</x:f>
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="F18" s="67" t="n">
+      <x:c r="F18" s="218" t="n">
         <x:f>$G$11</x:f>
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="G18" s="67" t="n">
+      <x:c r="G18" s="218" t="n">
         <x:f>$H$11</x:f>
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="H18" s="62" t="n">
+      <x:c r="H18" s="142" t="n">
         <x:f>$C18*(('Assumptions'!$B$8*(6*$E18^2+6*$E18^3)+'Assumptions'!$B$9*(10*$E18^2+2*$E18^3))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F18^2+6*$F18^3)+'Assumptions'!$B$12*(10*$F18^2+2*$F18^3))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>1428.483</x:v>
       </x:c>
-      <x:c r="I18" s="62" t="n">
+      <x:c r="I18" s="142" t="n">
         <x:f>('Assumptions'!$B$20*$D16*$E18^2*12+'Assumptions'!$C$20*$D17*$E18*12+'Assumptions'!$D$20*$D18*6.5)*'Assumptions'!$D$22</x:f>
         <x:v>83450</x:v>
       </x:c>
-      <x:c r="J18" s="62" t="n">
+      <x:c r="J18" s="142" t="n">
         <x:f>('Assumptions'!$B$23*$D16*$F18^2*12+'Assumptions'!$C$23*$D17*$F18*12+'Assumptions'!$D$23*$D18*6.5)*'Assumptions'!$D$25*'Assumptions'!$D$26</x:f>
         <x:v>160660.80000000002</x:v>
       </x:c>
-      <x:c r="K18" s="62" t="n">
+      <x:c r="K18" s="142" t="n">
         <x:f>('Assumptions'!$B$27*$D16*$F18^2*12+'Assumptions'!$C$27*$D17*$F18*12+'Assumptions'!$D$27*$D18*6.5)/12*'Assumptions'!$D$28</x:f>
         <x:v>44467.50000000001</x:v>
       </x:c>
-      <x:c r="L18" s="62" t="n">
+      <x:c r="L18" s="142" t="n">
         <x:f>('Assumptions'!$B$29*$D16*$G18^2*12+'Assumptions'!$C$29*$D17*$G18*12+'Assumptions'!$D$29*$D18*6.5)*'Assumptions'!$D$31</x:f>
         <x:v>60688.8</x:v>
       </x:c>
-      <x:c r="M18" s="62" t="n">
+      <x:c r="M18" s="142" t="n">
         <x:f>('Assumptions'!$D$23+'Assumptions'!$D$27)*$D18*'Assumptions'!$D$32</x:f>
         <x:v>40162.5</x:v>
       </x:c>
-      <x:c r="N18" s="62" t="n">
+      <x:c r="N18" s="142" t="n">
         <x:f>SUM(H18:M18)</x:f>
         <x:v>390858.083</x:v>
       </x:c>
-      <x:c r="O18" s="62" t="n">
+      <x:c r="O18" s="142" t="n">
         <x:f>('Assumptions'!$B$37*$D16*$F18^2*12+'Assumptions'!$C$37*$D17*$F18*12+'Assumptions'!$D$37*$D18*6.5)*'Assumptions'!$D$38+('Assumptions'!$B$39*$D16*$F18^2*12+'Assumptions'!$C$39*$D17*$F18*12+'Assumptions'!$D$39*$D18*6.5)*'Assumptions'!$D$40+('Assumptions'!$B$41*$D16*$F18^2*12+'Assumptions'!$C$41*$D17*$F18*12+'Assumptions'!$D$41*$D18*6.5)*'Assumptions'!$D$42+('Assumptions'!$B$43*$D16*$F18^2*12+'Assumptions'!$C$43*$D17*$F18*12+'Assumptions'!$D$43*$D18*6.5)*'Assumptions'!$D$44</x:f>
         <x:v>277119.97</x:v>
       </x:c>
-      <x:c r="P18" s="62" t="n">
+      <x:c r="P18" s="142" t="n">
         <x:f>O18*'Assumptions'!$D$46</x:f>
         <x:v>8313.5991</x:v>
       </x:c>
-      <x:c r="Q18" s="62" t="n">
+      <x:c r="Q18" s="142" t="n">
         <x:f>(('Assumptions'!$D$37+'Assumptions'!$D$39+'Assumptions'!$D$41)*'Assumptions'!$D$47+'Assumptions'!$D$43*'Assumptions'!$D$48)*$D18</x:f>
         <x:v>43180</x:v>
       </x:c>
-      <x:c r="R18" s="62" t="n">
+      <x:c r="R18" s="144" t="n">
         <x:f>N18+O18+P18+Q18</x:f>
         <x:v>719471.6521</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+    <x:row r="19" ht="2" customHeight="1">
+      <x:c r="A19" s="141" t="str">
         <x:f>$A$12</x:f>
         <x:v>Base</x:v>
       </x:c>
-      <x:c r="B19" s="29" t="n">
+      <x:c r="B19" s="143" t="n">
         <x:f>1</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C19" s="67" t="n">
+      <x:c r="C19" s="218" t="n">
         <x:f>$B$12</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D19" s="67" t="n">
+      <x:c r="D19" s="218" t="n">
         <x:f>$C$12</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E19" s="67" t="n">
+      <x:c r="E19" s="218" t="n">
         <x:f>$F$12</x:f>
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="F19" s="67" t="n">
+      <x:c r="F19" s="218" t="n">
         <x:f>$G$12</x:f>
         <x:v>0.9</x:v>
       </x:c>
-      <x:c r="G19" s="67" t="n">
+      <x:c r="G19" s="218" t="n">
         <x:f>$H$12</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="H19" s="62" t="n">
+      <x:c r="H19" s="142" t="n">
         <x:f>$C19*(('Assumptions'!$B$8*(6*$E19^0+6*$E19^1)+'Assumptions'!$B$9*(10*$E19^0+2*$E19^1))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F19^0+6*$F19^1)+'Assumptions'!$B$12*(10*$F19^0+2*$F19^1))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>6383.999999999999</x:v>
       </x:c>
-      <x:c r="I19" s="62" t="n">
+      <x:c r="I19" s="142" t="n">
         <x:f>('Assumptions'!$B$20*$D19*6.5)*'Assumptions'!$B$22</x:f>
         <x:v>10400</x:v>
       </x:c>
-      <x:c r="J19" s="62" t="n">
+      <x:c r="J19" s="142" t="n">
         <x:f>'Assumptions'!$B$23*$D19*6.5*'Assumptions'!$B$25*'Assumptions'!$B$26</x:f>
         <x:v>20800</x:v>
       </x:c>
-      <x:c r="K19" s="62" t="n">
+      <x:c r="K19" s="142" t="n">
         <x:f>'Assumptions'!$B$27*$D19*6.5/12*'Assumptions'!$B$28</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L19" s="62" t="n">
+      <x:c r="L19" s="142" t="n">
         <x:f>'Assumptions'!$B$29*$D19*6.5*'Assumptions'!$B$31</x:f>
         <x:v>3900</x:v>
       </x:c>
-      <x:c r="M19" s="62" t="n">
+      <x:c r="M19" s="142" t="n">
         <x:f>('Assumptions'!$B$23+'Assumptions'!$B$27)*$D19*'Assumptions'!$B$32</x:f>
         <x:v>20000</x:v>
       </x:c>
-      <x:c r="N19" s="62" t="n">
+      <x:c r="N19" s="142" t="n">
         <x:f>SUM(H19:M19)</x:f>
         <x:v>61484</x:v>
       </x:c>
-      <x:c r="O19" s="62" t="n">
+      <x:c r="O19" s="142" t="n">
         <x:f>'Assumptions'!$B$37*$D19*6.5*'Assumptions'!$B$38+'Assumptions'!$B$39*$D19*6.5*'Assumptions'!$B$40+'Assumptions'!$B$41*$D19*6.5*'Assumptions'!$B$42+'Assumptions'!$B$43*$D19*6.5*'Assumptions'!$B$44</x:f>
         <x:v>40755</x:v>
       </x:c>
-      <x:c r="P19" s="62" t="n">
+      <x:c r="P19" s="142" t="n">
         <x:f>O19*'Assumptions'!$B$46</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q19" s="62" t="n">
+      <x:c r="Q19" s="142" t="n">
         <x:f>(('Assumptions'!$B$37+'Assumptions'!$B$39+'Assumptions'!$B$41)*'Assumptions'!$B$47+'Assumptions'!$B$43*'Assumptions'!$B$48)*$D19</x:f>
         <x:v>18000</x:v>
       </x:c>
-      <x:c r="R19" s="62" t="n">
+      <x:c r="R19" s="144" t="n">
         <x:f>N19+O19+P19+Q19</x:f>
         <x:v>120239</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="29" t="str">
+    <x:row r="20" ht="2" customHeight="1">
+      <x:c r="A20" s="141" t="str">
         <x:f>$A$12</x:f>
         <x:v>Base</x:v>
       </x:c>
-      <x:c r="B20" s="29" t="n">
+      <x:c r="B20" s="143" t="n">
         <x:f>2</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C20" s="67" t="n">
+      <x:c r="C20" s="218" t="n">
         <x:f>$B$12</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D20" s="67" t="n">
+      <x:c r="D20" s="218" t="n">
         <x:f>$D$12</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E20" s="67" t="n">
+      <x:c r="E20" s="218" t="n">
         <x:f>$F$12</x:f>
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="F20" s="67" t="n">
+      <x:c r="F20" s="218" t="n">
         <x:f>$G$12</x:f>
         <x:v>0.9</x:v>
       </x:c>
-      <x:c r="G20" s="67" t="n">
+      <x:c r="G20" s="218" t="n">
         <x:f>$H$12</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="H20" s="62" t="n">
+      <x:c r="H20" s="142" t="n">
         <x:f>$C20*(('Assumptions'!$B$8*(6*$E20^1+6*$E20^2)+'Assumptions'!$B$9*(10*$E20^1+2*$E20^2))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F20^1+6*$F20^2)+'Assumptions'!$B$12*(10*$F20^1+2*$F20^2))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>4240.8</x:v>
       </x:c>
-      <x:c r="I20" s="62" t="n">
+      <x:c r="I20" s="142" t="n">
         <x:f>('Assumptions'!$B$20*$D19*$E20*12+'Assumptions'!$C$20*$D20*6.5)*'Assumptions'!$C$22</x:f>
         <x:v>42210</x:v>
       </x:c>
-      <x:c r="J20" s="62" t="n">
+      <x:c r="J20" s="142" t="n">
         <x:f>('Assumptions'!$B$23*$D19*$F20*12+'Assumptions'!$C$23*$D20*6.5)*'Assumptions'!$C$25*'Assumptions'!$C$26</x:f>
         <x:v>81378</x:v>
       </x:c>
-      <x:c r="K20" s="62" t="n">
+      <x:c r="K20" s="142" t="n">
         <x:f>('Assumptions'!$B$27*$D19*$F20*12+'Assumptions'!$C$27*$D20*6.5)/12*'Assumptions'!$C$28</x:f>
         <x:v>10833.333333333332</x:v>
       </x:c>
-      <x:c r="L20" s="62" t="n">
+      <x:c r="L20" s="142" t="n">
         <x:f>('Assumptions'!$B$29*$D19*$G20*12+'Assumptions'!$C$29*$D20*6.5)*'Assumptions'!$C$31</x:f>
         <x:v>22185</x:v>
       </x:c>
-      <x:c r="M20" s="62" t="n">
+      <x:c r="M20" s="142" t="n">
         <x:f>('Assumptions'!$C$23+'Assumptions'!$C$27)*$D20*'Assumptions'!$C$32</x:f>
         <x:v>27900</x:v>
       </x:c>
-      <x:c r="N20" s="62" t="n">
+      <x:c r="N20" s="142" t="n">
         <x:f>SUM(H20:M20)</x:f>
         <x:v>188747.13333333333</x:v>
       </x:c>
-      <x:c r="O20" s="62" t="n">
+      <x:c r="O20" s="142" t="n">
         <x:f>('Assumptions'!$B$37*$D19*$F20*12+'Assumptions'!$C$37*$D20*6.5)*'Assumptions'!$C$38+('Assumptions'!$B$39*$D19*$F20*12+'Assumptions'!$C$39*$D20*6.5)*'Assumptions'!$C$40+('Assumptions'!$B$41*$D19*$F20*12+'Assumptions'!$C$41*$D20*6.5)*'Assumptions'!$C$42+('Assumptions'!$B$43*$D19*$F20*12+'Assumptions'!$C$43*$D20*6.5)*'Assumptions'!$C$44</x:f>
         <x:v>147016</x:v>
       </x:c>
-      <x:c r="P20" s="62" t="n">
+      <x:c r="P20" s="142" t="n">
         <x:f>O20*'Assumptions'!$C$46</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q20" s="62" t="n">
+      <x:c r="Q20" s="142" t="n">
         <x:f>(('Assumptions'!$C$37+'Assumptions'!$C$39+'Assumptions'!$C$41)*'Assumptions'!$C$47+'Assumptions'!$C$43*'Assumptions'!$C$48)*$D20</x:f>
         <x:v>29000</x:v>
       </x:c>
-      <x:c r="R20" s="62" t="n">
+      <x:c r="R20" s="144" t="n">
         <x:f>N20+O20+P20+Q20</x:f>
         <x:v>364763.1333333333</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="29" t="str">
+    <x:row r="21" ht="2" customHeight="1">
+      <x:c r="A21" s="141" t="str">
         <x:f>$A$12</x:f>
         <x:v>Base</x:v>
       </x:c>
-      <x:c r="B21" s="29" t="n">
+      <x:c r="B21" s="143" t="n">
         <x:f>3</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C21" s="67" t="n">
+      <x:c r="C21" s="218" t="n">
         <x:f>$B$12</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D21" s="67" t="n">
+      <x:c r="D21" s="218" t="n">
         <x:f>$E$12</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E21" s="67" t="n">
+      <x:c r="E21" s="218" t="n">
         <x:f>$F$12</x:f>
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="F21" s="67" t="n">
+      <x:c r="F21" s="218" t="n">
         <x:f>$G$12</x:f>
         <x:v>0.9</x:v>
       </x:c>
-      <x:c r="G21" s="67" t="n">
+      <x:c r="G21" s="218" t="n">
         <x:f>$H$12</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="H21" s="62" t="n">
+      <x:c r="H21" s="142" t="n">
         <x:f>$C21*(('Assumptions'!$B$8*(6*$E21^2+6*$E21^3)+'Assumptions'!$B$9*(10*$E21^2+2*$E21^3))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F21^2+6*$F21^3)+'Assumptions'!$B$12*(10*$F21^2+2*$F21^3))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>2913.84</x:v>
       </x:c>
-      <x:c r="I21" s="62" t="n">
+      <x:c r="I21" s="142" t="n">
         <x:f>('Assumptions'!$B$20*$D19*$E21^2*12+'Assumptions'!$C$20*$D20*$E21*12+'Assumptions'!$D$20*$D21*6.5)*'Assumptions'!$D$22</x:f>
         <x:v>109640</x:v>
       </x:c>
-      <x:c r="J21" s="62" t="n">
+      <x:c r="J21" s="142" t="n">
         <x:f>('Assumptions'!$B$23*$D19*$F21^2*12+'Assumptions'!$C$23*$D20*$F21*12+'Assumptions'!$D$23*$D21*6.5)*'Assumptions'!$D$25*'Assumptions'!$D$26</x:f>
         <x:v>218016</x:v>
       </x:c>
-      <x:c r="K21" s="62" t="n">
+      <x:c r="K21" s="142" t="n">
         <x:f>('Assumptions'!$B$27*$D19*$F21^2*12+'Assumptions'!$C$27*$D20*$F21*12+'Assumptions'!$D$27*$D21*6.5)/12*'Assumptions'!$D$28</x:f>
         <x:v>55550</x:v>
       </x:c>
-      <x:c r="L21" s="62" t="n">
+      <x:c r="L21" s="142" t="n">
         <x:f>('Assumptions'!$B$29*$D19*$G21^2*12+'Assumptions'!$C$29*$D20*$G21*12+'Assumptions'!$D$29*$D21*6.5)*'Assumptions'!$D$31</x:f>
         <x:v>79056</x:v>
       </x:c>
-      <x:c r="M21" s="62" t="n">
+      <x:c r="M21" s="142" t="n">
         <x:f>('Assumptions'!$D$23+'Assumptions'!$D$27)*$D21*'Assumptions'!$D$32</x:f>
         <x:v>47250</x:v>
       </x:c>
-      <x:c r="N21" s="62" t="n">
+      <x:c r="N21" s="142" t="n">
         <x:f>SUM(H21:M21)</x:f>
         <x:v>512425.83999999997</x:v>
       </x:c>
-      <x:c r="O21" s="62" t="n">
+      <x:c r="O21" s="142" t="n">
         <x:f>('Assumptions'!$B$37*$D19*$F21^2*12+'Assumptions'!$C$37*$D20*$F21*12+'Assumptions'!$D$37*$D21*6.5)*'Assumptions'!$D$38+('Assumptions'!$B$39*$D19*$F21^2*12+'Assumptions'!$C$39*$D20*$F21*12+'Assumptions'!$D$39*$D21*6.5)*'Assumptions'!$D$40+('Assumptions'!$B$41*$D19*$F21^2*12+'Assumptions'!$C$41*$D20*$F21*12+'Assumptions'!$D$41*$D21*6.5)*'Assumptions'!$D$42+('Assumptions'!$B$43*$D19*$F21^2*12+'Assumptions'!$C$43*$D20*$F21*12+'Assumptions'!$D$43*$D21*6.5)*'Assumptions'!$D$44</x:f>
         <x:v>368841.4</x:v>
       </x:c>
-      <x:c r="P21" s="62" t="n">
+      <x:c r="P21" s="142" t="n">
         <x:f>O21*'Assumptions'!$D$46</x:f>
         <x:v>11065.242</x:v>
       </x:c>
-      <x:c r="Q21" s="62" t="n">
+      <x:c r="Q21" s="142" t="n">
         <x:f>(('Assumptions'!$D$37+'Assumptions'!$D$39+'Assumptions'!$D$41)*'Assumptions'!$D$47+'Assumptions'!$D$43*'Assumptions'!$D$48)*$D21</x:f>
         <x:v>50800</x:v>
       </x:c>
-      <x:c r="R21" s="62" t="n">
+      <x:c r="R21" s="144" t="n">
         <x:f>N21+O21+P21+Q21</x:f>
         <x:v>943132.482</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="29" t="str">
+    <x:row r="22" ht="2" customHeight="1">
+      <x:c r="A22" s="141" t="str">
         <x:f>$A$13</x:f>
         <x:v>Upside</x:v>
       </x:c>
-      <x:c r="B22" s="29" t="n">
+      <x:c r="B22" s="143" t="n">
         <x:f>1</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C22" s="67" t="n">
+      <x:c r="C22" s="218" t="n">
         <x:f>$B$13</x:f>
         <x:v>1.15</x:v>
       </x:c>
-      <x:c r="D22" s="67" t="n">
+      <x:c r="D22" s="218" t="n">
         <x:f>$C$13</x:f>
         <x:v>1.3</x:v>
       </x:c>
-      <x:c r="E22" s="67" t="n">
+      <x:c r="E22" s="218" t="n">
         <x:f>$F$13</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="F22" s="67" t="n">
+      <x:c r="F22" s="218" t="n">
         <x:f>$G$13</x:f>
         <x:v>0.93</x:v>
       </x:c>
-      <x:c r="G22" s="67" t="n">
+      <x:c r="G22" s="218" t="n">
         <x:f>$H$13</x:f>
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="H22" s="62" t="n">
+      <x:c r="H22" s="142" t="n">
         <x:f>$C22*(('Assumptions'!$B$8*(6*$E22^0+6*$E22^1)+'Assumptions'!$B$9*(10*$E22^0+2*$E22^1))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F22^0+6*$F22^1)+'Assumptions'!$B$12*(10*$F22^0+2*$F22^1))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>7563.090000000001</x:v>
       </x:c>
-      <x:c r="I22" s="62" t="n">
+      <x:c r="I22" s="142" t="n">
         <x:f>('Assumptions'!$B$20*$D22*6.5)*'Assumptions'!$B$22</x:f>
         <x:v>13520</x:v>
       </x:c>
-      <x:c r="J22" s="62" t="n">
+      <x:c r="J22" s="142" t="n">
         <x:f>'Assumptions'!$B$23*$D22*6.5*'Assumptions'!$B$25*'Assumptions'!$B$26</x:f>
         <x:v>27040</x:v>
       </x:c>
-      <x:c r="K22" s="62" t="n">
+      <x:c r="K22" s="142" t="n">
         <x:f>'Assumptions'!$B$27*$D22*6.5/12*'Assumptions'!$B$28</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L22" s="62" t="n">
+      <x:c r="L22" s="142" t="n">
         <x:f>'Assumptions'!$B$29*$D22*6.5*'Assumptions'!$B$31</x:f>
         <x:v>5070</x:v>
       </x:c>
-      <x:c r="M22" s="62" t="n">
+      <x:c r="M22" s="142" t="n">
         <x:f>('Assumptions'!$B$23+'Assumptions'!$B$27)*$D22*'Assumptions'!$B$32</x:f>
         <x:v>26000</x:v>
       </x:c>
-      <x:c r="N22" s="62" t="n">
+      <x:c r="N22" s="142" t="n">
         <x:f>SUM(H22:M22)</x:f>
         <x:v>79193.09</x:v>
       </x:c>
-      <x:c r="O22" s="62" t="n">
+      <x:c r="O22" s="142" t="n">
         <x:f>'Assumptions'!$B$37*$D22*6.5*'Assumptions'!$B$38+'Assumptions'!$B$39*$D22*6.5*'Assumptions'!$B$40+'Assumptions'!$B$41*$D22*6.5*'Assumptions'!$B$42+'Assumptions'!$B$43*$D22*6.5*'Assumptions'!$B$44</x:f>
         <x:v>52981.50000000001</x:v>
       </x:c>
-      <x:c r="P22" s="62" t="n">
+      <x:c r="P22" s="142" t="n">
         <x:f>O22*'Assumptions'!$B$46</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q22" s="62" t="n">
+      <x:c r="Q22" s="142" t="n">
         <x:f>(('Assumptions'!$B$37+'Assumptions'!$B$39+'Assumptions'!$B$41)*'Assumptions'!$B$47+'Assumptions'!$B$43*'Assumptions'!$B$48)*$D22</x:f>
         <x:v>23400</x:v>
       </x:c>
-      <x:c r="R22" s="62" t="n">
+      <x:c r="R22" s="144" t="n">
         <x:f>N22+O22+P22+Q22</x:f>
         <x:v>155574.59</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="29" t="str">
+    <x:row r="23" ht="2" customHeight="1">
+      <x:c r="A23" s="141" t="str">
         <x:f>$A$13</x:f>
         <x:v>Upside</x:v>
       </x:c>
-      <x:c r="B23" s="29" t="n">
+      <x:c r="B23" s="143" t="n">
         <x:f>2</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C23" s="67" t="n">
+      <x:c r="C23" s="218" t="n">
         <x:f>$B$13</x:f>
         <x:v>1.15</x:v>
       </x:c>
-      <x:c r="D23" s="67" t="n">
+      <x:c r="D23" s="218" t="n">
         <x:f>$D$13</x:f>
         <x:v>1.35</x:v>
       </x:c>
-      <x:c r="E23" s="67" t="n">
+      <x:c r="E23" s="218" t="n">
         <x:f>$F$13</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="F23" s="67" t="n">
+      <x:c r="F23" s="218" t="n">
         <x:f>$G$13</x:f>
         <x:v>0.93</x:v>
       </x:c>
-      <x:c r="G23" s="67" t="n">
+      <x:c r="G23" s="218" t="n">
         <x:f>$H$13</x:f>
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="H23" s="62" t="n">
+      <x:c r="H23" s="142" t="n">
         <x:f>$C23*(('Assumptions'!$B$8*(6*$E23^1+6*$E23^2)+'Assumptions'!$B$9*(10*$E23^1+2*$E23^2))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F23^1+6*$F23^2)+'Assumptions'!$B$12*(10*$F23^1+2*$F23^2))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>5661.712199999999</x:v>
       </x:c>
-      <x:c r="I23" s="62" t="n">
+      <x:c r="I23" s="142" t="n">
         <x:f>('Assumptions'!$B$20*$D22*$E23*12+'Assumptions'!$C$20*$D23*6.5)*'Assumptions'!$C$22</x:f>
         <x:v>59143.5</x:v>
       </x:c>
-      <x:c r="J23" s="62" t="n">
+      <x:c r="J23" s="142" t="n">
         <x:f>('Assumptions'!$B$23*$D22*$F23*12+'Assumptions'!$C$23*$D23*6.5)*'Assumptions'!$C$25*'Assumptions'!$C$26</x:f>
         <x:v>109575.18</x:v>
       </x:c>
-      <x:c r="K23" s="62" t="n">
+      <x:c r="K23" s="142" t="n">
         <x:f>('Assumptions'!$B$27*$D22*$F23*12+'Assumptions'!$C$27*$D23*6.5)/12*'Assumptions'!$C$28</x:f>
         <x:v>14625.000000000002</x:v>
       </x:c>
-      <x:c r="L23" s="62" t="n">
+      <x:c r="L23" s="142" t="n">
         <x:f>('Assumptions'!$B$29*$D22*$G23*12+'Assumptions'!$C$29*$D23*6.5)*'Assumptions'!$C$31</x:f>
         <x:v>30975.75</x:v>
       </x:c>
-      <x:c r="M23" s="62" t="n">
+      <x:c r="M23" s="142" t="n">
         <x:f>('Assumptions'!$C$23+'Assumptions'!$C$27)*$D23*'Assumptions'!$C$32</x:f>
         <x:v>37665</x:v>
       </x:c>
-      <x:c r="N23" s="62" t="n">
+      <x:c r="N23" s="142" t="n">
         <x:f>SUM(H23:M23)</x:f>
         <x:v>257646.1422</x:v>
       </x:c>
-      <x:c r="O23" s="62" t="n">
+      <x:c r="O23" s="142" t="n">
         <x:f>('Assumptions'!$B$37*$D22*$F23*12+'Assumptions'!$C$37*$D23*6.5)*'Assumptions'!$C$38+('Assumptions'!$B$39*$D22*$F23*12+'Assumptions'!$C$39*$D23*6.5)*'Assumptions'!$C$40+('Assumptions'!$B$41*$D22*$F23*12+'Assumptions'!$C$41*$D23*6.5)*'Assumptions'!$C$42+('Assumptions'!$B$43*$D22*$F23*12+'Assumptions'!$C$43*$D23*6.5)*'Assumptions'!$C$44</x:f>
         <x:v>198020.15999999997</x:v>
       </x:c>
-      <x:c r="P23" s="62" t="n">
+      <x:c r="P23" s="142" t="n">
         <x:f>O23*'Assumptions'!$C$46</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q23" s="62" t="n">
+      <x:c r="Q23" s="142" t="n">
         <x:f>(('Assumptions'!$C$37+'Assumptions'!$C$39+'Assumptions'!$C$41)*'Assumptions'!$C$47+'Assumptions'!$C$43*'Assumptions'!$C$48)*$D23</x:f>
         <x:v>39150</x:v>
       </x:c>
-      <x:c r="R23" s="62" t="n">
+      <x:c r="R23" s="144" t="n">
         <x:f>N23+O23+P23+Q23</x:f>
         <x:v>494816.3022</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="29" t="str">
+    <x:row r="24" ht="2" customHeight="1">
+      <x:c r="A24" s="141" t="str">
         <x:f>$A$13</x:f>
         <x:v>Upside</x:v>
       </x:c>
-      <x:c r="B24" s="29" t="n">
+      <x:c r="B24" s="143" t="n">
         <x:f>3</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C24" s="67" t="n">
+      <x:c r="C24" s="218" t="n">
         <x:f>$B$13</x:f>
         <x:v>1.15</x:v>
       </x:c>
-      <x:c r="D24" s="67" t="n">
+      <x:c r="D24" s="218" t="n">
         <x:f>$E$13</x:f>
         <x:v>1.4</x:v>
       </x:c>
-      <x:c r="E24" s="67" t="n">
+      <x:c r="E24" s="218" t="n">
         <x:f>$F$13</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="F24" s="67" t="n">
+      <x:c r="F24" s="218" t="n">
         <x:f>$G$13</x:f>
         <x:v>0.93</x:v>
       </x:c>
-      <x:c r="G24" s="67" t="n">
+      <x:c r="G24" s="218" t="n">
         <x:f>$H$13</x:f>
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="H24" s="62" t="n">
+      <x:c r="H24" s="142" t="n">
         <x:f>$C24*(('Assumptions'!$B$8*(6*$E24^2+6*$E24^3)+'Assumptions'!$B$9*(10*$E24^2+2*$E24^3))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F24^2+6*$F24^3)+'Assumptions'!$B$12*(10*$F24^2+2*$F24^3))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>4305.0192959999995</x:v>
       </x:c>
-      <x:c r="I24" s="62" t="n">
+      <x:c r="I24" s="142" t="n">
         <x:f>('Assumptions'!$B$20*$D22*$E24^2*12+'Assumptions'!$C$20*$D23*$E24*12+'Assumptions'!$D$20*$D24*6.5)*'Assumptions'!$D$22</x:f>
         <x:v>162988</x:v>
       </x:c>
-      <x:c r="J24" s="62" t="n">
+      <x:c r="J24" s="142" t="n">
         <x:f>('Assumptions'!$B$23*$D22*$F24^2*12+'Assumptions'!$C$23*$D23*$F24*12+'Assumptions'!$D$23*$D24*6.5)*'Assumptions'!$D$25*'Assumptions'!$D$26</x:f>
         <x:v>304278.912</x:v>
       </x:c>
-      <x:c r="K24" s="62" t="n">
+      <x:c r="K24" s="142" t="n">
         <x:f>('Assumptions'!$B$27*$D22*$F24^2*12+'Assumptions'!$C$27*$D23*$F24*12+'Assumptions'!$D$27*$D24*6.5)/12*'Assumptions'!$D$28</x:f>
         <x:v>77671</x:v>
       </x:c>
-      <x:c r="L24" s="62" t="n">
+      <x:c r="L24" s="142" t="n">
         <x:f>('Assumptions'!$B$29*$D22*$G24^2*12+'Assumptions'!$C$29*$D23*$G24*12+'Assumptions'!$D$29*$D24*6.5)*'Assumptions'!$D$31</x:f>
         <x:v>116380.8</x:v>
       </x:c>
-      <x:c r="M24" s="62" t="n">
+      <x:c r="M24" s="142" t="n">
         <x:f>('Assumptions'!$D$23+'Assumptions'!$D$27)*$D24*'Assumptions'!$D$32</x:f>
         <x:v>66149.99999999999</x:v>
       </x:c>
-      <x:c r="N24" s="62" t="n">
+      <x:c r="N24" s="142" t="n">
         <x:f>SUM(H24:M24)</x:f>
         <x:v>731773.7312960001</x:v>
       </x:c>
-      <x:c r="O24" s="62" t="n">
+      <x:c r="O24" s="142" t="n">
         <x:f>('Assumptions'!$B$37*$D22*$F24^2*12+'Assumptions'!$C$37*$D23*$F24*12+'Assumptions'!$D$37*$D24*6.5)*'Assumptions'!$D$38+('Assumptions'!$B$39*$D22*$F24^2*12+'Assumptions'!$C$39*$D23*$F24*12+'Assumptions'!$D$39*$D24*6.5)*'Assumptions'!$D$40+('Assumptions'!$B$41*$D22*$F24^2*12+'Assumptions'!$C$41*$D23*$F24*12+'Assumptions'!$D$41*$D24*6.5)*'Assumptions'!$D$42+('Assumptions'!$B$43*$D22*$F24^2*12+'Assumptions'!$C$43*$D23*$F24*12+'Assumptions'!$D$43*$D24*6.5)*'Assumptions'!$D$44</x:f>
         <x:v>514994.5988</x:v>
       </x:c>
-      <x:c r="P24" s="62" t="n">
+      <x:c r="P24" s="142" t="n">
         <x:f>O24*'Assumptions'!$D$46</x:f>
         <x:v>15449.837963999998</x:v>
       </x:c>
-      <x:c r="Q24" s="62" t="n">
+      <x:c r="Q24" s="142" t="n">
         <x:f>(('Assumptions'!$D$37+'Assumptions'!$D$39+'Assumptions'!$D$41)*'Assumptions'!$D$47+'Assumptions'!$D$43*'Assumptions'!$D$48)*$D24</x:f>
         <x:v>71120</x:v>
       </x:c>
-      <x:c r="R24" s="62" t="n">
+      <x:c r="R24" s="144" t="n">
         <x:f>N24+O24+P24+Q24</x:f>
         <x:v>1333338.16806</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="23" customHeight="1">
-      <x:c r="A25" s="88" t="str">
+    <x:row r="25" ht="2" customHeight="1">
+      <x:c r="A25" s="219" t="str">
         <x:f>$A$14</x:f>
         <x:v>Marketing-backed</x:v>
       </x:c>
-      <x:c r="B25" s="89" t="n">
+      <x:c r="B25" s="220" t="n">
         <x:f>1</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C25" s="90" t="n">
+      <x:c r="C25" s="221" t="n">
         <x:f>$B$14</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D25" s="90" t="n">
+      <x:c r="D25" s="221" t="n">
         <x:f>$C$14</x:f>
         <x:v>1.2</x:v>
       </x:c>
-      <x:c r="E25" s="90" t="n">
+      <x:c r="E25" s="221" t="n">
         <x:f>$F$14</x:f>
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="F25" s="90" t="n">
+      <x:c r="F25" s="221" t="n">
         <x:f>$G$14</x:f>
         <x:v>0.9</x:v>
       </x:c>
-      <x:c r="G25" s="90" t="n">
+      <x:c r="G25" s="221" t="n">
         <x:f>$H$14</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="H25" s="91" t="n">
+      <x:c r="H25" s="222" t="n">
         <x:f>$C25*(('Assumptions'!$B$8*(6*$E25^0+6*$E25^1)+'Assumptions'!$B$9*(10*$E25^0+2*$E25^1))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F25^0+6*$F25^1)+'Assumptions'!$B$12*(10*$F25^0+2*$F25^1))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>6383.999999999999</x:v>
       </x:c>
-      <x:c r="I25" s="91" t="n">
+      <x:c r="I25" s="222" t="n">
         <x:f>('Assumptions'!$B$20*$D25*6.5)*'Assumptions'!$B$22</x:f>
         <x:v>12480</x:v>
       </x:c>
-      <x:c r="J25" s="91" t="n">
+      <x:c r="J25" s="222" t="n">
         <x:f>'Assumptions'!$B$23*$D25*6.5*'Assumptions'!$B$25*'Assumptions'!$B$26</x:f>
         <x:v>24960</x:v>
       </x:c>
-      <x:c r="K25" s="91" t="n">
+      <x:c r="K25" s="222" t="n">
         <x:f>'Assumptions'!$B$27*$D25*6.5/12*'Assumptions'!$B$28</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L25" s="91" t="n">
+      <x:c r="L25" s="222" t="n">
         <x:f>'Assumptions'!$B$29*$D25*6.5*'Assumptions'!$B$31</x:f>
         <x:v>4680</x:v>
       </x:c>
-      <x:c r="M25" s="91" t="n">
+      <x:c r="M25" s="222" t="n">
         <x:f>('Assumptions'!$B$23+'Assumptions'!$B$27)*$D25*'Assumptions'!$B$32</x:f>
         <x:v>24000</x:v>
       </x:c>
-      <x:c r="N25" s="91" t="n">
+      <x:c r="N25" s="222" t="n">
         <x:f>SUM(H25:M25)</x:f>
         <x:v>72504</x:v>
       </x:c>
-      <x:c r="O25" s="91" t="n">
+      <x:c r="O25" s="222" t="n">
         <x:f>'Assumptions'!$B$37*$D25*6.5*'Assumptions'!$B$38+'Assumptions'!$B$39*$D25*6.5*'Assumptions'!$B$40+'Assumptions'!$B$41*$D25*6.5*'Assumptions'!$B$42+'Assumptions'!$B$43*$D25*6.5*'Assumptions'!$B$44</x:f>
         <x:v>48905.99999999999</x:v>
       </x:c>
-      <x:c r="P25" s="91" t="n">
+      <x:c r="P25" s="222" t="n">
         <x:f>O25*'Assumptions'!$B$46</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q25" s="91" t="n">
+      <x:c r="Q25" s="222" t="n">
         <x:f>(('Assumptions'!$B$37+'Assumptions'!$B$39+'Assumptions'!$B$41)*'Assumptions'!$B$47+'Assumptions'!$B$43*'Assumptions'!$B$48)*$D25</x:f>
         <x:v>21600</x:v>
       </x:c>
-      <x:c r="R25" s="91" t="n">
+      <x:c r="R25" s="223" t="n">
         <x:f>N25+O25+P25+Q25</x:f>
         <x:v>143010</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="23" customHeight="1">
-      <x:c r="A26" s="88" t="str">
+    <x:row r="26" ht="2" customHeight="1">
+      <x:c r="A26" s="219" t="str">
         <x:f>$A$14</x:f>
         <x:v>Marketing-backed</x:v>
       </x:c>
-      <x:c r="B26" s="89" t="n">
+      <x:c r="B26" s="220" t="n">
         <x:f>2</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C26" s="90" t="n">
+      <x:c r="C26" s="221" t="n">
         <x:f>$B$14</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D26" s="90" t="n">
+      <x:c r="D26" s="221" t="n">
         <x:f>$D$14</x:f>
         <x:v>1.25</x:v>
       </x:c>
-      <x:c r="E26" s="90" t="n">
+      <x:c r="E26" s="221" t="n">
         <x:f>$F$14</x:f>
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="F26" s="90" t="n">
+      <x:c r="F26" s="221" t="n">
         <x:f>$G$14</x:f>
         <x:v>0.9</x:v>
       </x:c>
-      <x:c r="G26" s="90" t="n">
+      <x:c r="G26" s="221" t="n">
         <x:f>$H$14</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="H26" s="91" t="n">
+      <x:c r="H26" s="222" t="n">
         <x:f>$C26*(('Assumptions'!$B$8*(6*$E26^1+6*$E26^2)+'Assumptions'!$B$9*(10*$E26^1+2*$E26^2))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F26^1+6*$F26^2)+'Assumptions'!$B$12*(10*$F26^1+2*$F26^2))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>4240.8</x:v>
       </x:c>
-      <x:c r="I26" s="91" t="n">
+      <x:c r="I26" s="222" t="n">
         <x:f>('Assumptions'!$B$20*$D25*$E26*12+'Assumptions'!$C$20*$D26*6.5)*'Assumptions'!$C$22</x:f>
         <x:v>52114.5</x:v>
       </x:c>
-      <x:c r="J26" s="91" t="n">
+      <x:c r="J26" s="222" t="n">
         <x:f>('Assumptions'!$B$23*$D25*$F26*12+'Assumptions'!$C$23*$D26*6.5)*'Assumptions'!$C$25*'Assumptions'!$C$26</x:f>
         <x:v>99584.1</x:v>
       </x:c>
-      <x:c r="K26" s="91" t="n">
+      <x:c r="K26" s="222" t="n">
         <x:f>('Assumptions'!$B$27*$D25*$F26*12+'Assumptions'!$C$27*$D26*6.5)/12*'Assumptions'!$C$28</x:f>
         <x:v>13541.666666666668</x:v>
       </x:c>
-      <x:c r="L26" s="91" t="n">
+      <x:c r="L26" s="222" t="n">
         <x:f>('Assumptions'!$B$29*$D25*$G26*12+'Assumptions'!$C$29*$D26*6.5)*'Assumptions'!$C$31</x:f>
         <x:v>27353.249999999996</x:v>
       </x:c>
-      <x:c r="M26" s="91" t="n">
+      <x:c r="M26" s="222" t="n">
         <x:f>('Assumptions'!$C$23+'Assumptions'!$C$27)*$D26*'Assumptions'!$C$32</x:f>
         <x:v>34875</x:v>
       </x:c>
-      <x:c r="N26" s="91" t="n">
+      <x:c r="N26" s="222" t="n">
         <x:f>SUM(H26:M26)</x:f>
         <x:v>231709.31666666668</x:v>
       </x:c>
-      <x:c r="O26" s="91" t="n">
+      <x:c r="O26" s="222" t="n">
         <x:f>('Assumptions'!$B$37*$D25*$F26*12+'Assumptions'!$C$37*$D26*6.5)*'Assumptions'!$C$38+('Assumptions'!$B$39*$D25*$F26*12+'Assumptions'!$C$39*$D26*6.5)*'Assumptions'!$C$40+('Assumptions'!$B$41*$D25*$F26*12+'Assumptions'!$C$41*$D26*6.5)*'Assumptions'!$C$42+('Assumptions'!$B$43*$D25*$F26*12+'Assumptions'!$C$43*$D26*6.5)*'Assumptions'!$C$44</x:f>
         <x:v>180384.19999999998</x:v>
       </x:c>
-      <x:c r="P26" s="91" t="n">
+      <x:c r="P26" s="222" t="n">
         <x:f>O26*'Assumptions'!$C$46</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q26" s="91" t="n">
+      <x:c r="Q26" s="222" t="n">
         <x:f>(('Assumptions'!$C$37+'Assumptions'!$C$39+'Assumptions'!$C$41)*'Assumptions'!$C$47+'Assumptions'!$C$43*'Assumptions'!$C$48)*$D26</x:f>
         <x:v>36250</x:v>
       </x:c>
-      <x:c r="R26" s="91" t="n">
+      <x:c r="R26" s="223" t="n">
         <x:f>N26+O26+P26+Q26</x:f>
         <x:v>448343.51666666666</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="23" customHeight="1">
-      <x:c r="A27" s="92" t="str">
+    <x:row r="27" ht="2" customHeight="1">
+      <x:c r="A27" s="224" t="str">
         <x:f>$A$14</x:f>
         <x:v>Marketing-backed</x:v>
       </x:c>
-      <x:c r="B27" s="93" t="n">
+      <x:c r="B27" s="225" t="n">
         <x:f>3</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C27" s="94" t="n">
+      <x:c r="C27" s="226" t="n">
         <x:f>$B$14</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D27" s="94" t="n">
+      <x:c r="D27" s="226" t="n">
         <x:f>$E$14</x:f>
         <x:v>1.3</x:v>
       </x:c>
-      <x:c r="E27" s="94" t="n">
+      <x:c r="E27" s="226" t="n">
         <x:f>$F$14</x:f>
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="F27" s="94" t="n">
+      <x:c r="F27" s="226" t="n">
         <x:f>$G$14</x:f>
         <x:v>0.9</x:v>
       </x:c>
-      <x:c r="G27" s="94" t="n">
+      <x:c r="G27" s="226" t="n">
         <x:f>$H$14</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="H27" s="95" t="n">
+      <x:c r="H27" s="227" t="n">
         <x:f>$C27*(('Assumptions'!$B$8*(6*$E27^2+6*$E27^3)+'Assumptions'!$B$9*(10*$E27^2+2*$E27^3))*'Assumptions'!$B$10/12+('Assumptions'!$B$11*(6*$F27^2+6*$F27^3)+'Assumptions'!$B$12*(10*$F27^2+2*$F27^3))*'Assumptions'!$B$13*'Assumptions'!$B$14/12)</x:f>
         <x:v>2913.84</x:v>
       </x:c>
-      <x:c r="I27" s="95" t="n">
+      <x:c r="I27" s="227" t="n">
         <x:f>('Assumptions'!$B$20*$D25*$E27^2*12+'Assumptions'!$C$20*$D26*$E27*12+'Assumptions'!$D$20*$D27*6.5)*'Assumptions'!$D$22</x:f>
         <x:v>139868</x:v>
       </x:c>
-      <x:c r="J27" s="95" t="n">
+      <x:c r="J27" s="227" t="n">
         <x:f>('Assumptions'!$B$23*$D25*$F27^2*12+'Assumptions'!$C$23*$D26*$F27*12+'Assumptions'!$D$23*$D27*6.5)*'Assumptions'!$D$25*'Assumptions'!$D$26</x:f>
         <x:v>274867.19999999995</x:v>
       </x:c>
-      <x:c r="K27" s="95" t="n">
+      <x:c r="K27" s="227" t="n">
         <x:f>('Assumptions'!$B$27*$D25*$F27^2*12+'Assumptions'!$C$27*$D26*$F27*12+'Assumptions'!$D$27*$D27*6.5)/12*'Assumptions'!$D$28</x:f>
         <x:v>71225</x:v>
       </x:c>
-      <x:c r="L27" s="95" t="n">
+      <x:c r="L27" s="227" t="n">
         <x:f>('Assumptions'!$B$29*$D25*$G27^2*12+'Assumptions'!$C$29*$D26*$G27*12+'Assumptions'!$D$29*$D27*6.5)*'Assumptions'!$D$31</x:f>
         <x:v>100807.2</x:v>
       </x:c>
-      <x:c r="M27" s="95" t="n">
+      <x:c r="M27" s="227" t="n">
         <x:f>('Assumptions'!$D$23+'Assumptions'!$D$27)*$D27*'Assumptions'!$D$32</x:f>
         <x:v>61425.00000000001</x:v>
       </x:c>
-      <x:c r="N27" s="95" t="n">
+      <x:c r="N27" s="227" t="n">
         <x:f>SUM(H27:M27)</x:f>
         <x:v>651106.2399999999</x:v>
       </x:c>
-      <x:c r="O27" s="95" t="n">
+      <x:c r="O27" s="227" t="n">
         <x:f>('Assumptions'!$B$37*$D25*$F27^2*12+'Assumptions'!$C$37*$D26*$F27*12+'Assumptions'!$D$37*$D27*6.5)*'Assumptions'!$D$38+('Assumptions'!$B$39*$D25*$F27^2*12+'Assumptions'!$C$39*$D26*$F27*12+'Assumptions'!$D$39*$D27*6.5)*'Assumptions'!$D$40+('Assumptions'!$B$41*$D25*$F27^2*12+'Assumptions'!$C$41*$D26*$F27*12+'Assumptions'!$D$41*$D27*6.5)*'Assumptions'!$D$42+('Assumptions'!$B$43*$D25*$F27^2*12+'Assumptions'!$C$43*$D26*$F27*12+'Assumptions'!$D$43*$D27*6.5)*'Assumptions'!$D$44</x:f>
         <x:v>466811.38</x:v>
       </x:c>
-      <x:c r="P27" s="95" t="n">
+      <x:c r="P27" s="227" t="n">
         <x:f>O27*'Assumptions'!$D$46</x:f>
         <x:v>14004.3414</x:v>
       </x:c>
-      <x:c r="Q27" s="95" t="n">
+      <x:c r="Q27" s="227" t="n">
         <x:f>(('Assumptions'!$D$37+'Assumptions'!$D$39+'Assumptions'!$D$41)*'Assumptions'!$D$47+'Assumptions'!$D$43*'Assumptions'!$D$48)*$D27</x:f>
         <x:v>66040</x:v>
       </x:c>
-      <x:c r="R27" s="95" t="n">
+      <x:c r="R27" s="228" t="n">
         <x:f>N27+O27+P27+Q27</x:f>
         <x:v>1197961.9614</x:v>
       </x:c>
@@ -12907,7 +13317,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>PASS means the workbook reconciles mechanically; market assumptions remain subject to signed Beta contracts and renewal evidence.</x:v>
+        <x:v>Formula integrity, cohort reconciliation, and revenue roll-forward tests</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>PASS means the workbook reconciles mechanically; market assumptions remain subject to signed Beta contracts and renewal evidence.</x:v>
@@ -13335,7 +13745,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>Sources and Benchmark Log</x:v>
+        <x:v>Sources and Evidence</x:v>
       </x:c>
       <x:c r="B1" s="19" t="str">
         <x:v>Sources and Benchmark Log</x:v>
@@ -13364,7 +13774,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>External benchmarks anchor retention, pricing and margins; management targets remain assumptions until observed.</x:v>
+        <x:v>External benchmarks, internal decisions, and validation status</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
         <x:v>External benchmarks anchor retention, pricing and margins; management targets remain assumptions until observed.</x:v>

</xml_diff>